<commit_message>
update some Dutch labels
</commit_message>
<xml_diff>
--- a/data-raw/data/VWO_itemtable.xlsx
+++ b/data-raw/data/VWO_itemtable.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eekhouti\Documents\GitHub\dscoreddi\data-raw\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4BD83C2-6C33-4B49-AAF0-6F4D4B9B8D13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C120CEC1-BE40-44B5-B012-3C659F6A7698}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="734" uniqueCount="525">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="734" uniqueCount="524">
   <si>
     <t>ID.VWO1996</t>
   </si>
@@ -310,9 +310,6 @@
     <t>v1472</t>
   </si>
   <si>
-    <t>Speelt geven en nemen(M)</t>
-  </si>
-  <si>
     <t>Plays give and take</t>
   </si>
   <si>
@@ -331,9 +328,6 @@
     <t>v1512</t>
   </si>
   <si>
-    <t>Stapelt twee blokjes -rl</t>
-  </si>
-  <si>
     <t>Makes tower of two cubes</t>
   </si>
   <si>
@@ -376,9 +370,6 @@
     <t>v1520</t>
   </si>
   <si>
-    <t>Stapelt 3 blokjes -rl</t>
-  </si>
-  <si>
     <t>Makes tower of three cubes</t>
   </si>
   <si>
@@ -1042,9 +1033,6 @@
     <t>v1449</t>
   </si>
   <si>
-    <t>Reacties bij optrekken tot zit (alleen occasion 4!)</t>
-  </si>
-  <si>
     <t>No head lag when pulled to sitting position</t>
   </si>
   <si>
@@ -1123,9 +1111,6 @@
     <t>v1452</t>
   </si>
   <si>
-    <t>Benen gebogen of trappelen bij verticaal zwaaien -rl</t>
-  </si>
-  <si>
     <t>When lifted vertically, legs bended or trampling</t>
   </si>
   <si>
@@ -1387,9 +1372,6 @@
     <t>v1534</t>
   </si>
   <si>
-    <t>Schopt bal weg (RL)</t>
-  </si>
-  <si>
     <t>Kicks ball away</t>
   </si>
   <si>
@@ -1477,9 +1459,6 @@
     <t>Begrijptanalogienentegenstellingen</t>
   </si>
   <si>
-    <t>Kan minstens 5 seconden op een been staan (RL)</t>
-  </si>
-  <si>
     <t>Kanminstens5secondenopbeenstaan</t>
   </si>
   <si>
@@ -1595,6 +1574,24 @@
   </si>
   <si>
     <t>ddigmd075</t>
+  </si>
+  <si>
+    <t>Speelt geven en nemen (M)</t>
+  </si>
+  <si>
+    <t>Benen gebogen of trappelen bij verticaal zwaaien - rl</t>
+  </si>
+  <si>
+    <t>Stapelt twee blokjes - rl</t>
+  </si>
+  <si>
+    <t>Stapelt 3 blokjes - rl</t>
+  </si>
+  <si>
+    <t>Schopt bal weg - rl</t>
+  </si>
+  <si>
+    <t>Kan minstens 5 seconden op een been staan - rl</t>
   </si>
 </sst>
 </file>
@@ -1932,6 +1929,7 @@
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="7" max="7" width="79.5703125" customWidth="1"/>
+    <col min="10" max="10" width="55.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -1951,7 +1949,7 @@
         <v>4</v>
       </c>
       <c r="F1" t="s">
-        <v>507</v>
+        <v>500</v>
       </c>
       <c r="G1" t="s">
         <v>5</v>
@@ -2374,19 +2372,19 @@
         <v>15</v>
       </c>
       <c r="G13" t="s">
+        <v>518</v>
+      </c>
+      <c r="H13" t="s">
         <v>96</v>
       </c>
-      <c r="H13" t="s">
+      <c r="I13" t="s">
         <v>97</v>
       </c>
-      <c r="I13" t="s">
+      <c r="J13" t="s">
         <v>98</v>
       </c>
-      <c r="J13" t="s">
+      <c r="K13" t="s">
         <v>99</v>
-      </c>
-      <c r="K13" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
@@ -2397,10 +2395,10 @@
         <v>42</v>
       </c>
       <c r="C14" t="s">
+        <v>100</v>
+      </c>
+      <c r="D14" t="s">
         <v>101</v>
-      </c>
-      <c r="D14" t="s">
-        <v>102</v>
       </c>
       <c r="E14">
         <v>8</v>
@@ -2409,19 +2407,19 @@
         <v>18</v>
       </c>
       <c r="G14" t="s">
+        <v>520</v>
+      </c>
+      <c r="H14" t="s">
+        <v>102</v>
+      </c>
+      <c r="I14" t="s">
         <v>103</v>
       </c>
-      <c r="H14" t="s">
+      <c r="J14" t="s">
         <v>104</v>
       </c>
-      <c r="I14" t="s">
+      <c r="K14" t="s">
         <v>105</v>
-      </c>
-      <c r="J14" t="s">
-        <v>106</v>
-      </c>
-      <c r="K14" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
@@ -2432,10 +2430,10 @@
         <v>50</v>
       </c>
       <c r="C15" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="D15" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="E15">
         <v>8</v>
@@ -2444,33 +2442,33 @@
         <v>18</v>
       </c>
       <c r="G15" t="s">
+        <v>108</v>
+      </c>
+      <c r="H15" t="s">
+        <v>109</v>
+      </c>
+      <c r="I15" t="s">
         <v>110</v>
       </c>
-      <c r="H15" t="s">
+      <c r="J15" t="s">
         <v>111</v>
       </c>
-      <c r="I15" t="s">
+      <c r="K15" t="s">
         <v>112</v>
-      </c>
-      <c r="J15" t="s">
-        <v>113</v>
-      </c>
-      <c r="K15" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>113</v>
+      </c>
+      <c r="B16" t="s">
+        <v>113</v>
+      </c>
+      <c r="C16" t="s">
+        <v>114</v>
+      </c>
+      <c r="D16" t="s">
         <v>115</v>
-      </c>
-      <c r="B16" t="s">
-        <v>115</v>
-      </c>
-      <c r="C16" t="s">
-        <v>116</v>
-      </c>
-      <c r="D16" t="s">
-        <v>117</v>
       </c>
       <c r="E16">
         <v>9</v>
@@ -2479,33 +2477,33 @@
         <v>24</v>
       </c>
       <c r="G16" t="s">
+        <v>521</v>
+      </c>
+      <c r="H16" t="s">
+        <v>116</v>
+      </c>
+      <c r="I16" t="s">
+        <v>117</v>
+      </c>
+      <c r="J16" t="s">
         <v>118</v>
       </c>
-      <c r="H16" t="s">
+      <c r="K16" t="s">
         <v>119</v>
-      </c>
-      <c r="I16" t="s">
-        <v>120</v>
-      </c>
-      <c r="J16" t="s">
-        <v>121</v>
-      </c>
-      <c r="K16" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="B17" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="C17" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="D17" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="E17">
         <v>9</v>
@@ -2514,30 +2512,30 @@
         <v>24</v>
       </c>
       <c r="G17" t="s">
+        <v>123</v>
+      </c>
+      <c r="H17" t="s">
+        <v>124</v>
+      </c>
+      <c r="I17" t="s">
+        <v>125</v>
+      </c>
+      <c r="J17" t="s">
         <v>126</v>
       </c>
-      <c r="H17" t="s">
+      <c r="K17" t="s">
         <v>127</v>
-      </c>
-      <c r="I17" t="s">
-        <v>128</v>
-      </c>
-      <c r="J17" t="s">
-        <v>129</v>
-      </c>
-      <c r="K17" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="B18" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="D18" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="E18">
         <v>10</v>
@@ -2546,30 +2544,30 @@
         <v>30</v>
       </c>
       <c r="G18" t="s">
+        <v>130</v>
+      </c>
+      <c r="H18" t="s">
+        <v>131</v>
+      </c>
+      <c r="I18" t="s">
+        <v>132</v>
+      </c>
+      <c r="J18" t="s">
         <v>133</v>
       </c>
-      <c r="H18" t="s">
+      <c r="K18" t="s">
         <v>134</v>
-      </c>
-      <c r="I18" t="s">
-        <v>135</v>
-      </c>
-      <c r="J18" t="s">
-        <v>136</v>
-      </c>
-      <c r="K18" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="B19" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D19" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="E19">
         <v>10</v>
@@ -2578,19 +2576,19 @@
         <v>30</v>
       </c>
       <c r="G19" t="s">
+        <v>137</v>
+      </c>
+      <c r="H19" t="s">
+        <v>138</v>
+      </c>
+      <c r="I19" t="s">
+        <v>139</v>
+      </c>
+      <c r="J19" t="s">
         <v>140</v>
       </c>
-      <c r="H19" t="s">
+      <c r="K19" t="s">
         <v>141</v>
-      </c>
-      <c r="I19" t="s">
-        <v>142</v>
-      </c>
-      <c r="J19" t="s">
-        <v>143</v>
-      </c>
-      <c r="K19" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
@@ -2601,7 +2599,7 @@
         <v>57</v>
       </c>
       <c r="D20" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="E20">
         <v>10</v>
@@ -2610,19 +2608,19 @@
         <v>30</v>
       </c>
       <c r="G20" t="s">
+        <v>143</v>
+      </c>
+      <c r="H20" t="s">
+        <v>144</v>
+      </c>
+      <c r="I20" t="s">
+        <v>145</v>
+      </c>
+      <c r="J20" t="s">
         <v>146</v>
       </c>
-      <c r="H20" t="s">
+      <c r="K20" t="s">
         <v>147</v>
-      </c>
-      <c r="I20" t="s">
-        <v>148</v>
-      </c>
-      <c r="J20" t="s">
-        <v>149</v>
-      </c>
-      <c r="K20" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
@@ -2639,19 +2637,19 @@
         <v>36</v>
       </c>
       <c r="G21" t="s">
+        <v>148</v>
+      </c>
+      <c r="H21" t="s">
         <v>151</v>
       </c>
-      <c r="H21" t="s">
-        <v>154</v>
-      </c>
       <c r="I21" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="J21" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="K21" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
@@ -2668,27 +2666,27 @@
         <v>36</v>
       </c>
       <c r="G22" t="s">
+        <v>153</v>
+      </c>
+      <c r="H22" t="s">
+        <v>155</v>
+      </c>
+      <c r="I22" t="s">
+        <v>154</v>
+      </c>
+      <c r="J22" t="s">
+        <v>155</v>
+      </c>
+      <c r="K22" t="s">
         <v>156</v>
-      </c>
-      <c r="H22" t="s">
-        <v>158</v>
-      </c>
-      <c r="I22" t="s">
-        <v>157</v>
-      </c>
-      <c r="J22" t="s">
-        <v>158</v>
-      </c>
-      <c r="K22" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="B23" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="E23">
         <v>11</v>
@@ -2697,27 +2695,27 @@
         <v>36</v>
       </c>
       <c r="G23" t="s">
+        <v>158</v>
+      </c>
+      <c r="H23" t="s">
+        <v>160</v>
+      </c>
+      <c r="I23" t="s">
+        <v>159</v>
+      </c>
+      <c r="J23" t="s">
+        <v>160</v>
+      </c>
+      <c r="K23" t="s">
         <v>161</v>
-      </c>
-      <c r="H23" t="s">
-        <v>163</v>
-      </c>
-      <c r="I23" t="s">
-        <v>162</v>
-      </c>
-      <c r="J23" t="s">
-        <v>163</v>
-      </c>
-      <c r="K23" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="B24" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="E24">
         <v>12</v>
@@ -2726,27 +2724,27 @@
         <v>42</v>
       </c>
       <c r="G24" t="s">
+        <v>163</v>
+      </c>
+      <c r="H24" t="s">
+        <v>165</v>
+      </c>
+      <c r="I24" t="s">
+        <v>164</v>
+      </c>
+      <c r="J24" t="s">
+        <v>165</v>
+      </c>
+      <c r="K24" t="s">
         <v>166</v>
-      </c>
-      <c r="H24" t="s">
-        <v>168</v>
-      </c>
-      <c r="I24" t="s">
-        <v>167</v>
-      </c>
-      <c r="J24" t="s">
-        <v>168</v>
-      </c>
-      <c r="K24" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="B25" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="E25">
         <v>12</v>
@@ -2755,27 +2753,27 @@
         <v>42</v>
       </c>
       <c r="G25" t="s">
+        <v>168</v>
+      </c>
+      <c r="H25" t="s">
+        <v>170</v>
+      </c>
+      <c r="I25" t="s">
+        <v>169</v>
+      </c>
+      <c r="J25" t="s">
+        <v>170</v>
+      </c>
+      <c r="K25" t="s">
         <v>171</v>
-      </c>
-      <c r="H25" t="s">
-        <v>173</v>
-      </c>
-      <c r="I25" t="s">
-        <v>172</v>
-      </c>
-      <c r="J25" t="s">
-        <v>173</v>
-      </c>
-      <c r="K25" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="B26" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="E26">
         <v>12</v>
@@ -2784,24 +2782,24 @@
         <v>42</v>
       </c>
       <c r="G26" t="s">
+        <v>173</v>
+      </c>
+      <c r="H26" t="s">
+        <v>175</v>
+      </c>
+      <c r="I26" t="s">
+        <v>174</v>
+      </c>
+      <c r="J26" t="s">
+        <v>175</v>
+      </c>
+      <c r="K26" t="s">
         <v>176</v>
-      </c>
-      <c r="H26" t="s">
-        <v>178</v>
-      </c>
-      <c r="I26" t="s">
-        <v>177</v>
-      </c>
-      <c r="J26" t="s">
-        <v>178</v>
-      </c>
-      <c r="K26" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="B27" t="s">
         <v>78</v>
@@ -2813,19 +2811,19 @@
         <v>48</v>
       </c>
       <c r="G27" t="s">
+        <v>178</v>
+      </c>
+      <c r="H27" t="s">
+        <v>180</v>
+      </c>
+      <c r="I27" t="s">
+        <v>179</v>
+      </c>
+      <c r="J27" t="s">
+        <v>180</v>
+      </c>
+      <c r="K27" t="s">
         <v>181</v>
-      </c>
-      <c r="H27" t="s">
-        <v>183</v>
-      </c>
-      <c r="I27" t="s">
-        <v>182</v>
-      </c>
-      <c r="J27" t="s">
-        <v>183</v>
-      </c>
-      <c r="K27" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
@@ -2833,7 +2831,7 @@
         <v>78</v>
       </c>
       <c r="B28" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="E28">
         <v>13</v>
@@ -2842,33 +2840,33 @@
         <v>48</v>
       </c>
       <c r="G28" t="s">
+        <v>182</v>
+      </c>
+      <c r="H28" t="s">
+        <v>184</v>
+      </c>
+      <c r="I28" t="s">
+        <v>183</v>
+      </c>
+      <c r="J28" t="s">
+        <v>184</v>
+      </c>
+      <c r="K28" t="s">
         <v>185</v>
-      </c>
-      <c r="H28" t="s">
-        <v>187</v>
-      </c>
-      <c r="I28" t="s">
-        <v>186</v>
-      </c>
-      <c r="J28" t="s">
-        <v>187</v>
-      </c>
-      <c r="K28" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="B29" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="C29" t="s">
         <v>17</v>
       </c>
       <c r="D29" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="E29">
         <v>1</v>
@@ -2877,33 +2875,33 @@
         <v>1</v>
       </c>
       <c r="G29" t="s">
+        <v>189</v>
+      </c>
+      <c r="H29" t="s">
+        <v>190</v>
+      </c>
+      <c r="I29" t="s">
+        <v>191</v>
+      </c>
+      <c r="J29" t="s">
         <v>192</v>
       </c>
-      <c r="H29" t="s">
+      <c r="K29" t="s">
         <v>193</v>
-      </c>
-      <c r="I29" t="s">
-        <v>194</v>
-      </c>
-      <c r="J29" t="s">
-        <v>195</v>
-      </c>
-      <c r="K29" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="B30" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="C30" t="s">
         <v>49</v>
       </c>
       <c r="D30" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="E30">
         <v>2</v>
@@ -2912,33 +2910,33 @@
         <v>2</v>
       </c>
       <c r="G30" t="s">
+        <v>196</v>
+      </c>
+      <c r="H30" t="s">
+        <v>197</v>
+      </c>
+      <c r="I30" t="s">
+        <v>198</v>
+      </c>
+      <c r="J30" t="s">
         <v>199</v>
       </c>
-      <c r="H30" t="s">
+      <c r="K30" t="s">
         <v>200</v>
-      </c>
-      <c r="I30" t="s">
-        <v>201</v>
-      </c>
-      <c r="J30" t="s">
-        <v>202</v>
-      </c>
-      <c r="K30" t="s">
-        <v>203</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="B31" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="C31" t="s">
         <v>77</v>
       </c>
       <c r="D31" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="E31">
         <v>3</v>
@@ -2947,33 +2945,33 @@
         <v>3</v>
       </c>
       <c r="G31" t="s">
+        <v>203</v>
+      </c>
+      <c r="H31" t="s">
+        <v>204</v>
+      </c>
+      <c r="I31" t="s">
+        <v>205</v>
+      </c>
+      <c r="J31" t="s">
         <v>206</v>
       </c>
-      <c r="H31" t="s">
+      <c r="K31" t="s">
         <v>207</v>
-      </c>
-      <c r="I31" t="s">
-        <v>208</v>
-      </c>
-      <c r="J31" t="s">
-        <v>209</v>
-      </c>
-      <c r="K31" t="s">
-        <v>210</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="B32" t="s">
         <v>86</v>
       </c>
       <c r="C32" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="D32" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="E32">
         <v>4</v>
@@ -2982,16 +2980,16 @@
         <v>6</v>
       </c>
       <c r="G32" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="H32" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="I32" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="K32" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
@@ -2999,7 +2997,7 @@
         <v>86</v>
       </c>
       <c r="C33" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="D33" t="s">
         <v>86</v>
@@ -3011,13 +3009,13 @@
         <v>6</v>
       </c>
       <c r="G33" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="H33" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="K33" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
@@ -3028,10 +3026,10 @@
         <v>94</v>
       </c>
       <c r="C34" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="D34" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="E34">
         <v>5</v>
@@ -3040,33 +3038,33 @@
         <v>9</v>
       </c>
       <c r="G34" t="s">
+        <v>216</v>
+      </c>
+      <c r="H34" t="s">
+        <v>217</v>
+      </c>
+      <c r="I34" t="s">
+        <v>218</v>
+      </c>
+      <c r="J34" t="s">
         <v>219</v>
       </c>
-      <c r="H34" t="s">
+      <c r="K34" t="s">
         <v>220</v>
-      </c>
-      <c r="I34" t="s">
-        <v>221</v>
-      </c>
-      <c r="J34" t="s">
-        <v>222</v>
-      </c>
-      <c r="K34" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="B35" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="C35" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="D35" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="E35">
         <v>6</v>
@@ -3075,33 +3073,33 @@
         <v>12</v>
       </c>
       <c r="G35" t="s">
+        <v>223</v>
+      </c>
+      <c r="H35" t="s">
+        <v>224</v>
+      </c>
+      <c r="I35" t="s">
+        <v>225</v>
+      </c>
+      <c r="J35" t="s">
         <v>226</v>
       </c>
-      <c r="H35" t="s">
+      <c r="K35" t="s">
         <v>227</v>
-      </c>
-      <c r="I35" t="s">
-        <v>228</v>
-      </c>
-      <c r="J35" t="s">
-        <v>229</v>
-      </c>
-      <c r="K35" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="B36" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="C36" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="D36" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="E36">
         <v>6</v>
@@ -3110,33 +3108,33 @@
         <v>12</v>
       </c>
       <c r="G36" t="s">
+        <v>230</v>
+      </c>
+      <c r="H36" t="s">
+        <v>232</v>
+      </c>
+      <c r="I36" t="s">
+        <v>231</v>
+      </c>
+      <c r="J36" t="s">
+        <v>232</v>
+      </c>
+      <c r="K36" t="s">
         <v>233</v>
-      </c>
-      <c r="H36" t="s">
-        <v>235</v>
-      </c>
-      <c r="I36" t="s">
-        <v>234</v>
-      </c>
-      <c r="J36" t="s">
-        <v>235</v>
-      </c>
-      <c r="K36" t="s">
-        <v>236</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="B37" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="C37" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="D37" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="E37">
         <v>6</v>
@@ -3145,33 +3143,33 @@
         <v>12</v>
       </c>
       <c r="G37" t="s">
+        <v>230</v>
+      </c>
+      <c r="H37" t="s">
+        <v>232</v>
+      </c>
+      <c r="I37" t="s">
+        <v>512</v>
+      </c>
+      <c r="J37" t="s">
+        <v>232</v>
+      </c>
+      <c r="K37" t="s">
         <v>233</v>
-      </c>
-      <c r="H37" t="s">
-        <v>235</v>
-      </c>
-      <c r="I37" t="s">
-        <v>519</v>
-      </c>
-      <c r="J37" t="s">
-        <v>235</v>
-      </c>
-      <c r="K37" t="s">
-        <v>236</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="B38" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="C38" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="D38" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="E38">
         <v>6</v>
@@ -3180,33 +3178,33 @@
         <v>12</v>
       </c>
       <c r="G38" t="s">
+        <v>236</v>
+      </c>
+      <c r="H38" t="s">
+        <v>237</v>
+      </c>
+      <c r="I38" t="s">
+        <v>238</v>
+      </c>
+      <c r="J38" t="s">
         <v>239</v>
       </c>
-      <c r="H38" t="s">
+      <c r="K38" t="s">
         <v>240</v>
-      </c>
-      <c r="I38" t="s">
-        <v>241</v>
-      </c>
-      <c r="J38" t="s">
-        <v>242</v>
-      </c>
-      <c r="K38" t="s">
-        <v>243</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="B39" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="C39" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="D39" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="E39">
         <v>7</v>
@@ -3215,33 +3213,33 @@
         <v>15</v>
       </c>
       <c r="G39" t="s">
+        <v>243</v>
+      </c>
+      <c r="H39" t="s">
+        <v>244</v>
+      </c>
+      <c r="I39" t="s">
+        <v>245</v>
+      </c>
+      <c r="J39" t="s">
         <v>246</v>
       </c>
-      <c r="H39" t="s">
+      <c r="K39" t="s">
         <v>247</v>
-      </c>
-      <c r="I39" t="s">
-        <v>248</v>
-      </c>
-      <c r="J39" t="s">
-        <v>249</v>
-      </c>
-      <c r="K39" t="s">
-        <v>250</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B40" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C40" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="D40" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E40">
         <v>7</v>
@@ -3250,30 +3248,30 @@
         <v>15</v>
       </c>
       <c r="G40" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="H40" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="I40" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="K40" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B41" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C41" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="D41" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="E41">
         <v>8</v>
@@ -3282,33 +3280,33 @@
         <v>18</v>
       </c>
       <c r="G41" t="s">
-        <v>522</v>
+        <v>515</v>
       </c>
       <c r="H41" t="s">
+        <v>254</v>
+      </c>
+      <c r="I41" t="s">
+        <v>255</v>
+      </c>
+      <c r="J41" t="s">
+        <v>256</v>
+      </c>
+      <c r="K41" t="s">
         <v>257</v>
-      </c>
-      <c r="I41" t="s">
-        <v>258</v>
-      </c>
-      <c r="J41" t="s">
-        <v>259</v>
-      </c>
-      <c r="K41" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="B42" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="C42" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="D42" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="E42">
         <v>8</v>
@@ -3317,33 +3315,33 @@
         <v>18</v>
       </c>
       <c r="G42" t="s">
+        <v>259</v>
+      </c>
+      <c r="H42" t="s">
+        <v>261</v>
+      </c>
+      <c r="I42" t="s">
+        <v>260</v>
+      </c>
+      <c r="J42" t="s">
+        <v>261</v>
+      </c>
+      <c r="K42" t="s">
         <v>262</v>
-      </c>
-      <c r="H42" t="s">
-        <v>264</v>
-      </c>
-      <c r="I42" t="s">
-        <v>263</v>
-      </c>
-      <c r="J42" t="s">
-        <v>264</v>
-      </c>
-      <c r="K42" t="s">
-        <v>265</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="B43" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="C43" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="D43" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="E43">
         <v>8</v>
@@ -3352,33 +3350,33 @@
         <v>18</v>
       </c>
       <c r="G43" t="s">
+        <v>259</v>
+      </c>
+      <c r="H43" t="s">
+        <v>261</v>
+      </c>
+      <c r="I43" t="s">
+        <v>510</v>
+      </c>
+      <c r="J43" t="s">
+        <v>261</v>
+      </c>
+      <c r="K43" t="s">
         <v>262</v>
-      </c>
-      <c r="H43" t="s">
-        <v>264</v>
-      </c>
-      <c r="I43" t="s">
-        <v>517</v>
-      </c>
-      <c r="J43" t="s">
-        <v>264</v>
-      </c>
-      <c r="K43" t="s">
-        <v>265</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="B44" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="C44" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="D44" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="E44">
         <v>9</v>
@@ -3387,33 +3385,33 @@
         <v>24</v>
       </c>
       <c r="G44" t="s">
+        <v>266</v>
+      </c>
+      <c r="H44" t="s">
+        <v>267</v>
+      </c>
+      <c r="I44" t="s">
+        <v>268</v>
+      </c>
+      <c r="J44" t="s">
         <v>269</v>
       </c>
-      <c r="H44" t="s">
+      <c r="K44" t="s">
         <v>270</v>
-      </c>
-      <c r="I44" t="s">
-        <v>271</v>
-      </c>
-      <c r="J44" t="s">
-        <v>272</v>
-      </c>
-      <c r="K44" t="s">
-        <v>273</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="B45" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="C45" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="D45" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="E45">
         <v>9</v>
@@ -3422,30 +3420,30 @@
         <v>24</v>
       </c>
       <c r="G45" t="s">
+        <v>273</v>
+      </c>
+      <c r="H45" t="s">
+        <v>275</v>
+      </c>
+      <c r="I45" t="s">
+        <v>274</v>
+      </c>
+      <c r="J45" t="s">
+        <v>275</v>
+      </c>
+      <c r="K45" t="s">
         <v>276</v>
-      </c>
-      <c r="H45" t="s">
-        <v>278</v>
-      </c>
-      <c r="I45" t="s">
-        <v>277</v>
-      </c>
-      <c r="J45" t="s">
-        <v>278</v>
-      </c>
-      <c r="K45" t="s">
-        <v>279</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="B46" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="D46" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="E46">
         <v>10</v>
@@ -3454,30 +3452,30 @@
         <v>30</v>
       </c>
       <c r="G46" t="s">
+        <v>279</v>
+      </c>
+      <c r="H46" t="s">
+        <v>280</v>
+      </c>
+      <c r="I46" t="s">
+        <v>281</v>
+      </c>
+      <c r="J46" t="s">
         <v>282</v>
       </c>
-      <c r="H46" t="s">
+      <c r="K46" t="s">
         <v>283</v>
-      </c>
-      <c r="I46" t="s">
-        <v>284</v>
-      </c>
-      <c r="J46" t="s">
-        <v>285</v>
-      </c>
-      <c r="K46" t="s">
-        <v>286</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B47" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D47" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="E47">
         <v>10</v>
@@ -3486,27 +3484,27 @@
         <v>30</v>
       </c>
       <c r="G47" t="s">
+        <v>285</v>
+      </c>
+      <c r="H47" t="s">
+        <v>286</v>
+      </c>
+      <c r="I47" t="s">
+        <v>287</v>
+      </c>
+      <c r="J47" t="s">
         <v>288</v>
       </c>
-      <c r="H47" t="s">
+      <c r="K47" t="s">
         <v>289</v>
-      </c>
-      <c r="I47" t="s">
-        <v>290</v>
-      </c>
-      <c r="J47" t="s">
-        <v>291</v>
-      </c>
-      <c r="K47" t="s">
-        <v>292</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="B48" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="E48">
         <v>11</v>
@@ -3515,27 +3513,27 @@
         <v>36</v>
       </c>
       <c r="G48" t="s">
+        <v>290</v>
+      </c>
+      <c r="H48" t="s">
+        <v>292</v>
+      </c>
+      <c r="I48" t="s">
+        <v>291</v>
+      </c>
+      <c r="J48" t="s">
+        <v>292</v>
+      </c>
+      <c r="K48" t="s">
         <v>293</v>
-      </c>
-      <c r="H48" t="s">
-        <v>295</v>
-      </c>
-      <c r="I48" t="s">
-        <v>294</v>
-      </c>
-      <c r="J48" t="s">
-        <v>295</v>
-      </c>
-      <c r="K48" t="s">
-        <v>296</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="B49" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="E49">
         <v>11</v>
@@ -3544,27 +3542,27 @@
         <v>36</v>
       </c>
       <c r="G49" t="s">
+        <v>295</v>
+      </c>
+      <c r="H49" t="s">
+        <v>297</v>
+      </c>
+      <c r="I49" t="s">
+        <v>296</v>
+      </c>
+      <c r="J49" t="s">
+        <v>297</v>
+      </c>
+      <c r="K49" t="s">
         <v>298</v>
-      </c>
-      <c r="H49" t="s">
-        <v>300</v>
-      </c>
-      <c r="I49" t="s">
-        <v>299</v>
-      </c>
-      <c r="J49" t="s">
-        <v>300</v>
-      </c>
-      <c r="K49" t="s">
-        <v>301</v>
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="B50" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="E50">
         <v>12</v>
@@ -3573,27 +3571,27 @@
         <v>42</v>
       </c>
       <c r="G50" t="s">
+        <v>299</v>
+      </c>
+      <c r="H50" t="s">
+        <v>301</v>
+      </c>
+      <c r="I50" t="s">
+        <v>300</v>
+      </c>
+      <c r="J50" t="s">
+        <v>301</v>
+      </c>
+      <c r="K50" t="s">
         <v>302</v>
-      </c>
-      <c r="H50" t="s">
-        <v>304</v>
-      </c>
-      <c r="I50" t="s">
-        <v>303</v>
-      </c>
-      <c r="J50" t="s">
-        <v>304</v>
-      </c>
-      <c r="K50" t="s">
-        <v>305</v>
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="B51" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="E51">
         <v>12</v>
@@ -3602,27 +3600,27 @@
         <v>42</v>
       </c>
       <c r="G51" t="s">
+        <v>304</v>
+      </c>
+      <c r="H51" t="s">
+        <v>306</v>
+      </c>
+      <c r="I51" t="s">
+        <v>305</v>
+      </c>
+      <c r="J51" t="s">
+        <v>306</v>
+      </c>
+      <c r="K51" t="s">
         <v>307</v>
-      </c>
-      <c r="H51" t="s">
-        <v>309</v>
-      </c>
-      <c r="I51" t="s">
-        <v>308</v>
-      </c>
-      <c r="J51" t="s">
-        <v>309</v>
-      </c>
-      <c r="K51" t="s">
-        <v>310</v>
       </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="B52" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="E52">
         <v>13</v>
@@ -3631,27 +3629,27 @@
         <v>48</v>
       </c>
       <c r="G52" t="s">
+        <v>309</v>
+      </c>
+      <c r="H52" t="s">
+        <v>311</v>
+      </c>
+      <c r="I52" t="s">
+        <v>310</v>
+      </c>
+      <c r="J52" t="s">
+        <v>311</v>
+      </c>
+      <c r="K52" t="s">
         <v>312</v>
-      </c>
-      <c r="H52" t="s">
-        <v>314</v>
-      </c>
-      <c r="I52" t="s">
-        <v>313</v>
-      </c>
-      <c r="J52" t="s">
-        <v>314</v>
-      </c>
-      <c r="K52" t="s">
-        <v>315</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="B53" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="E53">
         <v>13</v>
@@ -3660,33 +3658,33 @@
         <v>48</v>
       </c>
       <c r="G53" t="s">
+        <v>314</v>
+      </c>
+      <c r="H53" t="s">
+        <v>316</v>
+      </c>
+      <c r="I53" t="s">
+        <v>315</v>
+      </c>
+      <c r="J53" t="s">
+        <v>316</v>
+      </c>
+      <c r="K53" t="s">
         <v>317</v>
-      </c>
-      <c r="H53" t="s">
-        <v>319</v>
-      </c>
-      <c r="I53" t="s">
-        <v>318</v>
-      </c>
-      <c r="J53" t="s">
-        <v>319</v>
-      </c>
-      <c r="K53" t="s">
-        <v>320</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="B54" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="C54" t="s">
         <v>25</v>
       </c>
       <c r="D54" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
       <c r="E54">
         <v>1</v>
@@ -3695,33 +3693,33 @@
         <v>1</v>
       </c>
       <c r="G54" t="s">
+        <v>319</v>
+      </c>
+      <c r="H54" t="s">
+        <v>320</v>
+      </c>
+      <c r="I54" t="s">
+        <v>321</v>
+      </c>
+      <c r="J54" t="s">
         <v>322</v>
       </c>
-      <c r="H54" t="s">
+      <c r="K54" t="s">
         <v>323</v>
-      </c>
-      <c r="I54" t="s">
-        <v>324</v>
-      </c>
-      <c r="J54" t="s">
-        <v>325</v>
-      </c>
-      <c r="K54" t="s">
-        <v>326</v>
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="B55" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="C55" t="s">
         <v>33</v>
       </c>
       <c r="D55" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="E55">
         <v>1</v>
@@ -3730,33 +3728,33 @@
         <v>1</v>
       </c>
       <c r="G55" t="s">
+        <v>325</v>
+      </c>
+      <c r="H55" t="s">
+        <v>326</v>
+      </c>
+      <c r="I55" t="s">
+        <v>327</v>
+      </c>
+      <c r="J55" t="s">
         <v>328</v>
       </c>
-      <c r="H55" t="s">
+      <c r="K55" t="s">
         <v>329</v>
-      </c>
-      <c r="I55" t="s">
-        <v>330</v>
-      </c>
-      <c r="J55" t="s">
-        <v>331</v>
-      </c>
-      <c r="K55" t="s">
-        <v>332</v>
       </c>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="B56" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="C56" t="s">
         <v>85</v>
       </c>
       <c r="D56" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="E56">
         <v>3</v>
@@ -3765,33 +3763,33 @@
         <v>3</v>
       </c>
       <c r="G56" t="s">
+        <v>331</v>
+      </c>
+      <c r="H56" t="s">
+        <v>332</v>
+      </c>
+      <c r="I56" t="s">
+        <v>333</v>
+      </c>
+      <c r="J56" t="s">
         <v>334</v>
       </c>
-      <c r="H56" t="s">
+      <c r="K56" t="s">
         <v>335</v>
-      </c>
-      <c r="I56" t="s">
-        <v>336</v>
-      </c>
-      <c r="J56" t="s">
-        <v>337</v>
-      </c>
-      <c r="K56" t="s">
-        <v>338</v>
       </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="B57" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="C57" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D57" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="E57">
         <v>4</v>
@@ -3800,33 +3798,33 @@
         <v>6</v>
       </c>
       <c r="G57" t="s">
+        <v>499</v>
+      </c>
+      <c r="H57" t="s">
+        <v>337</v>
+      </c>
+      <c r="I57" t="s">
+        <v>338</v>
+      </c>
+      <c r="J57" t="s">
+        <v>339</v>
+      </c>
+      <c r="K57" t="s">
         <v>340</v>
-      </c>
-      <c r="H57" t="s">
-        <v>341</v>
-      </c>
-      <c r="I57" t="s">
-        <v>342</v>
-      </c>
-      <c r="J57" t="s">
-        <v>343</v>
-      </c>
-      <c r="K57" t="s">
-        <v>344</v>
       </c>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="B58" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="C58" t="s">
         <v>41</v>
       </c>
       <c r="D58" t="s">
-        <v>345</v>
+        <v>341</v>
       </c>
       <c r="E58">
         <v>1</v>
@@ -3835,33 +3833,33 @@
         <v>1</v>
       </c>
       <c r="G58" t="s">
+        <v>342</v>
+      </c>
+      <c r="H58" t="s">
+        <v>343</v>
+      </c>
+      <c r="I58" t="s">
+        <v>344</v>
+      </c>
+      <c r="J58" t="s">
+        <v>345</v>
+      </c>
+      <c r="K58" t="s">
         <v>346</v>
-      </c>
-      <c r="H58" t="s">
-        <v>347</v>
-      </c>
-      <c r="I58" t="s">
-        <v>348</v>
-      </c>
-      <c r="J58" t="s">
-        <v>349</v>
-      </c>
-      <c r="K58" t="s">
-        <v>350</v>
       </c>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="B59" t="s">
-        <v>351</v>
+        <v>347</v>
       </c>
       <c r="C59" t="s">
         <v>93</v>
       </c>
       <c r="D59" t="s">
-        <v>352</v>
+        <v>348</v>
       </c>
       <c r="E59">
         <v>3</v>
@@ -3870,33 +3868,33 @@
         <v>3</v>
       </c>
       <c r="G59" t="s">
+        <v>349</v>
+      </c>
+      <c r="H59" t="s">
+        <v>350</v>
+      </c>
+      <c r="I59" t="s">
+        <v>351</v>
+      </c>
+      <c r="J59" t="s">
+        <v>352</v>
+      </c>
+      <c r="K59" t="s">
         <v>353</v>
-      </c>
-      <c r="H59" t="s">
-        <v>354</v>
-      </c>
-      <c r="I59" t="s">
-        <v>355</v>
-      </c>
-      <c r="J59" t="s">
-        <v>356</v>
-      </c>
-      <c r="K59" t="s">
-        <v>357</v>
       </c>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>351</v>
+        <v>347</v>
       </c>
       <c r="B60" t="s">
-        <v>358</v>
+        <v>354</v>
       </c>
       <c r="C60" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D60" t="s">
-        <v>359</v>
+        <v>355</v>
       </c>
       <c r="E60">
         <v>4</v>
@@ -3905,33 +3903,33 @@
         <v>6</v>
       </c>
       <c r="G60" t="s">
+        <v>356</v>
+      </c>
+      <c r="H60" t="s">
+        <v>357</v>
+      </c>
+      <c r="I60" t="s">
+        <v>358</v>
+      </c>
+      <c r="J60" t="s">
+        <v>359</v>
+      </c>
+      <c r="K60" t="s">
         <v>360</v>
-      </c>
-      <c r="H60" t="s">
-        <v>361</v>
-      </c>
-      <c r="I60" t="s">
-        <v>362</v>
-      </c>
-      <c r="J60" t="s">
-        <v>363</v>
-      </c>
-      <c r="K60" t="s">
-        <v>364</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>358</v>
+        <v>354</v>
       </c>
       <c r="B61" t="s">
-        <v>365</v>
+        <v>361</v>
       </c>
       <c r="C61" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="D61" t="s">
-        <v>366</v>
+        <v>362</v>
       </c>
       <c r="E61">
         <v>4</v>
@@ -3940,33 +3938,33 @@
         <v>6</v>
       </c>
       <c r="G61" t="s">
-        <v>367</v>
+        <v>519</v>
       </c>
       <c r="H61" t="s">
-        <v>368</v>
+        <v>363</v>
       </c>
       <c r="I61" t="s">
-        <v>369</v>
+        <v>364</v>
       </c>
       <c r="J61" t="s">
-        <v>370</v>
+        <v>365</v>
       </c>
       <c r="K61" t="s">
-        <v>371</v>
+        <v>366</v>
       </c>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>365</v>
+        <v>361</v>
       </c>
       <c r="B62" t="s">
-        <v>372</v>
+        <v>367</v>
       </c>
       <c r="C62" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="D62" t="s">
-        <v>373</v>
+        <v>368</v>
       </c>
       <c r="E62">
         <v>5</v>
@@ -3975,33 +3973,33 @@
         <v>9</v>
       </c>
       <c r="G62" t="s">
-        <v>374</v>
+        <v>369</v>
       </c>
       <c r="H62" t="s">
-        <v>375</v>
+        <v>370</v>
       </c>
       <c r="I62" t="s">
-        <v>376</v>
+        <v>371</v>
       </c>
       <c r="J62" t="s">
-        <v>377</v>
+        <v>372</v>
       </c>
       <c r="K62" t="s">
-        <v>378</v>
+        <v>373</v>
       </c>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>372</v>
+        <v>367</v>
       </c>
       <c r="B63" t="s">
-        <v>379</v>
+        <v>374</v>
       </c>
       <c r="C63" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="D63" t="s">
-        <v>380</v>
+        <v>375</v>
       </c>
       <c r="E63">
         <v>5</v>
@@ -4010,33 +4008,33 @@
         <v>9</v>
       </c>
       <c r="G63" t="s">
-        <v>381</v>
+        <v>376</v>
       </c>
       <c r="H63" t="s">
-        <v>382</v>
+        <v>377</v>
       </c>
       <c r="I63" t="s">
-        <v>383</v>
+        <v>378</v>
       </c>
       <c r="J63" t="s">
-        <v>384</v>
+        <v>379</v>
       </c>
       <c r="K63" t="s">
-        <v>385</v>
+        <v>380</v>
       </c>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>379</v>
+        <v>374</v>
       </c>
       <c r="B64" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="C64" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="D64" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
       <c r="E64">
         <v>5</v>
@@ -4045,33 +4043,33 @@
         <v>9</v>
       </c>
       <c r="G64" t="s">
-        <v>388</v>
+        <v>383</v>
       </c>
       <c r="H64" t="s">
-        <v>389</v>
+        <v>384</v>
       </c>
       <c r="I64" t="s">
-        <v>390</v>
+        <v>385</v>
       </c>
       <c r="J64" t="s">
-        <v>391</v>
+        <v>386</v>
       </c>
       <c r="K64" t="s">
-        <v>392</v>
+        <v>387</v>
       </c>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="B65" t="s">
-        <v>393</v>
+        <v>388</v>
       </c>
       <c r="C65" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="D65" t="s">
-        <v>394</v>
+        <v>389</v>
       </c>
       <c r="E65">
         <v>6</v>
@@ -4080,33 +4078,33 @@
         <v>12</v>
       </c>
       <c r="G65" t="s">
-        <v>395</v>
+        <v>390</v>
       </c>
       <c r="H65" t="s">
-        <v>396</v>
+        <v>391</v>
       </c>
       <c r="I65" t="s">
-        <v>397</v>
+        <v>392</v>
       </c>
       <c r="J65" t="s">
-        <v>398</v>
+        <v>393</v>
       </c>
       <c r="K65" t="s">
-        <v>399</v>
+        <v>394</v>
       </c>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>393</v>
+        <v>388</v>
       </c>
       <c r="B66" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
       <c r="C66" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="D66" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
       <c r="E66">
         <v>6</v>
@@ -4115,33 +4113,33 @@
         <v>12</v>
       </c>
       <c r="G66" t="s">
-        <v>402</v>
+        <v>397</v>
       </c>
       <c r="H66" t="s">
-        <v>404</v>
+        <v>399</v>
       </c>
       <c r="I66" t="s">
-        <v>403</v>
+        <v>398</v>
       </c>
       <c r="J66" t="s">
-        <v>404</v>
+        <v>399</v>
       </c>
       <c r="K66" t="s">
-        <v>405</v>
+        <v>400</v>
       </c>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
       <c r="B67" t="s">
-        <v>406</v>
+        <v>401</v>
       </c>
       <c r="C67" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="D67" t="s">
-        <v>407</v>
+        <v>402</v>
       </c>
       <c r="E67">
         <v>6</v>
@@ -4150,33 +4148,33 @@
         <v>12</v>
       </c>
       <c r="G67" t="s">
-        <v>408</v>
+        <v>403</v>
       </c>
       <c r="H67" t="s">
-        <v>409</v>
+        <v>404</v>
       </c>
       <c r="I67" t="s">
-        <v>410</v>
+        <v>405</v>
       </c>
       <c r="J67" t="s">
-        <v>411</v>
+        <v>406</v>
       </c>
       <c r="K67" t="s">
-        <v>412</v>
+        <v>407</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>406</v>
+        <v>401</v>
       </c>
       <c r="B68" t="s">
-        <v>413</v>
+        <v>408</v>
       </c>
       <c r="C68" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="D68" t="s">
-        <v>414</v>
+        <v>409</v>
       </c>
       <c r="E68">
         <v>7</v>
@@ -4185,33 +4183,33 @@
         <v>15</v>
       </c>
       <c r="G68" t="s">
-        <v>415</v>
+        <v>410</v>
       </c>
       <c r="H68" t="s">
-        <v>416</v>
+        <v>411</v>
       </c>
       <c r="I68" t="s">
-        <v>417</v>
+        <v>412</v>
       </c>
       <c r="J68" t="s">
-        <v>418</v>
+        <v>413</v>
       </c>
       <c r="K68" t="s">
-        <v>419</v>
+        <v>414</v>
       </c>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>413</v>
+        <v>408</v>
       </c>
       <c r="B69" t="s">
-        <v>420</v>
+        <v>415</v>
       </c>
       <c r="C69" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="D69" t="s">
-        <v>421</v>
+        <v>416</v>
       </c>
       <c r="E69">
         <v>7</v>
@@ -4220,33 +4218,33 @@
         <v>15</v>
       </c>
       <c r="G69" t="s">
-        <v>422</v>
+        <v>417</v>
       </c>
       <c r="H69" t="s">
-        <v>423</v>
+        <v>418</v>
       </c>
       <c r="I69" t="s">
-        <v>424</v>
+        <v>419</v>
       </c>
       <c r="J69" t="s">
-        <v>425</v>
+        <v>420</v>
       </c>
       <c r="K69" t="s">
-        <v>426</v>
+        <v>421</v>
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>420</v>
+        <v>415</v>
       </c>
       <c r="B70" t="s">
-        <v>427</v>
+        <v>422</v>
       </c>
       <c r="C70" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="D70" t="s">
-        <v>428</v>
+        <v>423</v>
       </c>
       <c r="E70">
         <v>8</v>
@@ -4255,33 +4253,33 @@
         <v>18</v>
       </c>
       <c r="G70" t="s">
-        <v>429</v>
+        <v>424</v>
       </c>
       <c r="H70" t="s">
-        <v>430</v>
+        <v>425</v>
       </c>
       <c r="I70" t="s">
-        <v>431</v>
+        <v>426</v>
       </c>
       <c r="J70" t="s">
-        <v>432</v>
+        <v>427</v>
       </c>
       <c r="K70" t="s">
-        <v>433</v>
+        <v>428</v>
       </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
       <c r="B71" t="s">
-        <v>435</v>
+        <v>430</v>
       </c>
       <c r="C71" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="D71" t="s">
-        <v>436</v>
+        <v>431</v>
       </c>
       <c r="E71">
         <v>8</v>
@@ -4290,33 +4288,33 @@
         <v>18</v>
       </c>
       <c r="G71" t="s">
-        <v>437</v>
+        <v>432</v>
       </c>
       <c r="H71" t="s">
-        <v>438</v>
+        <v>433</v>
       </c>
       <c r="I71" t="s">
-        <v>439</v>
+        <v>434</v>
       </c>
       <c r="J71" t="s">
-        <v>438</v>
+        <v>433</v>
       </c>
       <c r="K71" t="s">
-        <v>440</v>
+        <v>435</v>
       </c>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>435</v>
+        <v>430</v>
       </c>
       <c r="B72" t="s">
-        <v>441</v>
+        <v>436</v>
       </c>
       <c r="C72" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="D72" t="s">
-        <v>442</v>
+        <v>437</v>
       </c>
       <c r="E72">
         <v>9</v>
@@ -4325,33 +4323,33 @@
         <v>24</v>
       </c>
       <c r="G72" t="s">
-        <v>443</v>
+        <v>438</v>
       </c>
       <c r="H72" t="s">
-        <v>445</v>
+        <v>440</v>
       </c>
       <c r="I72" t="s">
-        <v>444</v>
+        <v>439</v>
       </c>
       <c r="J72" t="s">
-        <v>445</v>
+        <v>440</v>
       </c>
       <c r="K72" t="s">
-        <v>446</v>
+        <v>441</v>
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>441</v>
+        <v>436</v>
       </c>
       <c r="B73" t="s">
-        <v>447</v>
+        <v>442</v>
       </c>
       <c r="C73" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="D73" t="s">
-        <v>448</v>
+        <v>443</v>
       </c>
       <c r="E73">
         <v>9</v>
@@ -4360,30 +4358,30 @@
         <v>24</v>
       </c>
       <c r="G73" t="s">
-        <v>449</v>
+        <v>444</v>
       </c>
       <c r="H73" t="s">
-        <v>450</v>
+        <v>445</v>
       </c>
       <c r="I73" t="s">
-        <v>451</v>
+        <v>446</v>
       </c>
       <c r="J73" t="s">
-        <v>450</v>
+        <v>445</v>
       </c>
       <c r="K73" t="s">
-        <v>452</v>
+        <v>447</v>
       </c>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>453</v>
+        <v>448</v>
       </c>
       <c r="B74" t="s">
-        <v>453</v>
+        <v>448</v>
       </c>
       <c r="D74" t="s">
-        <v>454</v>
+        <v>449</v>
       </c>
       <c r="E74">
         <v>10</v>
@@ -4392,27 +4390,27 @@
         <v>30</v>
       </c>
       <c r="G74" t="s">
-        <v>455</v>
+        <v>522</v>
       </c>
       <c r="H74" t="s">
-        <v>456</v>
+        <v>450</v>
       </c>
       <c r="I74" t="s">
-        <v>457</v>
+        <v>451</v>
       </c>
       <c r="J74" t="s">
-        <v>458</v>
+        <v>452</v>
       </c>
       <c r="K74" t="s">
-        <v>459</v>
+        <v>453</v>
       </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>460</v>
+        <v>454</v>
       </c>
       <c r="B75" t="s">
-        <v>460</v>
+        <v>454</v>
       </c>
       <c r="E75">
         <v>10</v>
@@ -4421,27 +4419,27 @@
         <v>30</v>
       </c>
       <c r="G75" t="s">
-        <v>461</v>
+        <v>455</v>
       </c>
       <c r="H75" t="s">
-        <v>463</v>
+        <v>457</v>
       </c>
       <c r="I75" t="s">
-        <v>462</v>
+        <v>456</v>
       </c>
       <c r="J75" t="s">
-        <v>463</v>
+        <v>457</v>
       </c>
       <c r="K75" t="s">
-        <v>464</v>
+        <v>458</v>
       </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>465</v>
+        <v>459</v>
       </c>
       <c r="B76" t="s">
-        <v>466</v>
+        <v>460</v>
       </c>
       <c r="E76">
         <v>11</v>
@@ -4450,27 +4448,27 @@
         <v>36</v>
       </c>
       <c r="G76" t="s">
-        <v>467</v>
+        <v>461</v>
       </c>
       <c r="H76" t="s">
-        <v>469</v>
+        <v>463</v>
       </c>
       <c r="I76" t="s">
-        <v>468</v>
+        <v>462</v>
       </c>
       <c r="J76" t="s">
-        <v>469</v>
+        <v>463</v>
       </c>
       <c r="K76" t="s">
-        <v>470</v>
+        <v>464</v>
       </c>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>471</v>
+        <v>465</v>
       </c>
       <c r="B77" t="s">
-        <v>465</v>
+        <v>459</v>
       </c>
       <c r="E77">
         <v>11</v>
@@ -4479,27 +4477,27 @@
         <v>36</v>
       </c>
       <c r="G77" t="s">
-        <v>472</v>
+        <v>466</v>
       </c>
       <c r="H77" t="s">
-        <v>474</v>
+        <v>468</v>
       </c>
       <c r="I77" t="s">
-        <v>473</v>
+        <v>467</v>
       </c>
       <c r="J77" t="s">
-        <v>474</v>
+        <v>468</v>
       </c>
       <c r="K77" t="s">
-        <v>475</v>
+        <v>469</v>
       </c>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>476</v>
+        <v>470</v>
       </c>
       <c r="B78" t="s">
-        <v>471</v>
+        <v>465</v>
       </c>
       <c r="E78">
         <v>12</v>
@@ -4508,24 +4506,24 @@
         <v>42</v>
       </c>
       <c r="G78" t="s">
-        <v>477</v>
+        <v>471</v>
       </c>
       <c r="H78" t="s">
-        <v>479</v>
+        <v>473</v>
       </c>
       <c r="I78" t="s">
-        <v>478</v>
+        <v>472</v>
       </c>
       <c r="J78" t="s">
-        <v>479</v>
+        <v>473</v>
       </c>
       <c r="K78" t="s">
-        <v>480</v>
+        <v>474</v>
       </c>
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B79" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="E79">
         <v>14</v>
@@ -4534,24 +4532,24 @@
         <v>54</v>
       </c>
       <c r="G79" t="s">
-        <v>481</v>
+        <v>475</v>
       </c>
       <c r="H79" t="s">
-        <v>518</v>
+        <v>511</v>
       </c>
       <c r="I79" t="s">
-        <v>521</v>
+        <v>514</v>
       </c>
       <c r="J79" t="s">
-        <v>518</v>
+        <v>511</v>
       </c>
       <c r="K79" t="s">
-        <v>482</v>
+        <v>476</v>
       </c>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B80" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="E80">
         <v>14</v>
@@ -4560,21 +4558,21 @@
         <v>54</v>
       </c>
       <c r="G80" t="s">
-        <v>483</v>
+        <v>477</v>
       </c>
       <c r="H80" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="I80" t="s">
-        <v>523</v>
+        <v>516</v>
       </c>
       <c r="K80" t="s">
-        <v>484</v>
+        <v>478</v>
       </c>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B81" t="s">
-        <v>476</v>
+        <v>470</v>
       </c>
       <c r="E81">
         <v>14</v>
@@ -4583,21 +4581,21 @@
         <v>54</v>
       </c>
       <c r="G81" t="s">
-        <v>485</v>
+        <v>523</v>
       </c>
       <c r="H81" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="I81" t="s">
-        <v>524</v>
+        <v>517</v>
       </c>
       <c r="K81" t="s">
-        <v>486</v>
+        <v>479</v>
       </c>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.25">
       <c r="D82" t="s">
-        <v>487</v>
+        <v>480</v>
       </c>
       <c r="E82">
         <v>4</v>
@@ -4606,24 +4604,24 @@
         <v>6</v>
       </c>
       <c r="G82" t="s">
-        <v>508</v>
+        <v>501</v>
       </c>
       <c r="H82" t="s">
-        <v>488</v>
+        <v>481</v>
       </c>
       <c r="I82" t="s">
-        <v>514</v>
+        <v>507</v>
       </c>
       <c r="J82" t="s">
-        <v>488</v>
+        <v>481</v>
       </c>
       <c r="K82" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
     </row>
     <row r="83" spans="1:11" x14ac:dyDescent="0.25">
       <c r="D83" t="s">
-        <v>489</v>
+        <v>482</v>
       </c>
       <c r="E83">
         <v>7</v>
@@ -4632,21 +4630,21 @@
         <v>15</v>
       </c>
       <c r="G83" t="s">
-        <v>509</v>
+        <v>502</v>
       </c>
       <c r="H83" t="s">
-        <v>490</v>
+        <v>483</v>
       </c>
       <c r="J83" t="s">
-        <v>490</v>
+        <v>483</v>
       </c>
       <c r="K83" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
     </row>
     <row r="84" spans="1:11" x14ac:dyDescent="0.25">
       <c r="D84" t="s">
-        <v>491</v>
+        <v>484</v>
       </c>
       <c r="E84">
         <v>8</v>
@@ -4655,24 +4653,24 @@
         <v>18</v>
       </c>
       <c r="G84" t="s">
-        <v>510</v>
+        <v>503</v>
       </c>
       <c r="H84" t="s">
-        <v>492</v>
+        <v>485</v>
       </c>
       <c r="I84" t="s">
-        <v>520</v>
+        <v>513</v>
       </c>
       <c r="J84" t="s">
-        <v>492</v>
+        <v>485</v>
       </c>
       <c r="K84" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
     </row>
     <row r="85" spans="1:11" x14ac:dyDescent="0.25">
       <c r="D85" t="s">
-        <v>493</v>
+        <v>486</v>
       </c>
       <c r="E85">
         <v>9</v>
@@ -4681,24 +4679,24 @@
         <v>24</v>
       </c>
       <c r="G85" t="s">
-        <v>511</v>
+        <v>504</v>
       </c>
       <c r="H85" t="s">
-        <v>494</v>
+        <v>487</v>
       </c>
       <c r="I85" t="s">
-        <v>515</v>
+        <v>508</v>
       </c>
       <c r="J85" t="s">
-        <v>494</v>
+        <v>487</v>
       </c>
       <c r="K85" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
     </row>
     <row r="86" spans="1:11" x14ac:dyDescent="0.25">
       <c r="D86" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="E86">
         <v>9</v>
@@ -4707,21 +4705,21 @@
         <v>24</v>
       </c>
       <c r="G86" t="s">
-        <v>512</v>
+        <v>505</v>
       </c>
       <c r="H86" t="s">
-        <v>496</v>
+        <v>489</v>
       </c>
       <c r="J86" t="s">
-        <v>496</v>
+        <v>489</v>
       </c>
       <c r="K86" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
     </row>
     <row r="87" spans="1:11" x14ac:dyDescent="0.25">
       <c r="D87" t="s">
-        <v>497</v>
+        <v>490</v>
       </c>
       <c r="E87">
         <v>10</v>
@@ -4730,33 +4728,33 @@
         <v>30</v>
       </c>
       <c r="G87" t="s">
-        <v>513</v>
+        <v>506</v>
       </c>
       <c r="H87" t="s">
-        <v>498</v>
+        <v>491</v>
       </c>
       <c r="I87" t="s">
-        <v>516</v>
+        <v>509</v>
       </c>
       <c r="J87" t="s">
-        <v>498</v>
+        <v>491</v>
       </c>
       <c r="K87" t="s">
-        <v>499</v>
+        <v>492</v>
       </c>
     </row>
     <row r="88" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="B88" t="s">
-        <v>500</v>
+        <v>493</v>
       </c>
       <c r="C88" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D88" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="E88">
         <v>1</v>
@@ -4765,33 +4763,33 @@
         <v>1</v>
       </c>
       <c r="G88" t="s">
-        <v>506</v>
+        <v>499</v>
       </c>
       <c r="H88" t="s">
-        <v>341</v>
+        <v>337</v>
       </c>
       <c r="I88" t="s">
-        <v>503</v>
+        <v>496</v>
       </c>
       <c r="J88" t="s">
-        <v>343</v>
+        <v>339</v>
       </c>
       <c r="K88" t="s">
-        <v>344</v>
+        <v>340</v>
       </c>
     </row>
     <row r="89" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="B89" t="s">
-        <v>501</v>
+        <v>494</v>
       </c>
       <c r="C89" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D89" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="E89">
         <v>2</v>
@@ -4800,33 +4798,33 @@
         <v>2</v>
       </c>
       <c r="G89" t="s">
-        <v>506</v>
+        <v>499</v>
       </c>
       <c r="H89" t="s">
-        <v>341</v>
+        <v>337</v>
       </c>
       <c r="I89" t="s">
-        <v>504</v>
+        <v>497</v>
       </c>
       <c r="J89" t="s">
-        <v>343</v>
+        <v>339</v>
       </c>
       <c r="K89" t="s">
-        <v>344</v>
+        <v>340</v>
       </c>
     </row>
     <row r="90" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="B90" t="s">
-        <v>502</v>
+        <v>495</v>
       </c>
       <c r="C90" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D90" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="E90">
         <v>3</v>
@@ -4835,19 +4833,19 @@
         <v>3</v>
       </c>
       <c r="G90" t="s">
-        <v>506</v>
+        <v>499</v>
       </c>
       <c r="H90" t="s">
-        <v>341</v>
+        <v>337</v>
       </c>
       <c r="I90" t="s">
-        <v>505</v>
+        <v>498</v>
       </c>
       <c r="J90" t="s">
-        <v>343</v>
+        <v>339</v>
       </c>
       <c r="K90" t="s">
-        <v>344</v>
+        <v>340</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update some english labels in vwo itemtable
</commit_message>
<xml_diff>
--- a/data-raw/data/VWO_itemtable.xlsx
+++ b/data-raw/data/VWO_itemtable.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24931"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eekhouti\Documents\GitHub\dscoreddi\data-raw\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eekhouti\OneDrive - TNO\Documents\GitHub\dscoreddi\data-raw\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C120CEC1-BE40-44B5-B012-3C659F6A7698}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D343584F-F834-412C-99A6-ED54469E9638}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="0" iterate="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="734" uniqueCount="524">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="734" uniqueCount="502">
   <si>
     <t>ID.VWO1996</t>
   </si>
@@ -109,9 +109,6 @@
     <t>Handen af en toe open</t>
   </si>
   <si>
-    <t>Hands open now and then</t>
-  </si>
-  <si>
     <t>ddifmd003</t>
   </si>
   <si>
@@ -133,9 +130,6 @@
     <t>Kijkt naar eigen handen</t>
   </si>
   <si>
-    <t>Looks at own hands</t>
-  </si>
-  <si>
     <t>ddifmm004</t>
   </si>
   <si>
@@ -157,9 +151,6 @@
     <t>Speelt met handen middenvoor</t>
   </si>
   <si>
-    <t>Hands playing in midline</t>
-  </si>
-  <si>
     <t>ddifmd005</t>
   </si>
   <si>
@@ -181,9 +172,6 @@
     <t>Pakt in rugligging voorwerp</t>
   </si>
   <si>
-    <t>Grasps toy within reach</t>
-  </si>
-  <si>
     <t>ddigmd006</t>
   </si>
   <si>
@@ -202,9 +190,6 @@
     <t>Pakt blokje over</t>
   </si>
   <si>
-    <t>Transfers toy easily, hand to hand</t>
-  </si>
-  <si>
     <t>ddifmd007</t>
   </si>
   <si>
@@ -223,9 +208,6 @@
     <t>Houdt blokje vast, pakt er nog een in andere hand</t>
   </si>
   <si>
-    <t>Picks up one small toy, then second</t>
-  </si>
-  <si>
     <t>ddifmd008</t>
   </si>
   <si>
@@ -289,9 +271,6 @@
     <t>Doet blokje in/uit doos</t>
   </si>
   <si>
-    <t>Gets cube into and out of box</t>
-  </si>
-  <si>
     <t>ddifmd011</t>
   </si>
   <si>
@@ -349,9 +328,6 @@
     <t>Gaat op onderzoek uit (M)</t>
   </si>
   <si>
-    <t>Explores room</t>
-  </si>
-  <si>
     <t>ddifmm014</t>
   </si>
   <si>
@@ -436,9 +412,6 @@
     <t>Plaatst ronde vorm in stoof</t>
   </si>
   <si>
-    <t>Puts round figure into place</t>
-  </si>
-  <si>
     <t>ddifmd018</t>
   </si>
   <si>
@@ -592,9 +565,6 @@
     <t>Reageert op toespreken (M)</t>
   </si>
   <si>
-    <t>Reacts to speech</t>
-  </si>
-  <si>
     <t>ddicmm029</t>
   </si>
   <si>
@@ -613,9 +583,6 @@
     <t>Lacht terug (M)</t>
   </si>
   <si>
-    <t>Smiles back</t>
-  </si>
-  <si>
     <t>ddicmm030</t>
   </si>
   <si>
@@ -694,9 +661,6 @@
     <t>Brabbelt bij zijn spel (M)</t>
   </si>
   <si>
-    <t>Jabbering</t>
-  </si>
-  <si>
     <t>ddicmm034</t>
   </si>
   <si>
@@ -733,9 +697,6 @@
     <t>Zwaait dag, dag (M)</t>
   </si>
   <si>
-    <t>Waves bye bye</t>
-  </si>
-  <si>
     <t>ddicmm036</t>
   </si>
   <si>
@@ -754,9 +715,6 @@
     <t>Zegt 2 geluidswoorden met begrip (M)</t>
   </si>
   <si>
-    <t>Uses two words</t>
-  </si>
-  <si>
     <t>ddicmm037</t>
   </si>
   <si>
@@ -823,9 +781,6 @@
     <t>Zegt zinnen van 2 woorden (M)</t>
   </si>
   <si>
-    <t>Makes 2-word sentences</t>
-  </si>
-  <si>
     <t>ddicmm041</t>
   </si>
   <si>
@@ -862,9 +817,6 @@
     <t>Noemt zichzelf mij of ik  (M)</t>
   </si>
   <si>
-    <t>Calls itself by name or I</t>
-  </si>
-  <si>
     <t>ddicmm043</t>
   </si>
   <si>
@@ -880,9 +832,6 @@
     <t>Wijst 5 plaatjes aan in boek</t>
   </si>
   <si>
-    <t>Identifies pictures in book</t>
-  </si>
-  <si>
     <t>ddicmd044</t>
   </si>
   <si>
@@ -1018,9 +967,6 @@
     <t>Blijft hangen bij optillen onder de oksels</t>
   </si>
   <si>
-    <t>Remains positioned when lifted under the armpits</t>
-  </si>
-  <si>
     <t>ddigmd054</t>
   </si>
   <si>
@@ -1051,9 +997,6 @@
     <t>Heft kin even van onderlaag</t>
   </si>
   <si>
-    <t>Lifts chin</t>
-  </si>
-  <si>
     <t>ddigmd056</t>
   </si>
   <si>
@@ -1093,9 +1036,6 @@
     <t>Kijkt rond met 90º geheven hoofd</t>
   </si>
   <si>
-    <t>Holds head up 90 degrees in prone position</t>
-  </si>
-  <si>
     <t>ddigmd058</t>
   </si>
   <si>
@@ -1111,9 +1051,6 @@
     <t>v1452</t>
   </si>
   <si>
-    <t>When lifted vertically, legs bended or trampling</t>
-  </si>
-  <si>
     <t>ddigmd059</t>
   </si>
   <si>
@@ -1132,9 +1069,6 @@
     <t>Rolt zich om van rug naar buik en omgekeerd (M)</t>
   </si>
   <si>
-    <t>Rolls from prone to supine and back</t>
-  </si>
-  <si>
     <t>ddigmm060</t>
   </si>
   <si>
@@ -1153,9 +1087,6 @@
     <t>Kan hoofd goed ophouden in zit</t>
   </si>
   <si>
-    <t>Holds head up in sitting position</t>
-  </si>
-  <si>
     <t>ddigmd061</t>
   </si>
   <si>
@@ -1174,9 +1105,6 @@
     <t>Zit op billen met gestrekte benen</t>
   </si>
   <si>
-    <t>Sits with stretched legs</t>
-  </si>
-  <si>
     <t>ddigmd062</t>
   </si>
   <si>
@@ -1195,9 +1123,6 @@
     <t>Zit stabiel los</t>
   </si>
   <si>
-    <t>Sits without support</t>
-  </si>
-  <si>
     <t>ddigmd063</t>
   </si>
   <si>
@@ -1255,9 +1180,6 @@
     <t>Kruipt, buik vrij van de grond (M)</t>
   </si>
   <si>
-    <t>Crawls, with belly lifted off the ground</t>
-  </si>
-  <si>
     <t>ddigmm066</t>
   </si>
   <si>
@@ -1297,9 +1219,6 @@
     <t>Loopt los</t>
   </si>
   <si>
-    <t>Walks on its own</t>
-  </si>
-  <si>
     <t>ddigmd068</t>
   </si>
   <si>
@@ -1372,9 +1291,6 @@
     <t>v1534</t>
   </si>
   <si>
-    <t>Kicks ball away</t>
-  </si>
-  <si>
     <t>ddigmd071</t>
   </si>
   <si>
@@ -1592,6 +1508,24 @@
   </si>
   <si>
     <t>Kan minstens 5 seconden op een been staan - rl</t>
+  </si>
+  <si>
+    <t>Rolls from prone to spine and back</t>
+  </si>
+  <si>
+    <t>Can stand on one leg for at least 5 seconds</t>
+  </si>
+  <si>
+    <t>Understands analogies and contradictions</t>
+  </si>
+  <si>
+    <t>Understands daily used sentences</t>
+  </si>
+  <si>
+    <t>Reacts to name</t>
+  </si>
+  <si>
+    <t>Makes varying sounds</t>
   </si>
 </sst>
 </file>
@@ -1928,7 +1862,8 @@
   <dimension ref="A1:K90"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="7" max="7" width="79.5703125" customWidth="1"/>
+    <col min="7" max="7" width="58" customWidth="1"/>
+    <col min="8" max="8" width="45.140625" customWidth="1"/>
     <col min="10" max="10" width="55.85546875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1949,7 +1884,7 @@
         <v>4</v>
       </c>
       <c r="F1" t="s">
-        <v>500</v>
+        <v>472</v>
       </c>
       <c r="G1" t="s">
         <v>5</v>
@@ -2060,30 +1995,30 @@
         <v>28</v>
       </c>
       <c r="H4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I4" t="s">
         <v>29</v>
       </c>
-      <c r="I4" t="s">
+      <c r="J4" t="s">
         <v>30</v>
       </c>
-      <c r="J4" t="s">
+      <c r="K4" t="s">
         <v>31</v>
-      </c>
-      <c r="K4" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C5" t="s">
         <v>33</v>
       </c>
-      <c r="B5" t="s">
-        <v>33</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>34</v>
-      </c>
-      <c r="D5" t="s">
-        <v>35</v>
       </c>
       <c r="E5">
         <v>3</v>
@@ -2092,33 +2027,33 @@
         <v>3</v>
       </c>
       <c r="G5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H5" t="s">
         <v>37</v>
       </c>
       <c r="I5" t="s">
+        <v>36</v>
+      </c>
+      <c r="J5" t="s">
+        <v>37</v>
+      </c>
+      <c r="K5" t="s">
         <v>38</v>
-      </c>
-      <c r="J5" t="s">
-        <v>39</v>
-      </c>
-      <c r="K5" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C6" t="s">
+        <v>40</v>
+      </c>
+      <c r="D6" t="s">
         <v>41</v>
-      </c>
-      <c r="B6" t="s">
-        <v>41</v>
-      </c>
-      <c r="C6" t="s">
-        <v>42</v>
-      </c>
-      <c r="D6" t="s">
-        <v>43</v>
       </c>
       <c r="E6">
         <v>4</v>
@@ -2127,33 +2062,33 @@
         <v>6</v>
       </c>
       <c r="G6" t="s">
+        <v>42</v>
+      </c>
+      <c r="H6" t="s">
         <v>44</v>
       </c>
-      <c r="H6" t="s">
+      <c r="I6" t="s">
+        <v>43</v>
+      </c>
+      <c r="J6" t="s">
+        <v>44</v>
+      </c>
+      <c r="K6" t="s">
         <v>45</v>
-      </c>
-      <c r="I6" t="s">
-        <v>46</v>
-      </c>
-      <c r="J6" t="s">
-        <v>47</v>
-      </c>
-      <c r="K6" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B7" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C7" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D7" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="E7">
         <v>4</v>
@@ -2162,19 +2097,19 @@
         <v>6</v>
       </c>
       <c r="G7" t="s">
+        <v>49</v>
+      </c>
+      <c r="H7" t="s">
+        <v>51</v>
+      </c>
+      <c r="I7" t="s">
+        <v>50</v>
+      </c>
+      <c r="J7" t="s">
+        <v>51</v>
+      </c>
+      <c r="K7" t="s">
         <v>52</v>
-      </c>
-      <c r="H7" t="s">
-        <v>53</v>
-      </c>
-      <c r="I7" t="s">
-        <v>54</v>
-      </c>
-      <c r="J7" t="s">
-        <v>55</v>
-      </c>
-      <c r="K7" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
@@ -2185,10 +2120,10 @@
         <v>18</v>
       </c>
       <c r="C8" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D8" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="E8">
         <v>5</v>
@@ -2197,19 +2132,19 @@
         <v>9</v>
       </c>
       <c r="G8" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="H8" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="I8" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="J8" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="K8" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
@@ -2220,10 +2155,10 @@
         <v>26</v>
       </c>
       <c r="C9" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="D9" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="E9">
         <v>5</v>
@@ -2232,33 +2167,33 @@
         <v>9</v>
       </c>
       <c r="G9" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="H9" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="I9" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="J9" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="K9" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B10" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C10" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="D10" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="E10">
         <v>5</v>
@@ -2267,33 +2202,33 @@
         <v>9</v>
       </c>
       <c r="G10" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="H10" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="I10" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="J10" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="K10" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="B11" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="C11" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="D11" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="E11">
         <v>6</v>
@@ -2302,33 +2237,33 @@
         <v>12</v>
       </c>
       <c r="G11" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="H11" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="I11" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="J11" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="K11" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="B12" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="C12" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="D12" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="E12">
         <v>7</v>
@@ -2337,33 +2272,33 @@
         <v>15</v>
       </c>
       <c r="G12" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="H12" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="I12" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="J12" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="K12" t="s">
-        <v>92</v>
+        <v>85</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="B13" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="C13" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="D13" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="E13">
         <v>7</v>
@@ -2372,33 +2307,33 @@
         <v>15</v>
       </c>
       <c r="G13" t="s">
-        <v>518</v>
+        <v>490</v>
       </c>
       <c r="H13" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="I13" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="J13" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="K13" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B14" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C14" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="D14" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="E14">
         <v>8</v>
@@ -2407,33 +2342,33 @@
         <v>18</v>
       </c>
       <c r="G14" t="s">
-        <v>520</v>
+        <v>492</v>
       </c>
       <c r="H14" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="I14" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="J14" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="K14" t="s">
-        <v>105</v>
+        <v>98</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="B15" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C15" t="s">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="D15" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="E15">
         <v>8</v>
@@ -2442,33 +2377,33 @@
         <v>18</v>
       </c>
       <c r="G15" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="H15" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="I15" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="J15" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="K15" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="B16" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="C16" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="D16" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="E16">
         <v>9</v>
@@ -2477,33 +2412,33 @@
         <v>24</v>
       </c>
       <c r="G16" t="s">
-        <v>521</v>
+        <v>493</v>
       </c>
       <c r="H16" t="s">
-        <v>116</v>
+        <v>108</v>
       </c>
       <c r="I16" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="J16" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="K16" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="B17" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="C17" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="D17" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="E17">
         <v>9</v>
@@ -2512,30 +2447,30 @@
         <v>24</v>
       </c>
       <c r="G17" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="H17" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="I17" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="J17" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="K17" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B18" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="D18" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="E18">
         <v>10</v>
@@ -2544,30 +2479,30 @@
         <v>30</v>
       </c>
       <c r="G18" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
       <c r="H18" t="s">
-        <v>131</v>
+        <v>123</v>
       </c>
       <c r="I18" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
       <c r="J18" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="K18" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="B19" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="D19" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="E19">
         <v>10</v>
@@ -2576,30 +2511,30 @@
         <v>30</v>
       </c>
       <c r="G19" t="s">
-        <v>137</v>
+        <v>129</v>
       </c>
       <c r="H19" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="I19" t="s">
-        <v>139</v>
+        <v>130</v>
       </c>
       <c r="J19" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="K19" t="s">
-        <v>141</v>
+        <v>132</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="B20" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D20" t="s">
-        <v>142</v>
+        <v>133</v>
       </c>
       <c r="E20">
         <v>10</v>
@@ -2608,27 +2543,27 @@
         <v>30</v>
       </c>
       <c r="G20" t="s">
-        <v>143</v>
+        <v>134</v>
       </c>
       <c r="H20" t="s">
-        <v>144</v>
+        <v>135</v>
       </c>
       <c r="I20" t="s">
-        <v>145</v>
+        <v>136</v>
       </c>
       <c r="J20" t="s">
-        <v>146</v>
+        <v>137</v>
       </c>
       <c r="K20" t="s">
-        <v>147</v>
+        <v>138</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="B21" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="E21">
         <v>11</v>
@@ -2637,27 +2572,27 @@
         <v>36</v>
       </c>
       <c r="G21" t="s">
-        <v>148</v>
+        <v>139</v>
       </c>
       <c r="H21" t="s">
-        <v>151</v>
+        <v>142</v>
       </c>
       <c r="I21" t="s">
-        <v>150</v>
+        <v>141</v>
       </c>
       <c r="J21" t="s">
-        <v>151</v>
+        <v>142</v>
       </c>
       <c r="K21" t="s">
-        <v>152</v>
+        <v>143</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="B22" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="E22">
         <v>11</v>
@@ -2666,27 +2601,27 @@
         <v>36</v>
       </c>
       <c r="G22" t="s">
-        <v>153</v>
+        <v>144</v>
       </c>
       <c r="H22" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="I22" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
       <c r="J22" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="K22" t="s">
-        <v>156</v>
+        <v>147</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>157</v>
+        <v>148</v>
       </c>
       <c r="B23" t="s">
-        <v>157</v>
+        <v>148</v>
       </c>
       <c r="E23">
         <v>11</v>
@@ -2695,27 +2630,27 @@
         <v>36</v>
       </c>
       <c r="G23" t="s">
-        <v>158</v>
+        <v>149</v>
       </c>
       <c r="H23" t="s">
-        <v>160</v>
+        <v>151</v>
       </c>
       <c r="I23" t="s">
-        <v>159</v>
+        <v>150</v>
       </c>
       <c r="J23" t="s">
-        <v>160</v>
+        <v>151</v>
       </c>
       <c r="K23" t="s">
-        <v>161</v>
+        <v>152</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>162</v>
+        <v>153</v>
       </c>
       <c r="B24" t="s">
-        <v>162</v>
+        <v>153</v>
       </c>
       <c r="E24">
         <v>12</v>
@@ -2724,27 +2659,27 @@
         <v>42</v>
       </c>
       <c r="G24" t="s">
-        <v>163</v>
+        <v>154</v>
       </c>
       <c r="H24" t="s">
-        <v>165</v>
+        <v>156</v>
       </c>
       <c r="I24" t="s">
-        <v>164</v>
+        <v>155</v>
       </c>
       <c r="J24" t="s">
-        <v>165</v>
+        <v>156</v>
       </c>
       <c r="K24" t="s">
-        <v>166</v>
+        <v>157</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="B25" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="E25">
         <v>12</v>
@@ -2753,27 +2688,27 @@
         <v>42</v>
       </c>
       <c r="G25" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="H25" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="I25" t="s">
-        <v>169</v>
+        <v>160</v>
       </c>
       <c r="J25" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="K25" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>172</v>
+        <v>163</v>
       </c>
       <c r="B26" t="s">
-        <v>172</v>
+        <v>163</v>
       </c>
       <c r="E26">
         <v>12</v>
@@ -2782,27 +2717,27 @@
         <v>42</v>
       </c>
       <c r="G26" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="H26" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
       <c r="I26" t="s">
-        <v>174</v>
+        <v>165</v>
       </c>
       <c r="J26" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
       <c r="K26" t="s">
-        <v>176</v>
+        <v>167</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="B27" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="E27">
         <v>13</v>
@@ -2811,27 +2746,27 @@
         <v>48</v>
       </c>
       <c r="G27" t="s">
-        <v>178</v>
+        <v>169</v>
       </c>
       <c r="H27" t="s">
-        <v>180</v>
+        <v>171</v>
       </c>
       <c r="I27" t="s">
-        <v>179</v>
+        <v>170</v>
       </c>
       <c r="J27" t="s">
-        <v>180</v>
+        <v>171</v>
       </c>
       <c r="K27" t="s">
-        <v>181</v>
+        <v>172</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="B28" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="E28">
         <v>13</v>
@@ -2840,33 +2775,33 @@
         <v>48</v>
       </c>
       <c r="G28" t="s">
-        <v>182</v>
+        <v>173</v>
       </c>
       <c r="H28" t="s">
-        <v>184</v>
+        <v>175</v>
       </c>
       <c r="I28" t="s">
-        <v>183</v>
+        <v>174</v>
       </c>
       <c r="J28" t="s">
-        <v>184</v>
+        <v>175</v>
       </c>
       <c r="K28" t="s">
-        <v>185</v>
+        <v>176</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>186</v>
+        <v>177</v>
       </c>
       <c r="B29" t="s">
-        <v>187</v>
+        <v>178</v>
       </c>
       <c r="C29" t="s">
         <v>17</v>
       </c>
       <c r="D29" t="s">
-        <v>188</v>
+        <v>179</v>
       </c>
       <c r="E29">
         <v>1</v>
@@ -2875,33 +2810,33 @@
         <v>1</v>
       </c>
       <c r="G29" t="s">
-        <v>189</v>
+        <v>180</v>
       </c>
       <c r="H29" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
       <c r="I29" t="s">
-        <v>191</v>
+        <v>181</v>
       </c>
       <c r="J29" t="s">
-        <v>192</v>
+        <v>182</v>
       </c>
       <c r="K29" t="s">
-        <v>193</v>
+        <v>183</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>187</v>
+        <v>178</v>
       </c>
       <c r="B30" t="s">
-        <v>194</v>
+        <v>184</v>
       </c>
       <c r="C30" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D30" t="s">
-        <v>195</v>
+        <v>185</v>
       </c>
       <c r="E30">
         <v>2</v>
@@ -2910,33 +2845,33 @@
         <v>2</v>
       </c>
       <c r="G30" t="s">
-        <v>196</v>
+        <v>186</v>
       </c>
       <c r="H30" t="s">
-        <v>197</v>
+        <v>188</v>
       </c>
       <c r="I30" t="s">
-        <v>198</v>
+        <v>187</v>
       </c>
       <c r="J30" t="s">
-        <v>199</v>
+        <v>188</v>
       </c>
       <c r="K30" t="s">
-        <v>200</v>
+        <v>189</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>194</v>
+        <v>184</v>
       </c>
       <c r="B31" t="s">
-        <v>201</v>
+        <v>190</v>
       </c>
       <c r="C31" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="D31" t="s">
-        <v>202</v>
+        <v>191</v>
       </c>
       <c r="E31">
         <v>3</v>
@@ -2945,33 +2880,33 @@
         <v>3</v>
       </c>
       <c r="G31" t="s">
-        <v>203</v>
+        <v>192</v>
       </c>
       <c r="H31" t="s">
-        <v>204</v>
+        <v>193</v>
       </c>
       <c r="I31" t="s">
-        <v>205</v>
+        <v>194</v>
       </c>
       <c r="J31" t="s">
-        <v>206</v>
+        <v>195</v>
       </c>
       <c r="K31" t="s">
-        <v>207</v>
+        <v>196</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>201</v>
+        <v>190</v>
       </c>
       <c r="B32" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="C32" t="s">
-        <v>208</v>
+        <v>197</v>
       </c>
       <c r="D32" t="s">
-        <v>201</v>
+        <v>190</v>
       </c>
       <c r="E32">
         <v>4</v>
@@ -2980,27 +2915,27 @@
         <v>6</v>
       </c>
       <c r="G32" t="s">
-        <v>209</v>
+        <v>198</v>
       </c>
       <c r="H32" t="s">
-        <v>149</v>
+        <v>501</v>
       </c>
       <c r="I32" t="s">
-        <v>210</v>
+        <v>199</v>
       </c>
       <c r="K32" t="s">
-        <v>211</v>
+        <v>200</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="C33" t="s">
-        <v>212</v>
+        <v>201</v>
       </c>
       <c r="D33" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="E33">
         <v>4</v>
@@ -3009,27 +2944,27 @@
         <v>6</v>
       </c>
       <c r="G33" t="s">
-        <v>213</v>
+        <v>202</v>
       </c>
       <c r="H33" t="s">
-        <v>149</v>
+        <v>500</v>
       </c>
       <c r="K33" t="s">
-        <v>214</v>
+        <v>203</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="B34" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="C34" t="s">
-        <v>172</v>
+        <v>163</v>
       </c>
       <c r="D34" t="s">
-        <v>215</v>
+        <v>204</v>
       </c>
       <c r="E34">
         <v>5</v>
@@ -3038,33 +2973,33 @@
         <v>9</v>
       </c>
       <c r="G34" t="s">
-        <v>216</v>
+        <v>205</v>
       </c>
       <c r="H34" t="s">
-        <v>217</v>
+        <v>206</v>
       </c>
       <c r="I34" t="s">
-        <v>218</v>
+        <v>207</v>
       </c>
       <c r="J34" t="s">
-        <v>219</v>
+        <v>208</v>
       </c>
       <c r="K34" t="s">
-        <v>220</v>
+        <v>209</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>221</v>
+        <v>210</v>
       </c>
       <c r="B35" t="s">
-        <v>221</v>
+        <v>210</v>
       </c>
       <c r="C35" t="s">
-        <v>201</v>
+        <v>190</v>
       </c>
       <c r="D35" t="s">
-        <v>222</v>
+        <v>211</v>
       </c>
       <c r="E35">
         <v>6</v>
@@ -3073,33 +3008,33 @@
         <v>12</v>
       </c>
       <c r="G35" t="s">
-        <v>223</v>
+        <v>212</v>
       </c>
       <c r="H35" t="s">
-        <v>224</v>
+        <v>214</v>
       </c>
       <c r="I35" t="s">
-        <v>225</v>
+        <v>213</v>
       </c>
       <c r="J35" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="K35" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>228</v>
+        <v>216</v>
       </c>
       <c r="B36" t="s">
-        <v>228</v>
+        <v>216</v>
       </c>
       <c r="C36" t="s">
-        <v>229</v>
+        <v>217</v>
       </c>
       <c r="D36" t="s">
-        <v>228</v>
+        <v>216</v>
       </c>
       <c r="E36">
         <v>6</v>
@@ -3108,33 +3043,33 @@
         <v>12</v>
       </c>
       <c r="G36" t="s">
-        <v>230</v>
+        <v>218</v>
       </c>
       <c r="H36" t="s">
-        <v>232</v>
+        <v>220</v>
       </c>
       <c r="I36" t="s">
-        <v>231</v>
+        <v>219</v>
       </c>
       <c r="J36" t="s">
-        <v>232</v>
+        <v>220</v>
       </c>
       <c r="K36" t="s">
-        <v>233</v>
+        <v>221</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>228</v>
+        <v>216</v>
       </c>
       <c r="B37" t="s">
-        <v>228</v>
+        <v>216</v>
       </c>
       <c r="C37" t="s">
-        <v>229</v>
+        <v>217</v>
       </c>
       <c r="D37" t="s">
-        <v>228</v>
+        <v>216</v>
       </c>
       <c r="E37">
         <v>6</v>
@@ -3143,33 +3078,33 @@
         <v>12</v>
       </c>
       <c r="G37" t="s">
-        <v>230</v>
+        <v>218</v>
       </c>
       <c r="H37" t="s">
-        <v>232</v>
+        <v>220</v>
       </c>
       <c r="I37" t="s">
-        <v>512</v>
+        <v>484</v>
       </c>
       <c r="J37" t="s">
-        <v>232</v>
+        <v>220</v>
       </c>
       <c r="K37" t="s">
-        <v>233</v>
+        <v>221</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>234</v>
+        <v>222</v>
       </c>
       <c r="B38" t="s">
-        <v>234</v>
+        <v>222</v>
       </c>
       <c r="C38" t="s">
-        <v>194</v>
+        <v>184</v>
       </c>
       <c r="D38" t="s">
-        <v>235</v>
+        <v>223</v>
       </c>
       <c r="E38">
         <v>6</v>
@@ -3178,33 +3113,33 @@
         <v>12</v>
       </c>
       <c r="G38" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="H38" t="s">
-        <v>237</v>
+        <v>226</v>
       </c>
       <c r="I38" t="s">
-        <v>238</v>
+        <v>225</v>
       </c>
       <c r="J38" t="s">
-        <v>239</v>
+        <v>226</v>
       </c>
       <c r="K38" t="s">
-        <v>240</v>
+        <v>227</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>241</v>
+        <v>228</v>
       </c>
       <c r="B39" t="s">
-        <v>241</v>
+        <v>228</v>
       </c>
       <c r="C39" t="s">
-        <v>241</v>
+        <v>228</v>
       </c>
       <c r="D39" t="s">
-        <v>242</v>
+        <v>229</v>
       </c>
       <c r="E39">
         <v>7</v>
@@ -3213,33 +3148,33 @@
         <v>15</v>
       </c>
       <c r="G39" t="s">
-        <v>243</v>
+        <v>230</v>
       </c>
       <c r="H39" t="s">
-        <v>244</v>
+        <v>232</v>
       </c>
       <c r="I39" t="s">
-        <v>245</v>
+        <v>231</v>
       </c>
       <c r="J39" t="s">
-        <v>246</v>
+        <v>232</v>
       </c>
       <c r="K39" t="s">
-        <v>247</v>
+        <v>233</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="B40" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="C40" t="s">
-        <v>248</v>
+        <v>234</v>
       </c>
       <c r="D40" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="E40">
         <v>7</v>
@@ -3248,30 +3183,30 @@
         <v>15</v>
       </c>
       <c r="G40" t="s">
-        <v>249</v>
+        <v>235</v>
       </c>
       <c r="H40" t="s">
-        <v>149</v>
+        <v>499</v>
       </c>
       <c r="I40" t="s">
-        <v>250</v>
+        <v>236</v>
       </c>
       <c r="K40" t="s">
-        <v>251</v>
+        <v>237</v>
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="B41" t="s">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="C41" t="s">
-        <v>252</v>
+        <v>238</v>
       </c>
       <c r="D41" t="s">
-        <v>253</v>
+        <v>239</v>
       </c>
       <c r="E41">
         <v>8</v>
@@ -3280,33 +3215,33 @@
         <v>18</v>
       </c>
       <c r="G41" t="s">
-        <v>515</v>
+        <v>487</v>
       </c>
       <c r="H41" t="s">
-        <v>254</v>
+        <v>240</v>
       </c>
       <c r="I41" t="s">
-        <v>255</v>
+        <v>241</v>
       </c>
       <c r="J41" t="s">
-        <v>256</v>
+        <v>242</v>
       </c>
       <c r="K41" t="s">
-        <v>257</v>
+        <v>243</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>252</v>
+        <v>238</v>
       </c>
       <c r="B42" t="s">
-        <v>252</v>
+        <v>238</v>
       </c>
       <c r="C42" t="s">
-        <v>258</v>
+        <v>244</v>
       </c>
       <c r="D42" t="s">
-        <v>252</v>
+        <v>238</v>
       </c>
       <c r="E42">
         <v>8</v>
@@ -3315,33 +3250,33 @@
         <v>18</v>
       </c>
       <c r="G42" t="s">
-        <v>259</v>
+        <v>245</v>
       </c>
       <c r="H42" t="s">
-        <v>261</v>
+        <v>247</v>
       </c>
       <c r="I42" t="s">
-        <v>260</v>
+        <v>246</v>
       </c>
       <c r="J42" t="s">
-        <v>261</v>
+        <v>247</v>
       </c>
       <c r="K42" t="s">
-        <v>262</v>
+        <v>248</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>252</v>
+        <v>238</v>
       </c>
       <c r="B43" t="s">
-        <v>252</v>
+        <v>238</v>
       </c>
       <c r="C43" t="s">
-        <v>258</v>
+        <v>244</v>
       </c>
       <c r="D43" t="s">
-        <v>252</v>
+        <v>238</v>
       </c>
       <c r="E43">
         <v>8</v>
@@ -3350,33 +3285,33 @@
         <v>18</v>
       </c>
       <c r="G43" t="s">
-        <v>259</v>
+        <v>245</v>
       </c>
       <c r="H43" t="s">
-        <v>261</v>
+        <v>247</v>
       </c>
       <c r="I43" t="s">
-        <v>510</v>
+        <v>482</v>
       </c>
       <c r="J43" t="s">
-        <v>261</v>
+        <v>247</v>
       </c>
       <c r="K43" t="s">
-        <v>262</v>
+        <v>248</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>263</v>
+        <v>249</v>
       </c>
       <c r="B44" t="s">
-        <v>263</v>
+        <v>249</v>
       </c>
       <c r="C44" t="s">
-        <v>264</v>
+        <v>250</v>
       </c>
       <c r="D44" t="s">
-        <v>265</v>
+        <v>251</v>
       </c>
       <c r="E44">
         <v>9</v>
@@ -3385,33 +3320,33 @@
         <v>24</v>
       </c>
       <c r="G44" t="s">
-        <v>266</v>
+        <v>252</v>
       </c>
       <c r="H44" t="s">
-        <v>267</v>
+        <v>254</v>
       </c>
       <c r="I44" t="s">
-        <v>268</v>
+        <v>253</v>
       </c>
       <c r="J44" t="s">
-        <v>269</v>
+        <v>254</v>
       </c>
       <c r="K44" t="s">
-        <v>270</v>
+        <v>255</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>271</v>
+        <v>256</v>
       </c>
       <c r="B45" t="s">
-        <v>271</v>
+        <v>256</v>
       </c>
       <c r="C45" t="s">
-        <v>272</v>
+        <v>257</v>
       </c>
       <c r="D45" t="s">
-        <v>271</v>
+        <v>256</v>
       </c>
       <c r="E45">
         <v>9</v>
@@ -3420,30 +3355,30 @@
         <v>24</v>
       </c>
       <c r="G45" t="s">
-        <v>273</v>
+        <v>258</v>
       </c>
       <c r="H45" t="s">
-        <v>275</v>
+        <v>260</v>
       </c>
       <c r="I45" t="s">
-        <v>274</v>
+        <v>259</v>
       </c>
       <c r="J45" t="s">
-        <v>275</v>
+        <v>260</v>
       </c>
       <c r="K45" t="s">
-        <v>276</v>
+        <v>261</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>277</v>
+        <v>262</v>
       </c>
       <c r="B46" t="s">
-        <v>277</v>
+        <v>262</v>
       </c>
       <c r="D46" t="s">
-        <v>278</v>
+        <v>263</v>
       </c>
       <c r="E46">
         <v>10</v>
@@ -3452,30 +3387,30 @@
         <v>30</v>
       </c>
       <c r="G46" t="s">
-        <v>279</v>
+        <v>264</v>
       </c>
       <c r="H46" t="s">
-        <v>280</v>
+        <v>266</v>
       </c>
       <c r="I46" t="s">
-        <v>281</v>
+        <v>265</v>
       </c>
       <c r="J46" t="s">
-        <v>282</v>
+        <v>266</v>
       </c>
       <c r="K46" t="s">
-        <v>283</v>
+        <v>267</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="B47" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="D47" t="s">
-        <v>284</v>
+        <v>268</v>
       </c>
       <c r="E47">
         <v>10</v>
@@ -3484,27 +3419,27 @@
         <v>30</v>
       </c>
       <c r="G47" t="s">
-        <v>285</v>
+        <v>269</v>
       </c>
       <c r="H47" t="s">
-        <v>286</v>
+        <v>271</v>
       </c>
       <c r="I47" t="s">
-        <v>287</v>
+        <v>270</v>
       </c>
       <c r="J47" t="s">
-        <v>288</v>
+        <v>271</v>
       </c>
       <c r="K47" t="s">
-        <v>289</v>
+        <v>272</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="B48" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="E48">
         <v>11</v>
@@ -3513,27 +3448,27 @@
         <v>36</v>
       </c>
       <c r="G48" t="s">
-        <v>290</v>
+        <v>273</v>
       </c>
       <c r="H48" t="s">
-        <v>292</v>
+        <v>275</v>
       </c>
       <c r="I48" t="s">
-        <v>291</v>
+        <v>274</v>
       </c>
       <c r="J48" t="s">
-        <v>292</v>
+        <v>275</v>
       </c>
       <c r="K48" t="s">
-        <v>293</v>
+        <v>276</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>294</v>
+        <v>277</v>
       </c>
       <c r="B49" t="s">
-        <v>294</v>
+        <v>277</v>
       </c>
       <c r="E49">
         <v>11</v>
@@ -3542,27 +3477,27 @@
         <v>36</v>
       </c>
       <c r="G49" t="s">
-        <v>295</v>
+        <v>278</v>
       </c>
       <c r="H49" t="s">
-        <v>297</v>
+        <v>280</v>
       </c>
       <c r="I49" t="s">
-        <v>296</v>
+        <v>279</v>
       </c>
       <c r="J49" t="s">
-        <v>297</v>
+        <v>280</v>
       </c>
       <c r="K49" t="s">
-        <v>298</v>
+        <v>281</v>
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>264</v>
+        <v>250</v>
       </c>
       <c r="B50" t="s">
-        <v>264</v>
+        <v>250</v>
       </c>
       <c r="E50">
         <v>12</v>
@@ -3571,27 +3506,27 @@
         <v>42</v>
       </c>
       <c r="G50" t="s">
-        <v>299</v>
+        <v>282</v>
       </c>
       <c r="H50" t="s">
-        <v>301</v>
+        <v>284</v>
       </c>
       <c r="I50" t="s">
-        <v>300</v>
+        <v>283</v>
       </c>
       <c r="J50" t="s">
-        <v>301</v>
+        <v>284</v>
       </c>
       <c r="K50" t="s">
-        <v>302</v>
+        <v>285</v>
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>303</v>
+        <v>286</v>
       </c>
       <c r="B51" t="s">
-        <v>303</v>
+        <v>286</v>
       </c>
       <c r="E51">
         <v>12</v>
@@ -3600,27 +3535,27 @@
         <v>42</v>
       </c>
       <c r="G51" t="s">
-        <v>304</v>
+        <v>287</v>
       </c>
       <c r="H51" t="s">
-        <v>306</v>
+        <v>289</v>
       </c>
       <c r="I51" t="s">
-        <v>305</v>
+        <v>288</v>
       </c>
       <c r="J51" t="s">
-        <v>306</v>
+        <v>289</v>
       </c>
       <c r="K51" t="s">
-        <v>307</v>
+        <v>290</v>
       </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>308</v>
+        <v>291</v>
       </c>
       <c r="B52" t="s">
-        <v>308</v>
+        <v>291</v>
       </c>
       <c r="E52">
         <v>13</v>
@@ -3629,27 +3564,27 @@
         <v>48</v>
       </c>
       <c r="G52" t="s">
-        <v>309</v>
+        <v>292</v>
       </c>
       <c r="H52" t="s">
-        <v>311</v>
+        <v>294</v>
       </c>
       <c r="I52" t="s">
-        <v>310</v>
+        <v>293</v>
       </c>
       <c r="J52" t="s">
-        <v>311</v>
+        <v>294</v>
       </c>
       <c r="K52" t="s">
-        <v>312</v>
+        <v>295</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>313</v>
+        <v>296</v>
       </c>
       <c r="B53" t="s">
-        <v>313</v>
+        <v>296</v>
       </c>
       <c r="E53">
         <v>13</v>
@@ -3658,33 +3593,33 @@
         <v>48</v>
       </c>
       <c r="G53" t="s">
-        <v>314</v>
+        <v>297</v>
       </c>
       <c r="H53" t="s">
-        <v>316</v>
+        <v>299</v>
       </c>
       <c r="I53" t="s">
-        <v>315</v>
+        <v>298</v>
       </c>
       <c r="J53" t="s">
-        <v>316</v>
+        <v>299</v>
       </c>
       <c r="K53" t="s">
-        <v>317</v>
+        <v>300</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>208</v>
+        <v>197</v>
       </c>
       <c r="B54" t="s">
-        <v>212</v>
+        <v>201</v>
       </c>
       <c r="C54" t="s">
         <v>25</v>
       </c>
       <c r="D54" t="s">
-        <v>318</v>
+        <v>301</v>
       </c>
       <c r="E54">
         <v>1</v>
@@ -3693,33 +3628,33 @@
         <v>1</v>
       </c>
       <c r="G54" t="s">
-        <v>319</v>
+        <v>302</v>
       </c>
       <c r="H54" t="s">
-        <v>320</v>
+        <v>303</v>
       </c>
       <c r="I54" t="s">
-        <v>321</v>
+        <v>304</v>
       </c>
       <c r="J54" t="s">
-        <v>322</v>
+        <v>305</v>
       </c>
       <c r="K54" t="s">
-        <v>323</v>
+        <v>306</v>
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>212</v>
+        <v>201</v>
       </c>
       <c r="B55" t="s">
-        <v>229</v>
+        <v>217</v>
       </c>
       <c r="C55" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D55" t="s">
-        <v>324</v>
+        <v>307</v>
       </c>
       <c r="E55">
         <v>1</v>
@@ -3728,33 +3663,33 @@
         <v>1</v>
       </c>
       <c r="G55" t="s">
-        <v>325</v>
+        <v>308</v>
       </c>
       <c r="H55" t="s">
-        <v>326</v>
+        <v>309</v>
       </c>
       <c r="I55" t="s">
-        <v>327</v>
+        <v>310</v>
       </c>
       <c r="J55" t="s">
-        <v>328</v>
+        <v>311</v>
       </c>
       <c r="K55" t="s">
-        <v>329</v>
+        <v>312</v>
       </c>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>229</v>
+        <v>217</v>
       </c>
       <c r="B56" t="s">
-        <v>248</v>
+        <v>234</v>
       </c>
       <c r="C56" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="D56" t="s">
-        <v>330</v>
+        <v>313</v>
       </c>
       <c r="E56">
         <v>3</v>
@@ -3763,33 +3698,33 @@
         <v>3</v>
       </c>
       <c r="G56" t="s">
-        <v>331</v>
+        <v>314</v>
       </c>
       <c r="H56" t="s">
-        <v>332</v>
+        <v>316</v>
       </c>
       <c r="I56" t="s">
-        <v>333</v>
+        <v>315</v>
       </c>
       <c r="J56" t="s">
-        <v>334</v>
+        <v>316</v>
       </c>
       <c r="K56" t="s">
-        <v>335</v>
+        <v>317</v>
       </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>248</v>
+        <v>234</v>
       </c>
       <c r="B57" t="s">
-        <v>258</v>
+        <v>244</v>
       </c>
       <c r="C57" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="D57" t="s">
-        <v>336</v>
+        <v>318</v>
       </c>
       <c r="E57">
         <v>4</v>
@@ -3798,33 +3733,33 @@
         <v>6</v>
       </c>
       <c r="G57" t="s">
-        <v>499</v>
+        <v>471</v>
       </c>
       <c r="H57" t="s">
-        <v>337</v>
+        <v>319</v>
       </c>
       <c r="I57" t="s">
-        <v>338</v>
+        <v>320</v>
       </c>
       <c r="J57" t="s">
-        <v>339</v>
+        <v>321</v>
       </c>
       <c r="K57" t="s">
-        <v>340</v>
+        <v>322</v>
       </c>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>258</v>
+        <v>244</v>
       </c>
       <c r="B58" t="s">
-        <v>272</v>
+        <v>257</v>
       </c>
       <c r="C58" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D58" t="s">
-        <v>341</v>
+        <v>323</v>
       </c>
       <c r="E58">
         <v>1</v>
@@ -3833,33 +3768,33 @@
         <v>1</v>
       </c>
       <c r="G58" t="s">
-        <v>342</v>
+        <v>324</v>
       </c>
       <c r="H58" t="s">
-        <v>343</v>
+        <v>326</v>
       </c>
       <c r="I58" t="s">
-        <v>344</v>
+        <v>325</v>
       </c>
       <c r="J58" t="s">
-        <v>345</v>
+        <v>326</v>
       </c>
       <c r="K58" t="s">
-        <v>346</v>
+        <v>327</v>
       </c>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>272</v>
+        <v>257</v>
       </c>
       <c r="B59" t="s">
-        <v>347</v>
+        <v>328</v>
       </c>
       <c r="C59" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="D59" t="s">
-        <v>348</v>
+        <v>329</v>
       </c>
       <c r="E59">
         <v>3</v>
@@ -3868,33 +3803,33 @@
         <v>3</v>
       </c>
       <c r="G59" t="s">
-        <v>349</v>
+        <v>330</v>
       </c>
       <c r="H59" t="s">
-        <v>350</v>
+        <v>331</v>
       </c>
       <c r="I59" t="s">
-        <v>351</v>
+        <v>332</v>
       </c>
       <c r="J59" t="s">
-        <v>352</v>
+        <v>333</v>
       </c>
       <c r="K59" t="s">
-        <v>353</v>
+        <v>334</v>
       </c>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>347</v>
+        <v>328</v>
       </c>
       <c r="B60" t="s">
-        <v>354</v>
+        <v>335</v>
       </c>
       <c r="C60" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="D60" t="s">
-        <v>355</v>
+        <v>336</v>
       </c>
       <c r="E60">
         <v>4</v>
@@ -3903,33 +3838,33 @@
         <v>6</v>
       </c>
       <c r="G60" t="s">
-        <v>356</v>
+        <v>337</v>
       </c>
       <c r="H60" t="s">
-        <v>357</v>
+        <v>339</v>
       </c>
       <c r="I60" t="s">
-        <v>358</v>
+        <v>338</v>
       </c>
       <c r="J60" t="s">
-        <v>359</v>
+        <v>339</v>
       </c>
       <c r="K60" t="s">
-        <v>360</v>
+        <v>340</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>354</v>
+        <v>335</v>
       </c>
       <c r="B61" t="s">
-        <v>361</v>
+        <v>341</v>
       </c>
       <c r="C61" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="D61" t="s">
-        <v>362</v>
+        <v>342</v>
       </c>
       <c r="E61">
         <v>4</v>
@@ -3938,33 +3873,33 @@
         <v>6</v>
       </c>
       <c r="G61" t="s">
-        <v>519</v>
+        <v>491</v>
       </c>
       <c r="H61" t="s">
-        <v>363</v>
+        <v>344</v>
       </c>
       <c r="I61" t="s">
-        <v>364</v>
+        <v>343</v>
       </c>
       <c r="J61" t="s">
-        <v>365</v>
+        <v>344</v>
       </c>
       <c r="K61" t="s">
-        <v>366</v>
+        <v>345</v>
       </c>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>361</v>
+        <v>341</v>
       </c>
       <c r="B62" t="s">
-        <v>367</v>
+        <v>346</v>
       </c>
       <c r="C62" t="s">
-        <v>157</v>
+        <v>148</v>
       </c>
       <c r="D62" t="s">
-        <v>368</v>
+        <v>347</v>
       </c>
       <c r="E62">
         <v>5</v>
@@ -3973,33 +3908,33 @@
         <v>9</v>
       </c>
       <c r="G62" t="s">
-        <v>369</v>
+        <v>348</v>
       </c>
       <c r="H62" t="s">
-        <v>370</v>
+        <v>496</v>
       </c>
       <c r="I62" t="s">
-        <v>371</v>
+        <v>349</v>
       </c>
       <c r="J62" t="s">
-        <v>372</v>
+        <v>350</v>
       </c>
       <c r="K62" t="s">
-        <v>373</v>
+        <v>351</v>
       </c>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>367</v>
+        <v>346</v>
       </c>
       <c r="B63" t="s">
-        <v>374</v>
+        <v>352</v>
       </c>
       <c r="C63" t="s">
-        <v>162</v>
+        <v>153</v>
       </c>
       <c r="D63" t="s">
-        <v>375</v>
+        <v>353</v>
       </c>
       <c r="E63">
         <v>5</v>
@@ -4008,33 +3943,33 @@
         <v>9</v>
       </c>
       <c r="G63" t="s">
-        <v>376</v>
+        <v>354</v>
       </c>
       <c r="H63" t="s">
-        <v>377</v>
+        <v>356</v>
       </c>
       <c r="I63" t="s">
-        <v>378</v>
+        <v>355</v>
       </c>
       <c r="J63" t="s">
-        <v>379</v>
+        <v>356</v>
       </c>
       <c r="K63" t="s">
-        <v>380</v>
+        <v>357</v>
       </c>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>374</v>
+        <v>352</v>
       </c>
       <c r="B64" t="s">
-        <v>381</v>
+        <v>358</v>
       </c>
       <c r="C64" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="D64" t="s">
-        <v>382</v>
+        <v>359</v>
       </c>
       <c r="E64">
         <v>5</v>
@@ -4043,33 +3978,33 @@
         <v>9</v>
       </c>
       <c r="G64" t="s">
-        <v>383</v>
+        <v>360</v>
       </c>
       <c r="H64" t="s">
-        <v>384</v>
+        <v>362</v>
       </c>
       <c r="I64" t="s">
-        <v>385</v>
+        <v>361</v>
       </c>
       <c r="J64" t="s">
-        <v>386</v>
+        <v>362</v>
       </c>
       <c r="K64" t="s">
-        <v>387</v>
+        <v>363</v>
       </c>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>381</v>
+        <v>358</v>
       </c>
       <c r="B65" t="s">
-        <v>388</v>
+        <v>364</v>
       </c>
       <c r="C65" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="D65" t="s">
-        <v>389</v>
+        <v>365</v>
       </c>
       <c r="E65">
         <v>6</v>
@@ -4078,33 +4013,33 @@
         <v>12</v>
       </c>
       <c r="G65" t="s">
-        <v>390</v>
+        <v>366</v>
       </c>
       <c r="H65" t="s">
-        <v>391</v>
+        <v>368</v>
       </c>
       <c r="I65" t="s">
-        <v>392</v>
+        <v>367</v>
       </c>
       <c r="J65" t="s">
-        <v>393</v>
+        <v>368</v>
       </c>
       <c r="K65" t="s">
-        <v>394</v>
+        <v>369</v>
       </c>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>388</v>
+        <v>364</v>
       </c>
       <c r="B66" t="s">
-        <v>395</v>
+        <v>370</v>
       </c>
       <c r="C66" t="s">
-        <v>186</v>
+        <v>177</v>
       </c>
       <c r="D66" t="s">
-        <v>396</v>
+        <v>371</v>
       </c>
       <c r="E66">
         <v>6</v>
@@ -4113,33 +4048,33 @@
         <v>12</v>
       </c>
       <c r="G66" t="s">
-        <v>397</v>
+        <v>372</v>
       </c>
       <c r="H66" t="s">
-        <v>399</v>
+        <v>374</v>
       </c>
       <c r="I66" t="s">
-        <v>398</v>
+        <v>373</v>
       </c>
       <c r="J66" t="s">
-        <v>399</v>
+        <v>374</v>
       </c>
       <c r="K66" t="s">
-        <v>400</v>
+        <v>375</v>
       </c>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>395</v>
+        <v>370</v>
       </c>
       <c r="B67" t="s">
-        <v>401</v>
+        <v>376</v>
       </c>
       <c r="C67" t="s">
-        <v>187</v>
+        <v>178</v>
       </c>
       <c r="D67" t="s">
-        <v>402</v>
+        <v>377</v>
       </c>
       <c r="E67">
         <v>6</v>
@@ -4148,33 +4083,33 @@
         <v>12</v>
       </c>
       <c r="G67" t="s">
-        <v>403</v>
+        <v>378</v>
       </c>
       <c r="H67" t="s">
-        <v>404</v>
+        <v>379</v>
       </c>
       <c r="I67" t="s">
-        <v>405</v>
+        <v>380</v>
       </c>
       <c r="J67" t="s">
-        <v>406</v>
+        <v>381</v>
       </c>
       <c r="K67" t="s">
-        <v>407</v>
+        <v>382</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>401</v>
+        <v>376</v>
       </c>
       <c r="B68" t="s">
-        <v>408</v>
+        <v>383</v>
       </c>
       <c r="C68" t="s">
-        <v>221</v>
+        <v>210</v>
       </c>
       <c r="D68" t="s">
-        <v>409</v>
+        <v>384</v>
       </c>
       <c r="E68">
         <v>7</v>
@@ -4183,33 +4118,33 @@
         <v>15</v>
       </c>
       <c r="G68" t="s">
-        <v>410</v>
+        <v>385</v>
       </c>
       <c r="H68" t="s">
-        <v>411</v>
+        <v>387</v>
       </c>
       <c r="I68" t="s">
-        <v>412</v>
+        <v>386</v>
       </c>
       <c r="J68" t="s">
-        <v>413</v>
+        <v>387</v>
       </c>
       <c r="K68" t="s">
-        <v>414</v>
+        <v>388</v>
       </c>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>408</v>
+        <v>383</v>
       </c>
       <c r="B69" t="s">
-        <v>415</v>
+        <v>389</v>
       </c>
       <c r="C69" t="s">
-        <v>228</v>
+        <v>216</v>
       </c>
       <c r="D69" t="s">
-        <v>416</v>
+        <v>390</v>
       </c>
       <c r="E69">
         <v>7</v>
@@ -4218,33 +4153,33 @@
         <v>15</v>
       </c>
       <c r="G69" t="s">
-        <v>417</v>
+        <v>391</v>
       </c>
       <c r="H69" t="s">
-        <v>418</v>
+        <v>392</v>
       </c>
       <c r="I69" t="s">
-        <v>419</v>
+        <v>393</v>
       </c>
       <c r="J69" t="s">
-        <v>420</v>
+        <v>394</v>
       </c>
       <c r="K69" t="s">
-        <v>421</v>
+        <v>395</v>
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>415</v>
+        <v>389</v>
       </c>
       <c r="B70" t="s">
-        <v>422</v>
+        <v>396</v>
       </c>
       <c r="C70" t="s">
-        <v>271</v>
+        <v>256</v>
       </c>
       <c r="D70" t="s">
-        <v>423</v>
+        <v>397</v>
       </c>
       <c r="E70">
         <v>8</v>
@@ -4253,33 +4188,33 @@
         <v>18</v>
       </c>
       <c r="G70" t="s">
-        <v>424</v>
+        <v>398</v>
       </c>
       <c r="H70" t="s">
-        <v>425</v>
+        <v>400</v>
       </c>
       <c r="I70" t="s">
-        <v>426</v>
+        <v>399</v>
       </c>
       <c r="J70" t="s">
-        <v>427</v>
+        <v>400</v>
       </c>
       <c r="K70" t="s">
-        <v>428</v>
+        <v>401</v>
       </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>429</v>
+        <v>402</v>
       </c>
       <c r="B71" t="s">
-        <v>430</v>
+        <v>403</v>
       </c>
       <c r="C71" t="s">
-        <v>277</v>
+        <v>262</v>
       </c>
       <c r="D71" t="s">
-        <v>431</v>
+        <v>404</v>
       </c>
       <c r="E71">
         <v>8</v>
@@ -4288,33 +4223,33 @@
         <v>18</v>
       </c>
       <c r="G71" t="s">
-        <v>432</v>
+        <v>405</v>
       </c>
       <c r="H71" t="s">
-        <v>433</v>
+        <v>406</v>
       </c>
       <c r="I71" t="s">
-        <v>434</v>
+        <v>407</v>
       </c>
       <c r="J71" t="s">
-        <v>433</v>
+        <v>406</v>
       </c>
       <c r="K71" t="s">
-        <v>435</v>
+        <v>408</v>
       </c>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>430</v>
+        <v>403</v>
       </c>
       <c r="B72" t="s">
-        <v>436</v>
+        <v>409</v>
       </c>
       <c r="C72" t="s">
-        <v>308</v>
+        <v>291</v>
       </c>
       <c r="D72" t="s">
-        <v>437</v>
+        <v>410</v>
       </c>
       <c r="E72">
         <v>9</v>
@@ -4323,33 +4258,33 @@
         <v>24</v>
       </c>
       <c r="G72" t="s">
-        <v>438</v>
+        <v>411</v>
       </c>
       <c r="H72" t="s">
-        <v>440</v>
+        <v>413</v>
       </c>
       <c r="I72" t="s">
-        <v>439</v>
+        <v>412</v>
       </c>
       <c r="J72" t="s">
-        <v>440</v>
+        <v>413</v>
       </c>
       <c r="K72" t="s">
-        <v>441</v>
+        <v>414</v>
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>436</v>
+        <v>409</v>
       </c>
       <c r="B73" t="s">
-        <v>442</v>
+        <v>415</v>
       </c>
       <c r="C73" t="s">
-        <v>313</v>
+        <v>296</v>
       </c>
       <c r="D73" t="s">
-        <v>443</v>
+        <v>416</v>
       </c>
       <c r="E73">
         <v>9</v>
@@ -4358,30 +4293,30 @@
         <v>24</v>
       </c>
       <c r="G73" t="s">
-        <v>444</v>
+        <v>417</v>
       </c>
       <c r="H73" t="s">
-        <v>445</v>
+        <v>418</v>
       </c>
       <c r="I73" t="s">
-        <v>446</v>
+        <v>419</v>
       </c>
       <c r="J73" t="s">
-        <v>445</v>
+        <v>418</v>
       </c>
       <c r="K73" t="s">
-        <v>447</v>
+        <v>420</v>
       </c>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>448</v>
+        <v>421</v>
       </c>
       <c r="B74" t="s">
-        <v>448</v>
+        <v>421</v>
       </c>
       <c r="D74" t="s">
-        <v>449</v>
+        <v>422</v>
       </c>
       <c r="E74">
         <v>10</v>
@@ -4390,27 +4325,27 @@
         <v>30</v>
       </c>
       <c r="G74" t="s">
-        <v>522</v>
+        <v>494</v>
       </c>
       <c r="H74" t="s">
-        <v>450</v>
+        <v>424</v>
       </c>
       <c r="I74" t="s">
-        <v>451</v>
+        <v>423</v>
       </c>
       <c r="J74" t="s">
-        <v>452</v>
+        <v>424</v>
       </c>
       <c r="K74" t="s">
-        <v>453</v>
+        <v>425</v>
       </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>454</v>
+        <v>426</v>
       </c>
       <c r="B75" t="s">
-        <v>454</v>
+        <v>426</v>
       </c>
       <c r="E75">
         <v>10</v>
@@ -4419,27 +4354,27 @@
         <v>30</v>
       </c>
       <c r="G75" t="s">
-        <v>455</v>
+        <v>427</v>
       </c>
       <c r="H75" t="s">
-        <v>457</v>
+        <v>429</v>
       </c>
       <c r="I75" t="s">
-        <v>456</v>
+        <v>428</v>
       </c>
       <c r="J75" t="s">
-        <v>457</v>
+        <v>429</v>
       </c>
       <c r="K75" t="s">
-        <v>458</v>
+        <v>430</v>
       </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>459</v>
+        <v>431</v>
       </c>
       <c r="B76" t="s">
-        <v>460</v>
+        <v>432</v>
       </c>
       <c r="E76">
         <v>11</v>
@@ -4448,27 +4383,27 @@
         <v>36</v>
       </c>
       <c r="G76" t="s">
-        <v>461</v>
+        <v>433</v>
       </c>
       <c r="H76" t="s">
-        <v>463</v>
+        <v>435</v>
       </c>
       <c r="I76" t="s">
-        <v>462</v>
+        <v>434</v>
       </c>
       <c r="J76" t="s">
-        <v>463</v>
+        <v>435</v>
       </c>
       <c r="K76" t="s">
-        <v>464</v>
+        <v>436</v>
       </c>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>465</v>
+        <v>437</v>
       </c>
       <c r="B77" t="s">
-        <v>459</v>
+        <v>431</v>
       </c>
       <c r="E77">
         <v>11</v>
@@ -4477,27 +4412,27 @@
         <v>36</v>
       </c>
       <c r="G77" t="s">
-        <v>466</v>
+        <v>438</v>
       </c>
       <c r="H77" t="s">
-        <v>468</v>
+        <v>440</v>
       </c>
       <c r="I77" t="s">
-        <v>467</v>
+        <v>439</v>
       </c>
       <c r="J77" t="s">
-        <v>468</v>
+        <v>440</v>
       </c>
       <c r="K77" t="s">
-        <v>469</v>
+        <v>441</v>
       </c>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>470</v>
+        <v>442</v>
       </c>
       <c r="B78" t="s">
-        <v>465</v>
+        <v>437</v>
       </c>
       <c r="E78">
         <v>12</v>
@@ -4506,24 +4441,24 @@
         <v>42</v>
       </c>
       <c r="G78" t="s">
-        <v>471</v>
+        <v>443</v>
       </c>
       <c r="H78" t="s">
-        <v>473</v>
+        <v>445</v>
       </c>
       <c r="I78" t="s">
-        <v>472</v>
+        <v>444</v>
       </c>
       <c r="J78" t="s">
-        <v>473</v>
+        <v>445</v>
       </c>
       <c r="K78" t="s">
-        <v>474</v>
+        <v>446</v>
       </c>
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B79" t="s">
-        <v>186</v>
+        <v>177</v>
       </c>
       <c r="E79">
         <v>14</v>
@@ -4532,24 +4467,24 @@
         <v>54</v>
       </c>
       <c r="G79" t="s">
-        <v>475</v>
+        <v>447</v>
       </c>
       <c r="H79" t="s">
-        <v>511</v>
+        <v>483</v>
       </c>
       <c r="I79" t="s">
-        <v>514</v>
+        <v>486</v>
       </c>
       <c r="J79" t="s">
-        <v>511</v>
+        <v>483</v>
       </c>
       <c r="K79" t="s">
-        <v>476</v>
+        <v>448</v>
       </c>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B80" t="s">
-        <v>208</v>
+        <v>197</v>
       </c>
       <c r="E80">
         <v>14</v>
@@ -4558,21 +4493,21 @@
         <v>54</v>
       </c>
       <c r="G80" t="s">
-        <v>477</v>
+        <v>449</v>
       </c>
       <c r="H80" t="s">
-        <v>149</v>
+        <v>498</v>
       </c>
       <c r="I80" t="s">
-        <v>516</v>
+        <v>488</v>
       </c>
       <c r="K80" t="s">
-        <v>478</v>
+        <v>450</v>
       </c>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B81" t="s">
-        <v>470</v>
+        <v>442</v>
       </c>
       <c r="E81">
         <v>14</v>
@@ -4581,21 +4516,21 @@
         <v>54</v>
       </c>
       <c r="G81" t="s">
-        <v>523</v>
+        <v>495</v>
       </c>
       <c r="H81" t="s">
-        <v>149</v>
+        <v>497</v>
       </c>
       <c r="I81" t="s">
-        <v>517</v>
+        <v>489</v>
       </c>
       <c r="K81" t="s">
-        <v>479</v>
+        <v>451</v>
       </c>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.25">
       <c r="D82" t="s">
-        <v>480</v>
+        <v>452</v>
       </c>
       <c r="E82">
         <v>4</v>
@@ -4604,24 +4539,24 @@
         <v>6</v>
       </c>
       <c r="G82" t="s">
-        <v>501</v>
+        <v>473</v>
       </c>
       <c r="H82" t="s">
-        <v>481</v>
+        <v>453</v>
       </c>
       <c r="I82" t="s">
-        <v>507</v>
+        <v>479</v>
       </c>
       <c r="J82" t="s">
-        <v>481</v>
+        <v>453</v>
       </c>
       <c r="K82" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
     </row>
     <row r="83" spans="1:11" x14ac:dyDescent="0.25">
       <c r="D83" t="s">
-        <v>482</v>
+        <v>454</v>
       </c>
       <c r="E83">
         <v>7</v>
@@ -4630,21 +4565,21 @@
         <v>15</v>
       </c>
       <c r="G83" t="s">
-        <v>502</v>
+        <v>474</v>
       </c>
       <c r="H83" t="s">
-        <v>483</v>
+        <v>455</v>
       </c>
       <c r="J83" t="s">
-        <v>483</v>
+        <v>455</v>
       </c>
       <c r="K83" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
     </row>
     <row r="84" spans="1:11" x14ac:dyDescent="0.25">
       <c r="D84" t="s">
-        <v>484</v>
+        <v>456</v>
       </c>
       <c r="E84">
         <v>8</v>
@@ -4653,24 +4588,24 @@
         <v>18</v>
       </c>
       <c r="G84" t="s">
-        <v>503</v>
+        <v>475</v>
       </c>
       <c r="H84" t="s">
+        <v>457</v>
+      </c>
+      <c r="I84" t="s">
         <v>485</v>
       </c>
-      <c r="I84" t="s">
-        <v>513</v>
-      </c>
       <c r="J84" t="s">
-        <v>485</v>
+        <v>457</v>
       </c>
       <c r="K84" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
     </row>
     <row r="85" spans="1:11" x14ac:dyDescent="0.25">
       <c r="D85" t="s">
-        <v>486</v>
+        <v>458</v>
       </c>
       <c r="E85">
         <v>9</v>
@@ -4679,24 +4614,24 @@
         <v>24</v>
       </c>
       <c r="G85" t="s">
-        <v>504</v>
+        <v>476</v>
       </c>
       <c r="H85" t="s">
-        <v>487</v>
+        <v>459</v>
       </c>
       <c r="I85" t="s">
-        <v>508</v>
+        <v>480</v>
       </c>
       <c r="J85" t="s">
-        <v>487</v>
+        <v>459</v>
       </c>
       <c r="K85" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
     </row>
     <row r="86" spans="1:11" x14ac:dyDescent="0.25">
       <c r="D86" t="s">
-        <v>488</v>
+        <v>460</v>
       </c>
       <c r="E86">
         <v>9</v>
@@ -4705,21 +4640,21 @@
         <v>24</v>
       </c>
       <c r="G86" t="s">
-        <v>505</v>
+        <v>477</v>
       </c>
       <c r="H86" t="s">
-        <v>489</v>
+        <v>461</v>
       </c>
       <c r="J86" t="s">
-        <v>489</v>
+        <v>461</v>
       </c>
       <c r="K86" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
     </row>
     <row r="87" spans="1:11" x14ac:dyDescent="0.25">
       <c r="D87" t="s">
-        <v>490</v>
+        <v>462</v>
       </c>
       <c r="E87">
         <v>10</v>
@@ -4728,33 +4663,33 @@
         <v>30</v>
       </c>
       <c r="G87" t="s">
-        <v>506</v>
+        <v>478</v>
       </c>
       <c r="H87" t="s">
-        <v>491</v>
+        <v>463</v>
       </c>
       <c r="I87" t="s">
-        <v>509</v>
+        <v>481</v>
       </c>
       <c r="J87" t="s">
-        <v>491</v>
+        <v>463</v>
       </c>
       <c r="K87" t="s">
-        <v>492</v>
+        <v>464</v>
       </c>
     </row>
     <row r="88" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>248</v>
+        <v>234</v>
       </c>
       <c r="B88" t="s">
-        <v>493</v>
+        <v>465</v>
       </c>
       <c r="C88" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="D88" t="s">
-        <v>336</v>
+        <v>318</v>
       </c>
       <c r="E88">
         <v>1</v>
@@ -4763,33 +4698,33 @@
         <v>1</v>
       </c>
       <c r="G88" t="s">
-        <v>499</v>
+        <v>471</v>
       </c>
       <c r="H88" t="s">
-        <v>337</v>
+        <v>319</v>
       </c>
       <c r="I88" t="s">
-        <v>496</v>
+        <v>468</v>
       </c>
       <c r="J88" t="s">
-        <v>339</v>
+        <v>321</v>
       </c>
       <c r="K88" t="s">
-        <v>340</v>
+        <v>322</v>
       </c>
     </row>
     <row r="89" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>248</v>
+        <v>234</v>
       </c>
       <c r="B89" t="s">
-        <v>494</v>
+        <v>466</v>
       </c>
       <c r="C89" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="D89" t="s">
-        <v>336</v>
+        <v>318</v>
       </c>
       <c r="E89">
         <v>2</v>
@@ -4798,33 +4733,33 @@
         <v>2</v>
       </c>
       <c r="G89" t="s">
-        <v>499</v>
+        <v>471</v>
       </c>
       <c r="H89" t="s">
-        <v>337</v>
+        <v>319</v>
       </c>
       <c r="I89" t="s">
-        <v>497</v>
+        <v>469</v>
       </c>
       <c r="J89" t="s">
-        <v>339</v>
+        <v>321</v>
       </c>
       <c r="K89" t="s">
-        <v>340</v>
+        <v>322</v>
       </c>
     </row>
     <row r="90" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>248</v>
+        <v>234</v>
       </c>
       <c r="B90" t="s">
-        <v>495</v>
+        <v>467</v>
       </c>
       <c r="C90" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="D90" t="s">
-        <v>336</v>
+        <v>318</v>
       </c>
       <c r="E90">
         <v>3</v>
@@ -4833,19 +4768,19 @@
         <v>3</v>
       </c>
       <c r="G90" t="s">
-        <v>499</v>
+        <v>471</v>
       </c>
       <c r="H90" t="s">
-        <v>337</v>
+        <v>319</v>
       </c>
       <c r="I90" t="s">
-        <v>498</v>
+        <v>470</v>
       </c>
       <c r="J90" t="s">
-        <v>339</v>
+        <v>321</v>
       </c>
       <c r="K90" t="s">
-        <v>340</v>
+        <v>322</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
edit some of the labelNL kenmerk labels in overeenstemming met informatie NCJ.
</commit_message>
<xml_diff>
--- a/data-raw/data/VWO_itemtable.xlsx
+++ b/data-raw/data/VWO_itemtable.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24931"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26130"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eekhouti\OneDrive - TNO\Documents\GitHub\dscoreddi\data-raw\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://365tno-my.sharepoint.com/personal/iris_eekhout_tno_nl/Documents/Documents/GitHub/dscoreddi/data-raw/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D343584F-F834-412C-99A6-ED54469E9638}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="101" documentId="13_ncr:1_{D343584F-F834-412C-99A6-ED54469E9638}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A2F8589F-9F7E-406B-A92F-77176A54D483}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="54600" yWindow="0" windowWidth="25800" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0" iterate="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="734" uniqueCount="502">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="732" uniqueCount="503">
   <si>
     <t>ID.VWO1996</t>
   </si>
@@ -106,9 +106,6 @@
     <t>v1440</t>
   </si>
   <si>
-    <t>Handen af en toe open</t>
-  </si>
-  <si>
     <t>ddifmd003</t>
   </si>
   <si>
@@ -169,9 +166,6 @@
     <t>v1447</t>
   </si>
   <si>
-    <t>Pakt in rugligging voorwerp</t>
-  </si>
-  <si>
     <t>ddigmd006</t>
   </si>
   <si>
@@ -694,9 +688,6 @@
     <t>v1468</t>
   </si>
   <si>
-    <t>Zwaait dag, dag (M)</t>
-  </si>
-  <si>
     <t>ddicmm036</t>
   </si>
   <si>
@@ -868,9 +859,6 @@
     <t>Isverstaanbaarvoorbekenden</t>
   </si>
   <si>
-    <t>Praat spontaan over gebeurtenissen thuis (M)</t>
-  </si>
-  <si>
     <t>ddicmm047</t>
   </si>
   <si>
@@ -1255,9 +1243,6 @@
     <t>v1526</t>
   </si>
   <si>
-    <t>Raapt vanuit hurkzit iets op</t>
-  </si>
-  <si>
     <t>ddigmd070</t>
   </si>
   <si>
@@ -1498,9 +1483,6 @@
     <t>Benen gebogen of trappelen bij verticaal zwaaien - rl</t>
   </si>
   <si>
-    <t>Stapelt twee blokjes - rl</t>
-  </si>
-  <si>
     <t>Stapelt 3 blokjes - rl</t>
   </si>
   <si>
@@ -1526,6 +1508,27 @@
   </si>
   <si>
     <t>Makes varying sounds</t>
+  </si>
+  <si>
+    <t>Handen af en toe openen</t>
+  </si>
+  <si>
+    <t>Pakt in rugligging voorwerp binnen bereik</t>
+  </si>
+  <si>
+    <t>Stapelt 2 blokjes - rl</t>
+  </si>
+  <si>
+    <t>Maakt communicatieve gebaren (M)</t>
+  </si>
+  <si>
+    <t>Begrijpt fantasieopdrachtjes (M)</t>
+  </si>
+  <si>
+    <t>Praat spontaan over gebeurtenissen thuis/speelzaal (M)</t>
+  </si>
+  <si>
+    <t>Kan hurken en weer gaan staan zonder steun en zonder hulp van anderen</t>
   </si>
 </sst>
 </file>
@@ -1541,12 +1544,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -1561,8 +1570,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1860,14 +1870,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K90"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="7" max="7" width="58" customWidth="1"/>
-    <col min="8" max="8" width="45.140625" customWidth="1"/>
-    <col min="10" max="10" width="55.85546875" customWidth="1"/>
+    <col min="8" max="8" width="45.109375" customWidth="1"/>
+    <col min="10" max="10" width="55.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1884,7 +1894,7 @@
         <v>4</v>
       </c>
       <c r="F1" t="s">
-        <v>472</v>
+        <v>467</v>
       </c>
       <c r="G1" t="s">
         <v>5</v>
@@ -1902,7 +1912,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -1937,7 +1947,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -1972,7 +1982,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>25</v>
       </c>
@@ -1992,33 +2002,33 @@
         <v>3</v>
       </c>
       <c r="G4" t="s">
+        <v>496</v>
+      </c>
+      <c r="H4" t="s">
+        <v>29</v>
+      </c>
+      <c r="I4" t="s">
         <v>28</v>
       </c>
-      <c r="H4" t="s">
+      <c r="J4" t="s">
+        <v>29</v>
+      </c>
+      <c r="K4" t="s">
         <v>30</v>
       </c>
-      <c r="I4" t="s">
-        <v>29</v>
-      </c>
-      <c r="J4" t="s">
-        <v>30</v>
-      </c>
-      <c r="K4" t="s">
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="B5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" t="s">
         <v>32</v>
       </c>
-      <c r="B5" t="s">
-        <v>32</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>33</v>
-      </c>
-      <c r="D5" t="s">
-        <v>34</v>
       </c>
       <c r="E5">
         <v>3</v>
@@ -2027,33 +2037,33 @@
         <v>3</v>
       </c>
       <c r="G5" t="s">
+        <v>34</v>
+      </c>
+      <c r="H5" t="s">
+        <v>36</v>
+      </c>
+      <c r="I5" t="s">
         <v>35</v>
       </c>
-      <c r="H5" t="s">
+      <c r="J5" t="s">
+        <v>36</v>
+      </c>
+      <c r="K5" t="s">
         <v>37</v>
       </c>
-      <c r="I5" t="s">
-        <v>36</v>
-      </c>
-      <c r="J5" t="s">
-        <v>37</v>
-      </c>
-      <c r="K5" t="s">
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="B6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C6" t="s">
         <v>39</v>
       </c>
-      <c r="B6" t="s">
-        <v>39</v>
-      </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>40</v>
-      </c>
-      <c r="D6" t="s">
-        <v>41</v>
       </c>
       <c r="E6">
         <v>4</v>
@@ -2062,33 +2072,33 @@
         <v>6</v>
       </c>
       <c r="G6" t="s">
+        <v>41</v>
+      </c>
+      <c r="H6" t="s">
+        <v>43</v>
+      </c>
+      <c r="I6" t="s">
         <v>42</v>
       </c>
-      <c r="H6" t="s">
+      <c r="J6" t="s">
+        <v>43</v>
+      </c>
+      <c r="K6" t="s">
         <v>44</v>
       </c>
-      <c r="I6" t="s">
-        <v>43</v>
-      </c>
-      <c r="J6" t="s">
-        <v>44</v>
-      </c>
-      <c r="K6" t="s">
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="B7" t="s">
+        <v>45</v>
+      </c>
+      <c r="C7" t="s">
         <v>46</v>
       </c>
-      <c r="B7" t="s">
-        <v>46</v>
-      </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>47</v>
-      </c>
-      <c r="D7" t="s">
-        <v>48</v>
       </c>
       <c r="E7">
         <v>4</v>
@@ -2097,22 +2107,22 @@
         <v>6</v>
       </c>
       <c r="G7" t="s">
+        <v>497</v>
+      </c>
+      <c r="H7" t="s">
         <v>49</v>
       </c>
-      <c r="H7" t="s">
-        <v>51</v>
-      </c>
       <c r="I7" t="s">
+        <v>48</v>
+      </c>
+      <c r="J7" t="s">
+        <v>49</v>
+      </c>
+      <c r="K7" t="s">
         <v>50</v>
       </c>
-      <c r="J7" t="s">
-        <v>51</v>
-      </c>
-      <c r="K7" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>18</v>
       </c>
@@ -2120,10 +2130,10 @@
         <v>18</v>
       </c>
       <c r="C8" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D8" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E8">
         <v>5</v>
@@ -2132,22 +2142,22 @@
         <v>9</v>
       </c>
       <c r="G8" t="s">
+        <v>53</v>
+      </c>
+      <c r="H8" t="s">
         <v>55</v>
       </c>
-      <c r="H8" t="s">
-        <v>57</v>
-      </c>
       <c r="I8" t="s">
+        <v>54</v>
+      </c>
+      <c r="J8" t="s">
+        <v>55</v>
+      </c>
+      <c r="K8" t="s">
         <v>56</v>
       </c>
-      <c r="J8" t="s">
-        <v>57</v>
-      </c>
-      <c r="K8" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>26</v>
       </c>
@@ -2155,10 +2165,10 @@
         <v>26</v>
       </c>
       <c r="C9" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D9" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E9">
         <v>5</v>
@@ -2167,33 +2177,33 @@
         <v>9</v>
       </c>
       <c r="G9" t="s">
+        <v>59</v>
+      </c>
+      <c r="H9" t="s">
         <v>61</v>
       </c>
-      <c r="H9" t="s">
+      <c r="I9" t="s">
+        <v>60</v>
+      </c>
+      <c r="J9" t="s">
+        <v>61</v>
+      </c>
+      <c r="K9" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" t="s">
+        <v>32</v>
+      </c>
+      <c r="C10" t="s">
         <v>63</v>
       </c>
-      <c r="I9" t="s">
-        <v>62</v>
-      </c>
-      <c r="J9" t="s">
-        <v>63</v>
-      </c>
-      <c r="K9" t="s">
+      <c r="D10" t="s">
         <v>64</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>33</v>
-      </c>
-      <c r="B10" t="s">
-        <v>33</v>
-      </c>
-      <c r="C10" t="s">
-        <v>65</v>
-      </c>
-      <c r="D10" t="s">
-        <v>66</v>
       </c>
       <c r="E10">
         <v>5</v>
@@ -2202,33 +2212,33 @@
         <v>9</v>
       </c>
       <c r="G10" t="s">
+        <v>65</v>
+      </c>
+      <c r="H10" t="s">
+        <v>66</v>
+      </c>
+      <c r="I10" t="s">
         <v>67</v>
       </c>
-      <c r="H10" t="s">
+      <c r="J10" t="s">
+        <v>66</v>
+      </c>
+      <c r="K10" t="s">
         <v>68</v>
       </c>
-      <c r="I10" t="s">
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
         <v>69</v>
       </c>
-      <c r="J10" t="s">
-        <v>68</v>
-      </c>
-      <c r="K10" t="s">
+      <c r="B11" t="s">
+        <v>69</v>
+      </c>
+      <c r="C11" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+      <c r="D11" t="s">
         <v>71</v>
-      </c>
-      <c r="B11" t="s">
-        <v>71</v>
-      </c>
-      <c r="C11" t="s">
-        <v>72</v>
-      </c>
-      <c r="D11" t="s">
-        <v>73</v>
       </c>
       <c r="E11">
         <v>6</v>
@@ -2237,33 +2247,33 @@
         <v>12</v>
       </c>
       <c r="G11" t="s">
+        <v>72</v>
+      </c>
+      <c r="H11" t="s">
+        <v>73</v>
+      </c>
+      <c r="I11" t="s">
         <v>74</v>
       </c>
-      <c r="H11" t="s">
+      <c r="J11" t="s">
         <v>75</v>
       </c>
-      <c r="I11" t="s">
+      <c r="K11" t="s">
         <v>76</v>
       </c>
-      <c r="J11" t="s">
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
         <v>77</v>
       </c>
-      <c r="K11" t="s">
+      <c r="B12" t="s">
+        <v>77</v>
+      </c>
+      <c r="C12" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+      <c r="D12" t="s">
         <v>79</v>
-      </c>
-      <c r="B12" t="s">
-        <v>79</v>
-      </c>
-      <c r="C12" t="s">
-        <v>80</v>
-      </c>
-      <c r="D12" t="s">
-        <v>81</v>
       </c>
       <c r="E12">
         <v>7</v>
@@ -2272,33 +2282,33 @@
         <v>15</v>
       </c>
       <c r="G12" t="s">
+        <v>80</v>
+      </c>
+      <c r="H12" t="s">
         <v>82</v>
       </c>
-      <c r="H12" t="s">
+      <c r="I12" t="s">
+        <v>81</v>
+      </c>
+      <c r="J12" t="s">
+        <v>82</v>
+      </c>
+      <c r="K12" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
         <v>84</v>
       </c>
-      <c r="I12" t="s">
-        <v>83</v>
-      </c>
-      <c r="J12" t="s">
+      <c r="B13" t="s">
         <v>84</v>
       </c>
-      <c r="K12" t="s">
+      <c r="C13" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+      <c r="D13" t="s">
         <v>86</v>
-      </c>
-      <c r="B13" t="s">
-        <v>86</v>
-      </c>
-      <c r="C13" t="s">
-        <v>87</v>
-      </c>
-      <c r="D13" t="s">
-        <v>88</v>
       </c>
       <c r="E13">
         <v>7</v>
@@ -2307,33 +2317,33 @@
         <v>15</v>
       </c>
       <c r="G13" t="s">
-        <v>490</v>
+        <v>485</v>
       </c>
       <c r="H13" t="s">
+        <v>87</v>
+      </c>
+      <c r="I13" t="s">
+        <v>88</v>
+      </c>
+      <c r="J13" t="s">
         <v>89</v>
       </c>
-      <c r="I13" t="s">
+      <c r="K13" t="s">
         <v>90</v>
       </c>
-      <c r="J13" t="s">
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>39</v>
+      </c>
+      <c r="B14" t="s">
+        <v>39</v>
+      </c>
+      <c r="C14" t="s">
         <v>91</v>
       </c>
-      <c r="K13" t="s">
+      <c r="D14" t="s">
         <v>92</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>40</v>
-      </c>
-      <c r="B14" t="s">
-        <v>40</v>
-      </c>
-      <c r="C14" t="s">
-        <v>93</v>
-      </c>
-      <c r="D14" t="s">
-        <v>94</v>
       </c>
       <c r="E14">
         <v>8</v>
@@ -2342,33 +2352,33 @@
         <v>18</v>
       </c>
       <c r="G14" t="s">
-        <v>492</v>
+        <v>498</v>
       </c>
       <c r="H14" t="s">
+        <v>93</v>
+      </c>
+      <c r="I14" t="s">
+        <v>94</v>
+      </c>
+      <c r="J14" t="s">
         <v>95</v>
       </c>
-      <c r="I14" t="s">
+      <c r="K14" t="s">
         <v>96</v>
       </c>
-      <c r="J14" t="s">
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>46</v>
+      </c>
+      <c r="B15" t="s">
+        <v>46</v>
+      </c>
+      <c r="C15" t="s">
         <v>97</v>
       </c>
-      <c r="K14" t="s">
+      <c r="D15" t="s">
         <v>98</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>47</v>
-      </c>
-      <c r="B15" t="s">
-        <v>47</v>
-      </c>
-      <c r="C15" t="s">
-        <v>99</v>
-      </c>
-      <c r="D15" t="s">
-        <v>100</v>
       </c>
       <c r="E15">
         <v>8</v>
@@ -2377,33 +2387,33 @@
         <v>18</v>
       </c>
       <c r="G15" t="s">
+        <v>99</v>
+      </c>
+      <c r="H15" t="s">
         <v>101</v>
       </c>
-      <c r="H15" t="s">
+      <c r="I15" t="s">
+        <v>100</v>
+      </c>
+      <c r="J15" t="s">
+        <v>101</v>
+      </c>
+      <c r="K15" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
         <v>103</v>
       </c>
-      <c r="I15" t="s">
-        <v>102</v>
-      </c>
-      <c r="J15" t="s">
+      <c r="B16" t="s">
         <v>103</v>
       </c>
-      <c r="K15" t="s">
+      <c r="C16" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+      <c r="D16" t="s">
         <v>105</v>
-      </c>
-      <c r="B16" t="s">
-        <v>105</v>
-      </c>
-      <c r="C16" t="s">
-        <v>106</v>
-      </c>
-      <c r="D16" t="s">
-        <v>107</v>
       </c>
       <c r="E16">
         <v>9</v>
@@ -2412,33 +2422,33 @@
         <v>24</v>
       </c>
       <c r="G16" t="s">
-        <v>493</v>
+        <v>487</v>
       </c>
       <c r="H16" t="s">
+        <v>106</v>
+      </c>
+      <c r="I16" t="s">
+        <v>107</v>
+      </c>
+      <c r="J16" t="s">
         <v>108</v>
       </c>
-      <c r="I16" t="s">
+      <c r="K16" t="s">
         <v>109</v>
       </c>
-      <c r="J16" t="s">
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
         <v>110</v>
       </c>
-      <c r="K16" t="s">
+      <c r="B17" t="s">
+        <v>110</v>
+      </c>
+      <c r="C17" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+      <c r="D17" t="s">
         <v>112</v>
-      </c>
-      <c r="B17" t="s">
-        <v>112</v>
-      </c>
-      <c r="C17" t="s">
-        <v>113</v>
-      </c>
-      <c r="D17" t="s">
-        <v>114</v>
       </c>
       <c r="E17">
         <v>9</v>
@@ -2447,30 +2457,30 @@
         <v>24</v>
       </c>
       <c r="G17" t="s">
+        <v>113</v>
+      </c>
+      <c r="H17" t="s">
+        <v>114</v>
+      </c>
+      <c r="I17" t="s">
         <v>115</v>
       </c>
-      <c r="H17" t="s">
+      <c r="J17" t="s">
         <v>116</v>
       </c>
-      <c r="I17" t="s">
+      <c r="K17" t="s">
         <v>117</v>
       </c>
-      <c r="J17" t="s">
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
         <v>118</v>
       </c>
-      <c r="K17" t="s">
+      <c r="B18" t="s">
+        <v>118</v>
+      </c>
+      <c r="D18" t="s">
         <v>119</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>120</v>
-      </c>
-      <c r="B18" t="s">
-        <v>120</v>
-      </c>
-      <c r="D18" t="s">
-        <v>121</v>
       </c>
       <c r="E18">
         <v>10</v>
@@ -2479,30 +2489,30 @@
         <v>30</v>
       </c>
       <c r="G18" t="s">
+        <v>120</v>
+      </c>
+      <c r="H18" t="s">
+        <v>121</v>
+      </c>
+      <c r="I18" t="s">
         <v>122</v>
       </c>
-      <c r="H18" t="s">
+      <c r="J18" t="s">
         <v>123</v>
       </c>
-      <c r="I18" t="s">
+      <c r="K18" t="s">
         <v>124</v>
       </c>
-      <c r="J18" t="s">
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
         <v>125</v>
       </c>
-      <c r="K18" t="s">
+      <c r="B19" t="s">
+        <v>125</v>
+      </c>
+      <c r="D19" t="s">
         <v>126</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>127</v>
-      </c>
-      <c r="B19" t="s">
-        <v>127</v>
-      </c>
-      <c r="D19" t="s">
-        <v>128</v>
       </c>
       <c r="E19">
         <v>10</v>
@@ -2511,30 +2521,30 @@
         <v>30</v>
       </c>
       <c r="G19" t="s">
+        <v>127</v>
+      </c>
+      <c r="H19" t="s">
         <v>129</v>
       </c>
-      <c r="H19" t="s">
+      <c r="I19" t="s">
+        <v>128</v>
+      </c>
+      <c r="J19" t="s">
+        <v>129</v>
+      </c>
+      <c r="K19" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>51</v>
+      </c>
+      <c r="B20" t="s">
+        <v>51</v>
+      </c>
+      <c r="D20" t="s">
         <v>131</v>
-      </c>
-      <c r="I19" t="s">
-        <v>130</v>
-      </c>
-      <c r="J19" t="s">
-        <v>131</v>
-      </c>
-      <c r="K19" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>53</v>
-      </c>
-      <c r="B20" t="s">
-        <v>53</v>
-      </c>
-      <c r="D20" t="s">
-        <v>133</v>
       </c>
       <c r="E20">
         <v>10</v>
@@ -2543,27 +2553,27 @@
         <v>30</v>
       </c>
       <c r="G20" t="s">
+        <v>132</v>
+      </c>
+      <c r="H20" t="s">
+        <v>133</v>
+      </c>
+      <c r="I20" t="s">
         <v>134</v>
       </c>
-      <c r="H20" t="s">
+      <c r="J20" t="s">
         <v>135</v>
       </c>
-      <c r="I20" t="s">
+      <c r="K20" t="s">
         <v>136</v>
       </c>
-      <c r="J20" t="s">
-        <v>137</v>
-      </c>
-      <c r="K20" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B21" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E21">
         <v>11</v>
@@ -2572,27 +2582,27 @@
         <v>36</v>
       </c>
       <c r="G21" t="s">
+        <v>137</v>
+      </c>
+      <c r="H21" t="s">
+        <v>140</v>
+      </c>
+      <c r="I21" t="s">
         <v>139</v>
       </c>
-      <c r="H21" t="s">
-        <v>142</v>
-      </c>
-      <c r="I21" t="s">
+      <c r="J21" t="s">
+        <v>140</v>
+      </c>
+      <c r="K21" t="s">
         <v>141</v>
       </c>
-      <c r="J21" t="s">
-        <v>142</v>
-      </c>
-      <c r="K21" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B22" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E22">
         <v>11</v>
@@ -2601,27 +2611,27 @@
         <v>36</v>
       </c>
       <c r="G22" t="s">
+        <v>142</v>
+      </c>
+      <c r="H22" t="s">
         <v>144</v>
       </c>
-      <c r="H22" t="s">
+      <c r="I22" t="s">
+        <v>143</v>
+      </c>
+      <c r="J22" t="s">
+        <v>144</v>
+      </c>
+      <c r="K22" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
         <v>146</v>
       </c>
-      <c r="I22" t="s">
-        <v>145</v>
-      </c>
-      <c r="J22" t="s">
+      <c r="B23" t="s">
         <v>146</v>
-      </c>
-      <c r="K22" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>148</v>
-      </c>
-      <c r="B23" t="s">
-        <v>148</v>
       </c>
       <c r="E23">
         <v>11</v>
@@ -2630,27 +2640,27 @@
         <v>36</v>
       </c>
       <c r="G23" t="s">
+        <v>147</v>
+      </c>
+      <c r="H23" t="s">
         <v>149</v>
       </c>
-      <c r="H23" t="s">
+      <c r="I23" t="s">
+        <v>148</v>
+      </c>
+      <c r="J23" t="s">
+        <v>149</v>
+      </c>
+      <c r="K23" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
         <v>151</v>
       </c>
-      <c r="I23" t="s">
-        <v>150</v>
-      </c>
-      <c r="J23" t="s">
+      <c r="B24" t="s">
         <v>151</v>
-      </c>
-      <c r="K23" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>153</v>
-      </c>
-      <c r="B24" t="s">
-        <v>153</v>
       </c>
       <c r="E24">
         <v>12</v>
@@ -2659,27 +2669,27 @@
         <v>42</v>
       </c>
       <c r="G24" t="s">
+        <v>152</v>
+      </c>
+      <c r="H24" t="s">
         <v>154</v>
       </c>
-      <c r="H24" t="s">
+      <c r="I24" t="s">
+        <v>153</v>
+      </c>
+      <c r="J24" t="s">
+        <v>154</v>
+      </c>
+      <c r="K24" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
         <v>156</v>
       </c>
-      <c r="I24" t="s">
-        <v>155</v>
-      </c>
-      <c r="J24" t="s">
+      <c r="B25" t="s">
         <v>156</v>
-      </c>
-      <c r="K24" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>158</v>
-      </c>
-      <c r="B25" t="s">
-        <v>158</v>
       </c>
       <c r="E25">
         <v>12</v>
@@ -2688,27 +2698,27 @@
         <v>42</v>
       </c>
       <c r="G25" t="s">
+        <v>157</v>
+      </c>
+      <c r="H25" t="s">
         <v>159</v>
       </c>
-      <c r="H25" t="s">
+      <c r="I25" t="s">
+        <v>158</v>
+      </c>
+      <c r="J25" t="s">
+        <v>159</v>
+      </c>
+      <c r="K25" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
         <v>161</v>
       </c>
-      <c r="I25" t="s">
-        <v>160</v>
-      </c>
-      <c r="J25" t="s">
+      <c r="B26" t="s">
         <v>161</v>
-      </c>
-      <c r="K25" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>163</v>
-      </c>
-      <c r="B26" t="s">
-        <v>163</v>
       </c>
       <c r="E26">
         <v>12</v>
@@ -2717,27 +2727,27 @@
         <v>42</v>
       </c>
       <c r="G26" t="s">
+        <v>162</v>
+      </c>
+      <c r="H26" t="s">
         <v>164</v>
       </c>
-      <c r="H26" t="s">
+      <c r="I26" t="s">
+        <v>163</v>
+      </c>
+      <c r="J26" t="s">
+        <v>164</v>
+      </c>
+      <c r="K26" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
         <v>166</v>
       </c>
-      <c r="I26" t="s">
-        <v>165</v>
-      </c>
-      <c r="J26" t="s">
-        <v>166</v>
-      </c>
-      <c r="K26" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>168</v>
-      </c>
       <c r="B27" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="E27">
         <v>13</v>
@@ -2746,27 +2756,27 @@
         <v>48</v>
       </c>
       <c r="G27" t="s">
+        <v>167</v>
+      </c>
+      <c r="H27" t="s">
         <v>169</v>
       </c>
-      <c r="H27" t="s">
-        <v>171</v>
-      </c>
       <c r="I27" t="s">
+        <v>168</v>
+      </c>
+      <c r="J27" t="s">
+        <v>169</v>
+      </c>
+      <c r="K27" t="s">
         <v>170</v>
       </c>
-      <c r="J27" t="s">
-        <v>171</v>
-      </c>
-      <c r="K27" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B28" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="E28">
         <v>13</v>
@@ -2775,33 +2785,33 @@
         <v>48</v>
       </c>
       <c r="G28" t="s">
+        <v>171</v>
+      </c>
+      <c r="H28" t="s">
         <v>173</v>
       </c>
-      <c r="H28" t="s">
+      <c r="I28" t="s">
+        <v>172</v>
+      </c>
+      <c r="J28" t="s">
+        <v>173</v>
+      </c>
+      <c r="K28" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
         <v>175</v>
       </c>
-      <c r="I28" t="s">
-        <v>174</v>
-      </c>
-      <c r="J28" t="s">
-        <v>175</v>
-      </c>
-      <c r="K28" t="s">
+      <c r="B29" t="s">
         <v>176</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>177</v>
-      </c>
-      <c r="B29" t="s">
-        <v>178</v>
       </c>
       <c r="C29" t="s">
         <v>17</v>
       </c>
       <c r="D29" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E29">
         <v>1</v>
@@ -2810,33 +2820,33 @@
         <v>1</v>
       </c>
       <c r="G29" t="s">
+        <v>178</v>
+      </c>
+      <c r="H29" t="s">
         <v>180</v>
       </c>
-      <c r="H29" t="s">
+      <c r="I29" t="s">
+        <v>179</v>
+      </c>
+      <c r="J29" t="s">
+        <v>180</v>
+      </c>
+      <c r="K29" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>176</v>
+      </c>
+      <c r="B30" t="s">
         <v>182</v>
       </c>
-      <c r="I29" t="s">
-        <v>181</v>
-      </c>
-      <c r="J29" t="s">
-        <v>182</v>
-      </c>
-      <c r="K29" t="s">
+      <c r="C30" t="s">
+        <v>45</v>
+      </c>
+      <c r="D30" t="s">
         <v>183</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>178</v>
-      </c>
-      <c r="B30" t="s">
-        <v>184</v>
-      </c>
-      <c r="C30" t="s">
-        <v>46</v>
-      </c>
-      <c r="D30" t="s">
-        <v>185</v>
       </c>
       <c r="E30">
         <v>2</v>
@@ -2845,33 +2855,33 @@
         <v>2</v>
       </c>
       <c r="G30" t="s">
+        <v>184</v>
+      </c>
+      <c r="H30" t="s">
         <v>186</v>
       </c>
-      <c r="H30" t="s">
+      <c r="I30" t="s">
+        <v>185</v>
+      </c>
+      <c r="J30" t="s">
+        <v>186</v>
+      </c>
+      <c r="K30" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>182</v>
+      </c>
+      <c r="B31" t="s">
         <v>188</v>
       </c>
-      <c r="I30" t="s">
-        <v>187</v>
-      </c>
-      <c r="J30" t="s">
-        <v>188</v>
-      </c>
-      <c r="K30" t="s">
+      <c r="C31" t="s">
+        <v>69</v>
+      </c>
+      <c r="D31" t="s">
         <v>189</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>184</v>
-      </c>
-      <c r="B31" t="s">
-        <v>190</v>
-      </c>
-      <c r="C31" t="s">
-        <v>71</v>
-      </c>
-      <c r="D31" t="s">
-        <v>191</v>
       </c>
       <c r="E31">
         <v>3</v>
@@ -2880,33 +2890,33 @@
         <v>3</v>
       </c>
       <c r="G31" t="s">
+        <v>190</v>
+      </c>
+      <c r="H31" t="s">
+        <v>191</v>
+      </c>
+      <c r="I31" t="s">
         <v>192</v>
       </c>
-      <c r="H31" t="s">
+      <c r="J31" t="s">
         <v>193</v>
       </c>
-      <c r="I31" t="s">
+      <c r="K31" t="s">
         <v>194</v>
       </c>
-      <c r="J31" t="s">
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>188</v>
+      </c>
+      <c r="B32" t="s">
+        <v>78</v>
+      </c>
+      <c r="C32" t="s">
         <v>195</v>
       </c>
-      <c r="K31" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>190</v>
-      </c>
-      <c r="B32" t="s">
-        <v>80</v>
-      </c>
-      <c r="C32" t="s">
-        <v>197</v>
-      </c>
       <c r="D32" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="E32">
         <v>4</v>
@@ -2915,27 +2925,27 @@
         <v>6</v>
       </c>
       <c r="G32" t="s">
+        <v>196</v>
+      </c>
+      <c r="H32" t="s">
+        <v>495</v>
+      </c>
+      <c r="I32" t="s">
+        <v>197</v>
+      </c>
+      <c r="K32" t="s">
         <v>198</v>
       </c>
-      <c r="H32" t="s">
-        <v>501</v>
-      </c>
-      <c r="I32" t="s">
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>78</v>
+      </c>
+      <c r="C33" t="s">
         <v>199</v>
       </c>
-      <c r="K32" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>80</v>
-      </c>
-      <c r="C33" t="s">
-        <v>201</v>
-      </c>
       <c r="D33" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="E33">
         <v>4</v>
@@ -2943,28 +2953,28 @@
       <c r="F33">
         <v>6</v>
       </c>
-      <c r="G33" t="s">
+      <c r="G33" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="H33" t="s">
+        <v>494</v>
+      </c>
+      <c r="K33" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>85</v>
+      </c>
+      <c r="B34" t="s">
+        <v>85</v>
+      </c>
+      <c r="C34" t="s">
+        <v>161</v>
+      </c>
+      <c r="D34" t="s">
         <v>202</v>
-      </c>
-      <c r="H33" t="s">
-        <v>500</v>
-      </c>
-      <c r="K33" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>87</v>
-      </c>
-      <c r="B34" t="s">
-        <v>87</v>
-      </c>
-      <c r="C34" t="s">
-        <v>163</v>
-      </c>
-      <c r="D34" t="s">
-        <v>204</v>
       </c>
       <c r="E34">
         <v>5</v>
@@ -2973,33 +2983,33 @@
         <v>9</v>
       </c>
       <c r="G34" t="s">
+        <v>203</v>
+      </c>
+      <c r="H34" t="s">
+        <v>204</v>
+      </c>
+      <c r="I34" t="s">
         <v>205</v>
       </c>
-      <c r="H34" t="s">
+      <c r="J34" t="s">
         <v>206</v>
       </c>
-      <c r="I34" t="s">
+      <c r="K34" t="s">
         <v>207</v>
       </c>
-      <c r="J34" t="s">
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
         <v>208</v>
       </c>
-      <c r="K34" t="s">
+      <c r="B35" t="s">
+        <v>208</v>
+      </c>
+      <c r="C35" t="s">
+        <v>188</v>
+      </c>
+      <c r="D35" t="s">
         <v>209</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>210</v>
-      </c>
-      <c r="B35" t="s">
-        <v>210</v>
-      </c>
-      <c r="C35" t="s">
-        <v>190</v>
-      </c>
-      <c r="D35" t="s">
-        <v>211</v>
       </c>
       <c r="E35">
         <v>6</v>
@@ -3008,33 +3018,33 @@
         <v>12</v>
       </c>
       <c r="G35" t="s">
+        <v>210</v>
+      </c>
+      <c r="H35" t="s">
         <v>212</v>
       </c>
-      <c r="H35" t="s">
+      <c r="I35" t="s">
+        <v>211</v>
+      </c>
+      <c r="J35" t="s">
+        <v>212</v>
+      </c>
+      <c r="K35" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
         <v>214</v>
       </c>
-      <c r="I35" t="s">
-        <v>213</v>
-      </c>
-      <c r="J35" t="s">
+      <c r="B36" t="s">
         <v>214</v>
       </c>
-      <c r="K35" t="s">
+      <c r="C36" t="s">
         <v>215</v>
       </c>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>216</v>
-      </c>
-      <c r="B36" t="s">
-        <v>216</v>
-      </c>
-      <c r="C36" t="s">
-        <v>217</v>
-      </c>
       <c r="D36" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="E36">
         <v>6</v>
@@ -3043,33 +3053,30 @@
         <v>12</v>
       </c>
       <c r="G36" t="s">
+        <v>216</v>
+      </c>
+      <c r="H36" t="s">
         <v>218</v>
       </c>
-      <c r="H36" t="s">
-        <v>220</v>
-      </c>
       <c r="I36" t="s">
+        <v>217</v>
+      </c>
+      <c r="J36" t="s">
+        <v>218</v>
+      </c>
+      <c r="K36" t="s">
         <v>219</v>
       </c>
-      <c r="J36" t="s">
-        <v>220</v>
-      </c>
-      <c r="K36" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>216</v>
-      </c>
-      <c r="B37" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="C37" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="D37" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="E37">
         <v>6</v>
@@ -3077,34 +3084,34 @@
       <c r="F37">
         <v>12</v>
       </c>
-      <c r="G37" t="s">
+      <c r="G37" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="H37" t="s">
         <v>218</v>
       </c>
-      <c r="H37" t="s">
+      <c r="I37" t="s">
+        <v>479</v>
+      </c>
+      <c r="J37" t="s">
+        <v>218</v>
+      </c>
+      <c r="K37" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
         <v>220</v>
       </c>
-      <c r="I37" t="s">
-        <v>484</v>
-      </c>
-      <c r="J37" t="s">
+      <c r="B38" t="s">
         <v>220</v>
       </c>
-      <c r="K37" t="s">
+      <c r="C38" t="s">
+        <v>182</v>
+      </c>
+      <c r="D38" t="s">
         <v>221</v>
-      </c>
-    </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>222</v>
-      </c>
-      <c r="B38" t="s">
-        <v>222</v>
-      </c>
-      <c r="C38" t="s">
-        <v>184</v>
-      </c>
-      <c r="D38" t="s">
-        <v>223</v>
       </c>
       <c r="E38">
         <v>6</v>
@@ -3113,33 +3120,33 @@
         <v>12</v>
       </c>
       <c r="G38" t="s">
+        <v>499</v>
+      </c>
+      <c r="H38" t="s">
+        <v>223</v>
+      </c>
+      <c r="I38" t="s">
+        <v>222</v>
+      </c>
+      <c r="J38" t="s">
+        <v>223</v>
+      </c>
+      <c r="K38" t="s">
         <v>224</v>
       </c>
-      <c r="H38" t="s">
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>225</v>
+      </c>
+      <c r="B39" t="s">
+        <v>225</v>
+      </c>
+      <c r="C39" t="s">
+        <v>225</v>
+      </c>
+      <c r="D39" t="s">
         <v>226</v>
-      </c>
-      <c r="I38" t="s">
-        <v>225</v>
-      </c>
-      <c r="J38" t="s">
-        <v>226</v>
-      </c>
-      <c r="K38" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>228</v>
-      </c>
-      <c r="B39" t="s">
-        <v>228</v>
-      </c>
-      <c r="C39" t="s">
-        <v>228</v>
-      </c>
-      <c r="D39" t="s">
-        <v>229</v>
       </c>
       <c r="E39">
         <v>7</v>
@@ -3148,33 +3155,33 @@
         <v>15</v>
       </c>
       <c r="G39" t="s">
+        <v>227</v>
+      </c>
+      <c r="H39" t="s">
+        <v>229</v>
+      </c>
+      <c r="I39" t="s">
+        <v>228</v>
+      </c>
+      <c r="J39" t="s">
+        <v>229</v>
+      </c>
+      <c r="K39" t="s">
         <v>230</v>
       </c>
-      <c r="H39" t="s">
-        <v>232</v>
-      </c>
-      <c r="I39" t="s">
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>91</v>
+      </c>
+      <c r="B40" t="s">
+        <v>91</v>
+      </c>
+      <c r="C40" t="s">
         <v>231</v>
       </c>
-      <c r="J39" t="s">
-        <v>232</v>
-      </c>
-      <c r="K39" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>93</v>
-      </c>
-      <c r="B40" t="s">
-        <v>93</v>
-      </c>
-      <c r="C40" t="s">
-        <v>234</v>
-      </c>
       <c r="D40" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="E40">
         <v>7</v>
@@ -3183,30 +3190,30 @@
         <v>15</v>
       </c>
       <c r="G40" t="s">
+        <v>232</v>
+      </c>
+      <c r="H40" t="s">
+        <v>493</v>
+      </c>
+      <c r="I40" t="s">
+        <v>233</v>
+      </c>
+      <c r="K40" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>97</v>
+      </c>
+      <c r="B41" t="s">
+        <v>97</v>
+      </c>
+      <c r="C41" t="s">
         <v>235</v>
       </c>
-      <c r="H40" t="s">
-        <v>499</v>
-      </c>
-      <c r="I40" t="s">
+      <c r="D41" t="s">
         <v>236</v>
-      </c>
-      <c r="K40" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
-        <v>99</v>
-      </c>
-      <c r="B41" t="s">
-        <v>99</v>
-      </c>
-      <c r="C41" t="s">
-        <v>238</v>
-      </c>
-      <c r="D41" t="s">
-        <v>239</v>
       </c>
       <c r="E41">
         <v>8</v>
@@ -3215,33 +3222,33 @@
         <v>18</v>
       </c>
       <c r="G41" t="s">
-        <v>487</v>
+        <v>482</v>
       </c>
       <c r="H41" t="s">
+        <v>237</v>
+      </c>
+      <c r="I41" t="s">
+        <v>238</v>
+      </c>
+      <c r="J41" t="s">
+        <v>239</v>
+      </c>
+      <c r="K41" t="s">
         <v>240</v>
       </c>
-      <c r="I41" t="s">
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>235</v>
+      </c>
+      <c r="B42" t="s">
+        <v>235</v>
+      </c>
+      <c r="C42" t="s">
         <v>241</v>
       </c>
-      <c r="J41" t="s">
-        <v>242</v>
-      </c>
-      <c r="K41" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
-        <v>238</v>
-      </c>
-      <c r="B42" t="s">
-        <v>238</v>
-      </c>
-      <c r="C42" t="s">
-        <v>244</v>
-      </c>
       <c r="D42" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="E42">
         <v>8</v>
@@ -3250,33 +3257,30 @@
         <v>18</v>
       </c>
       <c r="G42" t="s">
+        <v>500</v>
+      </c>
+      <c r="H42" t="s">
+        <v>244</v>
+      </c>
+      <c r="I42" t="s">
+        <v>243</v>
+      </c>
+      <c r="J42" t="s">
+        <v>244</v>
+      </c>
+      <c r="K42" t="s">
         <v>245</v>
       </c>
-      <c r="H42" t="s">
-        <v>247</v>
-      </c>
-      <c r="I42" t="s">
-        <v>246</v>
-      </c>
-      <c r="J42" t="s">
-        <v>247</v>
-      </c>
-      <c r="K42" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>238</v>
-      </c>
-      <c r="B43" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="C43" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="D43" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="E43">
         <v>8</v>
@@ -3284,34 +3288,34 @@
       <c r="F43">
         <v>18</v>
       </c>
-      <c r="G43" t="s">
+      <c r="G43" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="H43" t="s">
+        <v>244</v>
+      </c>
+      <c r="I43" t="s">
+        <v>477</v>
+      </c>
+      <c r="J43" t="s">
+        <v>244</v>
+      </c>
+      <c r="K43" t="s">
         <v>245</v>
       </c>
-      <c r="H43" t="s">
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>246</v>
+      </c>
+      <c r="B44" t="s">
+        <v>246</v>
+      </c>
+      <c r="C44" t="s">
         <v>247</v>
       </c>
-      <c r="I43" t="s">
-        <v>482</v>
-      </c>
-      <c r="J43" t="s">
-        <v>247</v>
-      </c>
-      <c r="K43" t="s">
+      <c r="D44" t="s">
         <v>248</v>
-      </c>
-    </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
-        <v>249</v>
-      </c>
-      <c r="B44" t="s">
-        <v>249</v>
-      </c>
-      <c r="C44" t="s">
-        <v>250</v>
-      </c>
-      <c r="D44" t="s">
-        <v>251</v>
       </c>
       <c r="E44">
         <v>9</v>
@@ -3320,33 +3324,33 @@
         <v>24</v>
       </c>
       <c r="G44" t="s">
+        <v>249</v>
+      </c>
+      <c r="H44" t="s">
+        <v>251</v>
+      </c>
+      <c r="I44" t="s">
+        <v>250</v>
+      </c>
+      <c r="J44" t="s">
+        <v>251</v>
+      </c>
+      <c r="K44" t="s">
         <v>252</v>
       </c>
-      <c r="H44" t="s">
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>253</v>
+      </c>
+      <c r="B45" t="s">
+        <v>253</v>
+      </c>
+      <c r="C45" t="s">
         <v>254</v>
       </c>
-      <c r="I44" t="s">
+      <c r="D45" t="s">
         <v>253</v>
-      </c>
-      <c r="J44" t="s">
-        <v>254</v>
-      </c>
-      <c r="K44" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
-        <v>256</v>
-      </c>
-      <c r="B45" t="s">
-        <v>256</v>
-      </c>
-      <c r="C45" t="s">
-        <v>257</v>
-      </c>
-      <c r="D45" t="s">
-        <v>256</v>
       </c>
       <c r="E45">
         <v>9</v>
@@ -3355,30 +3359,30 @@
         <v>24</v>
       </c>
       <c r="G45" t="s">
+        <v>255</v>
+      </c>
+      <c r="H45" t="s">
+        <v>257</v>
+      </c>
+      <c r="I45" t="s">
+        <v>256</v>
+      </c>
+      <c r="J45" t="s">
+        <v>257</v>
+      </c>
+      <c r="K45" t="s">
         <v>258</v>
       </c>
-      <c r="H45" t="s">
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>259</v>
+      </c>
+      <c r="B46" t="s">
+        <v>259</v>
+      </c>
+      <c r="D46" t="s">
         <v>260</v>
-      </c>
-      <c r="I45" t="s">
-        <v>259</v>
-      </c>
-      <c r="J45" t="s">
-        <v>260</v>
-      </c>
-      <c r="K45" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
-        <v>262</v>
-      </c>
-      <c r="B46" t="s">
-        <v>262</v>
-      </c>
-      <c r="D46" t="s">
-        <v>263</v>
       </c>
       <c r="E46">
         <v>10</v>
@@ -3387,30 +3391,30 @@
         <v>30</v>
       </c>
       <c r="G46" t="s">
+        <v>261</v>
+      </c>
+      <c r="H46" t="s">
+        <v>263</v>
+      </c>
+      <c r="I46" t="s">
+        <v>262</v>
+      </c>
+      <c r="J46" t="s">
+        <v>263</v>
+      </c>
+      <c r="K46" t="s">
         <v>264</v>
       </c>
-      <c r="H46" t="s">
-        <v>266</v>
-      </c>
-      <c r="I46" t="s">
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>104</v>
+      </c>
+      <c r="B47" t="s">
+        <v>104</v>
+      </c>
+      <c r="D47" t="s">
         <v>265</v>
-      </c>
-      <c r="J46" t="s">
-        <v>266</v>
-      </c>
-      <c r="K46" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
-        <v>106</v>
-      </c>
-      <c r="B47" t="s">
-        <v>106</v>
-      </c>
-      <c r="D47" t="s">
-        <v>268</v>
       </c>
       <c r="E47">
         <v>10</v>
@@ -3419,27 +3423,27 @@
         <v>30</v>
       </c>
       <c r="G47" t="s">
+        <v>266</v>
+      </c>
+      <c r="H47" t="s">
+        <v>268</v>
+      </c>
+      <c r="I47" t="s">
+        <v>267</v>
+      </c>
+      <c r="J47" t="s">
+        <v>268</v>
+      </c>
+      <c r="K47" t="s">
         <v>269</v>
       </c>
-      <c r="H47" t="s">
-        <v>271</v>
-      </c>
-      <c r="I47" t="s">
-        <v>270</v>
-      </c>
-      <c r="J47" t="s">
-        <v>271</v>
-      </c>
-      <c r="K47" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B48" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="E48">
         <v>11</v>
@@ -3448,27 +3452,27 @@
         <v>36</v>
       </c>
       <c r="G48" t="s">
+        <v>270</v>
+      </c>
+      <c r="H48" t="s">
+        <v>272</v>
+      </c>
+      <c r="I48" t="s">
+        <v>271</v>
+      </c>
+      <c r="J48" t="s">
+        <v>272</v>
+      </c>
+      <c r="K48" t="s">
         <v>273</v>
       </c>
-      <c r="H48" t="s">
-        <v>275</v>
-      </c>
-      <c r="I48" t="s">
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
         <v>274</v>
       </c>
-      <c r="J48" t="s">
-        <v>275</v>
-      </c>
-      <c r="K48" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
-        <v>277</v>
-      </c>
       <c r="B49" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="E49">
         <v>11</v>
@@ -3477,27 +3481,27 @@
         <v>36</v>
       </c>
       <c r="G49" t="s">
+        <v>275</v>
+      </c>
+      <c r="H49" t="s">
+        <v>277</v>
+      </c>
+      <c r="I49" t="s">
+        <v>276</v>
+      </c>
+      <c r="J49" t="s">
+        <v>277</v>
+      </c>
+      <c r="K49" t="s">
         <v>278</v>
       </c>
-      <c r="H49" t="s">
-        <v>280</v>
-      </c>
-      <c r="I49" t="s">
-        <v>279</v>
-      </c>
-      <c r="J49" t="s">
-        <v>280</v>
-      </c>
-      <c r="K49" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="B50" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="E50">
         <v>12</v>
@@ -3506,27 +3510,27 @@
         <v>42</v>
       </c>
       <c r="G50" t="s">
+        <v>501</v>
+      </c>
+      <c r="H50" t="s">
+        <v>280</v>
+      </c>
+      <c r="I50" t="s">
+        <v>279</v>
+      </c>
+      <c r="J50" t="s">
+        <v>280</v>
+      </c>
+      <c r="K50" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
         <v>282</v>
       </c>
-      <c r="H50" t="s">
-        <v>284</v>
-      </c>
-      <c r="I50" t="s">
-        <v>283</v>
-      </c>
-      <c r="J50" t="s">
-        <v>284</v>
-      </c>
-      <c r="K50" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
-        <v>286</v>
-      </c>
       <c r="B51" t="s">
-        <v>286</v>
+        <v>282</v>
       </c>
       <c r="E51">
         <v>12</v>
@@ -3535,27 +3539,27 @@
         <v>42</v>
       </c>
       <c r="G51" t="s">
+        <v>283</v>
+      </c>
+      <c r="H51" t="s">
+        <v>285</v>
+      </c>
+      <c r="I51" t="s">
+        <v>284</v>
+      </c>
+      <c r="J51" t="s">
+        <v>285</v>
+      </c>
+      <c r="K51" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
         <v>287</v>
       </c>
-      <c r="H51" t="s">
-        <v>289</v>
-      </c>
-      <c r="I51" t="s">
-        <v>288</v>
-      </c>
-      <c r="J51" t="s">
-        <v>289</v>
-      </c>
-      <c r="K51" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
-        <v>291</v>
-      </c>
       <c r="B52" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="E52">
         <v>13</v>
@@ -3564,27 +3568,27 @@
         <v>48</v>
       </c>
       <c r="G52" t="s">
+        <v>288</v>
+      </c>
+      <c r="H52" t="s">
+        <v>290</v>
+      </c>
+      <c r="I52" t="s">
+        <v>289</v>
+      </c>
+      <c r="J52" t="s">
+        <v>290</v>
+      </c>
+      <c r="K52" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
         <v>292</v>
       </c>
-      <c r="H52" t="s">
-        <v>294</v>
-      </c>
-      <c r="I52" t="s">
-        <v>293</v>
-      </c>
-      <c r="J52" t="s">
-        <v>294</v>
-      </c>
-      <c r="K52" t="s">
-        <v>295</v>
-      </c>
-    </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
-        <v>296</v>
-      </c>
       <c r="B53" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
       <c r="E53">
         <v>13</v>
@@ -3593,33 +3597,33 @@
         <v>48</v>
       </c>
       <c r="G53" t="s">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="H53" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="I53" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="J53" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="K53" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B54" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="C54" t="s">
         <v>25</v>
       </c>
       <c r="D54" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="E54">
         <v>1</v>
@@ -3628,33 +3632,33 @@
         <v>1</v>
       </c>
       <c r="G54" t="s">
+        <v>298</v>
+      </c>
+      <c r="H54" t="s">
+        <v>299</v>
+      </c>
+      <c r="I54" t="s">
+        <v>300</v>
+      </c>
+      <c r="J54" t="s">
+        <v>301</v>
+      </c>
+      <c r="K54" t="s">
         <v>302</v>
       </c>
-      <c r="H54" t="s">
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>199</v>
+      </c>
+      <c r="B55" t="s">
+        <v>215</v>
+      </c>
+      <c r="C55" t="s">
+        <v>31</v>
+      </c>
+      <c r="D55" t="s">
         <v>303</v>
-      </c>
-      <c r="I54" t="s">
-        <v>304</v>
-      </c>
-      <c r="J54" t="s">
-        <v>305</v>
-      </c>
-      <c r="K54" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
-        <v>201</v>
-      </c>
-      <c r="B55" t="s">
-        <v>217</v>
-      </c>
-      <c r="C55" t="s">
-        <v>32</v>
-      </c>
-      <c r="D55" t="s">
-        <v>307</v>
       </c>
       <c r="E55">
         <v>1</v>
@@ -3663,33 +3667,33 @@
         <v>1</v>
       </c>
       <c r="G55" t="s">
+        <v>304</v>
+      </c>
+      <c r="H55" t="s">
+        <v>305</v>
+      </c>
+      <c r="I55" t="s">
+        <v>306</v>
+      </c>
+      <c r="J55" t="s">
+        <v>307</v>
+      </c>
+      <c r="K55" t="s">
         <v>308</v>
       </c>
-      <c r="H55" t="s">
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>215</v>
+      </c>
+      <c r="B56" t="s">
+        <v>231</v>
+      </c>
+      <c r="C56" t="s">
+        <v>77</v>
+      </c>
+      <c r="D56" t="s">
         <v>309</v>
-      </c>
-      <c r="I55" t="s">
-        <v>310</v>
-      </c>
-      <c r="J55" t="s">
-        <v>311</v>
-      </c>
-      <c r="K55" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A56" t="s">
-        <v>217</v>
-      </c>
-      <c r="B56" t="s">
-        <v>234</v>
-      </c>
-      <c r="C56" t="s">
-        <v>79</v>
-      </c>
-      <c r="D56" t="s">
-        <v>313</v>
       </c>
       <c r="E56">
         <v>3</v>
@@ -3698,33 +3702,33 @@
         <v>3</v>
       </c>
       <c r="G56" t="s">
+        <v>310</v>
+      </c>
+      <c r="H56" t="s">
+        <v>312</v>
+      </c>
+      <c r="I56" t="s">
+        <v>311</v>
+      </c>
+      <c r="J56" t="s">
+        <v>312</v>
+      </c>
+      <c r="K56" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
+        <v>231</v>
+      </c>
+      <c r="B57" t="s">
+        <v>241</v>
+      </c>
+      <c r="C57" t="s">
+        <v>103</v>
+      </c>
+      <c r="D57" t="s">
         <v>314</v>
-      </c>
-      <c r="H56" t="s">
-        <v>316</v>
-      </c>
-      <c r="I56" t="s">
-        <v>315</v>
-      </c>
-      <c r="J56" t="s">
-        <v>316</v>
-      </c>
-      <c r="K56" t="s">
-        <v>317</v>
-      </c>
-    </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A57" t="s">
-        <v>234</v>
-      </c>
-      <c r="B57" t="s">
-        <v>244</v>
-      </c>
-      <c r="C57" t="s">
-        <v>105</v>
-      </c>
-      <c r="D57" t="s">
-        <v>318</v>
       </c>
       <c r="E57">
         <v>4</v>
@@ -3733,33 +3737,33 @@
         <v>6</v>
       </c>
       <c r="G57" t="s">
-        <v>471</v>
+        <v>466</v>
       </c>
       <c r="H57" t="s">
+        <v>315</v>
+      </c>
+      <c r="I57" t="s">
+        <v>316</v>
+      </c>
+      <c r="J57" t="s">
+        <v>317</v>
+      </c>
+      <c r="K57" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>241</v>
+      </c>
+      <c r="B58" t="s">
+        <v>254</v>
+      </c>
+      <c r="C58" t="s">
+        <v>38</v>
+      </c>
+      <c r="D58" t="s">
         <v>319</v>
-      </c>
-      <c r="I57" t="s">
-        <v>320</v>
-      </c>
-      <c r="J57" t="s">
-        <v>321</v>
-      </c>
-      <c r="K57" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
-        <v>244</v>
-      </c>
-      <c r="B58" t="s">
-        <v>257</v>
-      </c>
-      <c r="C58" t="s">
-        <v>39</v>
-      </c>
-      <c r="D58" t="s">
-        <v>323</v>
       </c>
       <c r="E58">
         <v>1</v>
@@ -3768,33 +3772,33 @@
         <v>1</v>
       </c>
       <c r="G58" t="s">
+        <v>320</v>
+      </c>
+      <c r="H58" t="s">
+        <v>322</v>
+      </c>
+      <c r="I58" t="s">
+        <v>321</v>
+      </c>
+      <c r="J58" t="s">
+        <v>322</v>
+      </c>
+      <c r="K58" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>254</v>
+      </c>
+      <c r="B59" t="s">
         <v>324</v>
       </c>
-      <c r="H58" t="s">
-        <v>326</v>
-      </c>
-      <c r="I58" t="s">
+      <c r="C59" t="s">
+        <v>84</v>
+      </c>
+      <c r="D59" t="s">
         <v>325</v>
-      </c>
-      <c r="J58" t="s">
-        <v>326</v>
-      </c>
-      <c r="K58" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
-        <v>257</v>
-      </c>
-      <c r="B59" t="s">
-        <v>328</v>
-      </c>
-      <c r="C59" t="s">
-        <v>86</v>
-      </c>
-      <c r="D59" t="s">
-        <v>329</v>
       </c>
       <c r="E59">
         <v>3</v>
@@ -3803,33 +3807,33 @@
         <v>3</v>
       </c>
       <c r="G59" t="s">
+        <v>326</v>
+      </c>
+      <c r="H59" t="s">
+        <v>327</v>
+      </c>
+      <c r="I59" t="s">
+        <v>328</v>
+      </c>
+      <c r="J59" t="s">
+        <v>329</v>
+      </c>
+      <c r="K59" t="s">
         <v>330</v>
       </c>
-      <c r="H59" t="s">
+    </row>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
+        <v>324</v>
+      </c>
+      <c r="B60" t="s">
         <v>331</v>
       </c>
-      <c r="I59" t="s">
+      <c r="C60" t="s">
+        <v>125</v>
+      </c>
+      <c r="D60" t="s">
         <v>332</v>
-      </c>
-      <c r="J59" t="s">
-        <v>333</v>
-      </c>
-      <c r="K59" t="s">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A60" t="s">
-        <v>328</v>
-      </c>
-      <c r="B60" t="s">
-        <v>335</v>
-      </c>
-      <c r="C60" t="s">
-        <v>127</v>
-      </c>
-      <c r="D60" t="s">
-        <v>336</v>
       </c>
       <c r="E60">
         <v>4</v>
@@ -3838,33 +3842,33 @@
         <v>6</v>
       </c>
       <c r="G60" t="s">
+        <v>333</v>
+      </c>
+      <c r="H60" t="s">
+        <v>335</v>
+      </c>
+      <c r="I60" t="s">
+        <v>334</v>
+      </c>
+      <c r="J60" t="s">
+        <v>335</v>
+      </c>
+      <c r="K60" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
+        <v>331</v>
+      </c>
+      <c r="B61" t="s">
         <v>337</v>
       </c>
-      <c r="H60" t="s">
-        <v>339</v>
-      </c>
-      <c r="I60" t="s">
+      <c r="C61" t="s">
+        <v>118</v>
+      </c>
+      <c r="D61" t="s">
         <v>338</v>
-      </c>
-      <c r="J60" t="s">
-        <v>339</v>
-      </c>
-      <c r="K60" t="s">
-        <v>340</v>
-      </c>
-    </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
-        <v>335</v>
-      </c>
-      <c r="B61" t="s">
-        <v>341</v>
-      </c>
-      <c r="C61" t="s">
-        <v>120</v>
-      </c>
-      <c r="D61" t="s">
-        <v>342</v>
       </c>
       <c r="E61">
         <v>4</v>
@@ -3873,33 +3877,33 @@
         <v>6</v>
       </c>
       <c r="G61" t="s">
-        <v>491</v>
+        <v>486</v>
       </c>
       <c r="H61" t="s">
-        <v>344</v>
+        <v>340</v>
       </c>
       <c r="I61" t="s">
+        <v>339</v>
+      </c>
+      <c r="J61" t="s">
+        <v>340</v>
+      </c>
+      <c r="K61" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A62" t="s">
+        <v>337</v>
+      </c>
+      <c r="B62" t="s">
+        <v>342</v>
+      </c>
+      <c r="C62" t="s">
+        <v>146</v>
+      </c>
+      <c r="D62" t="s">
         <v>343</v>
-      </c>
-      <c r="J61" t="s">
-        <v>344</v>
-      </c>
-      <c r="K61" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
-        <v>341</v>
-      </c>
-      <c r="B62" t="s">
-        <v>346</v>
-      </c>
-      <c r="C62" t="s">
-        <v>148</v>
-      </c>
-      <c r="D62" t="s">
-        <v>347</v>
       </c>
       <c r="E62">
         <v>5</v>
@@ -3908,33 +3912,33 @@
         <v>9</v>
       </c>
       <c r="G62" t="s">
+        <v>344</v>
+      </c>
+      <c r="H62" t="s">
+        <v>490</v>
+      </c>
+      <c r="I62" t="s">
+        <v>345</v>
+      </c>
+      <c r="J62" t="s">
+        <v>346</v>
+      </c>
+      <c r="K62" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A63" t="s">
+        <v>342</v>
+      </c>
+      <c r="B63" t="s">
         <v>348</v>
       </c>
-      <c r="H62" t="s">
-        <v>496</v>
-      </c>
-      <c r="I62" t="s">
+      <c r="C63" t="s">
+        <v>151</v>
+      </c>
+      <c r="D63" t="s">
         <v>349</v>
-      </c>
-      <c r="J62" t="s">
-        <v>350</v>
-      </c>
-      <c r="K62" t="s">
-        <v>351</v>
-      </c>
-    </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
-        <v>346</v>
-      </c>
-      <c r="B63" t="s">
-        <v>352</v>
-      </c>
-      <c r="C63" t="s">
-        <v>153</v>
-      </c>
-      <c r="D63" t="s">
-        <v>353</v>
       </c>
       <c r="E63">
         <v>5</v>
@@ -3943,33 +3947,33 @@
         <v>9</v>
       </c>
       <c r="G63" t="s">
+        <v>350</v>
+      </c>
+      <c r="H63" t="s">
+        <v>352</v>
+      </c>
+      <c r="I63" t="s">
+        <v>351</v>
+      </c>
+      <c r="J63" t="s">
+        <v>352</v>
+      </c>
+      <c r="K63" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A64" t="s">
+        <v>348</v>
+      </c>
+      <c r="B64" t="s">
         <v>354</v>
       </c>
-      <c r="H63" t="s">
-        <v>356</v>
-      </c>
-      <c r="I63" t="s">
+      <c r="C64" t="s">
+        <v>156</v>
+      </c>
+      <c r="D64" t="s">
         <v>355</v>
-      </c>
-      <c r="J63" t="s">
-        <v>356</v>
-      </c>
-      <c r="K63" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A64" t="s">
-        <v>352</v>
-      </c>
-      <c r="B64" t="s">
-        <v>358</v>
-      </c>
-      <c r="C64" t="s">
-        <v>158</v>
-      </c>
-      <c r="D64" t="s">
-        <v>359</v>
       </c>
       <c r="E64">
         <v>5</v>
@@ -3978,33 +3982,33 @@
         <v>9</v>
       </c>
       <c r="G64" t="s">
+        <v>356</v>
+      </c>
+      <c r="H64" t="s">
+        <v>358</v>
+      </c>
+      <c r="I64" t="s">
+        <v>357</v>
+      </c>
+      <c r="J64" t="s">
+        <v>358</v>
+      </c>
+      <c r="K64" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A65" t="s">
+        <v>354</v>
+      </c>
+      <c r="B65" t="s">
         <v>360</v>
       </c>
-      <c r="H64" t="s">
-        <v>362</v>
-      </c>
-      <c r="I64" t="s">
+      <c r="C65" t="s">
+        <v>166</v>
+      </c>
+      <c r="D65" t="s">
         <v>361</v>
-      </c>
-      <c r="J64" t="s">
-        <v>362</v>
-      </c>
-      <c r="K64" t="s">
-        <v>363</v>
-      </c>
-    </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A65" t="s">
-        <v>358</v>
-      </c>
-      <c r="B65" t="s">
-        <v>364</v>
-      </c>
-      <c r="C65" t="s">
-        <v>168</v>
-      </c>
-      <c r="D65" t="s">
-        <v>365</v>
       </c>
       <c r="E65">
         <v>6</v>
@@ -4013,33 +4017,33 @@
         <v>12</v>
       </c>
       <c r="G65" t="s">
+        <v>362</v>
+      </c>
+      <c r="H65" t="s">
+        <v>364</v>
+      </c>
+      <c r="I65" t="s">
+        <v>363</v>
+      </c>
+      <c r="J65" t="s">
+        <v>364</v>
+      </c>
+      <c r="K65" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A66" t="s">
+        <v>360</v>
+      </c>
+      <c r="B66" t="s">
         <v>366</v>
       </c>
-      <c r="H65" t="s">
-        <v>368</v>
-      </c>
-      <c r="I65" t="s">
+      <c r="C66" t="s">
+        <v>175</v>
+      </c>
+      <c r="D66" t="s">
         <v>367</v>
-      </c>
-      <c r="J65" t="s">
-        <v>368</v>
-      </c>
-      <c r="K65" t="s">
-        <v>369</v>
-      </c>
-    </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A66" t="s">
-        <v>364</v>
-      </c>
-      <c r="B66" t="s">
-        <v>370</v>
-      </c>
-      <c r="C66" t="s">
-        <v>177</v>
-      </c>
-      <c r="D66" t="s">
-        <v>371</v>
       </c>
       <c r="E66">
         <v>6</v>
@@ -4048,33 +4052,33 @@
         <v>12</v>
       </c>
       <c r="G66" t="s">
+        <v>368</v>
+      </c>
+      <c r="H66" t="s">
+        <v>370</v>
+      </c>
+      <c r="I66" t="s">
+        <v>369</v>
+      </c>
+      <c r="J66" t="s">
+        <v>370</v>
+      </c>
+      <c r="K66" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A67" t="s">
+        <v>366</v>
+      </c>
+      <c r="B67" t="s">
         <v>372</v>
       </c>
-      <c r="H66" t="s">
-        <v>374</v>
-      </c>
-      <c r="I66" t="s">
+      <c r="C67" t="s">
+        <v>176</v>
+      </c>
+      <c r="D67" t="s">
         <v>373</v>
-      </c>
-      <c r="J66" t="s">
-        <v>374</v>
-      </c>
-      <c r="K66" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A67" t="s">
-        <v>370</v>
-      </c>
-      <c r="B67" t="s">
-        <v>376</v>
-      </c>
-      <c r="C67" t="s">
-        <v>178</v>
-      </c>
-      <c r="D67" t="s">
-        <v>377</v>
       </c>
       <c r="E67">
         <v>6</v>
@@ -4083,33 +4087,33 @@
         <v>12</v>
       </c>
       <c r="G67" t="s">
+        <v>374</v>
+      </c>
+      <c r="H67" t="s">
+        <v>375</v>
+      </c>
+      <c r="I67" t="s">
+        <v>376</v>
+      </c>
+      <c r="J67" t="s">
+        <v>377</v>
+      </c>
+      <c r="K67" t="s">
         <v>378</v>
       </c>
-      <c r="H67" t="s">
+    </row>
+    <row r="68" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A68" t="s">
+        <v>372</v>
+      </c>
+      <c r="B68" t="s">
         <v>379</v>
       </c>
-      <c r="I67" t="s">
+      <c r="C68" t="s">
+        <v>208</v>
+      </c>
+      <c r="D68" t="s">
         <v>380</v>
-      </c>
-      <c r="J67" t="s">
-        <v>381</v>
-      </c>
-      <c r="K67" t="s">
-        <v>382</v>
-      </c>
-    </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A68" t="s">
-        <v>376</v>
-      </c>
-      <c r="B68" t="s">
-        <v>383</v>
-      </c>
-      <c r="C68" t="s">
-        <v>210</v>
-      </c>
-      <c r="D68" t="s">
-        <v>384</v>
       </c>
       <c r="E68">
         <v>7</v>
@@ -4118,33 +4122,33 @@
         <v>15</v>
       </c>
       <c r="G68" t="s">
+        <v>381</v>
+      </c>
+      <c r="H68" t="s">
+        <v>383</v>
+      </c>
+      <c r="I68" t="s">
+        <v>382</v>
+      </c>
+      <c r="J68" t="s">
+        <v>383</v>
+      </c>
+      <c r="K68" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A69" t="s">
+        <v>379</v>
+      </c>
+      <c r="B69" t="s">
         <v>385</v>
       </c>
-      <c r="H68" t="s">
-        <v>387</v>
-      </c>
-      <c r="I68" t="s">
+      <c r="C69" t="s">
+        <v>214</v>
+      </c>
+      <c r="D69" t="s">
         <v>386</v>
-      </c>
-      <c r="J68" t="s">
-        <v>387</v>
-      </c>
-      <c r="K68" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A69" t="s">
-        <v>383</v>
-      </c>
-      <c r="B69" t="s">
-        <v>389</v>
-      </c>
-      <c r="C69" t="s">
-        <v>216</v>
-      </c>
-      <c r="D69" t="s">
-        <v>390</v>
       </c>
       <c r="E69">
         <v>7</v>
@@ -4153,33 +4157,33 @@
         <v>15</v>
       </c>
       <c r="G69" t="s">
+        <v>387</v>
+      </c>
+      <c r="H69" t="s">
+        <v>388</v>
+      </c>
+      <c r="I69" t="s">
+        <v>389</v>
+      </c>
+      <c r="J69" t="s">
+        <v>390</v>
+      </c>
+      <c r="K69" t="s">
         <v>391</v>
       </c>
-      <c r="H69" t="s">
+    </row>
+    <row r="70" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A70" t="s">
+        <v>385</v>
+      </c>
+      <c r="B70" t="s">
         <v>392</v>
       </c>
-      <c r="I69" t="s">
+      <c r="C70" t="s">
+        <v>253</v>
+      </c>
+      <c r="D70" t="s">
         <v>393</v>
-      </c>
-      <c r="J69" t="s">
-        <v>394</v>
-      </c>
-      <c r="K69" t="s">
-        <v>395</v>
-      </c>
-    </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A70" t="s">
-        <v>389</v>
-      </c>
-      <c r="B70" t="s">
-        <v>396</v>
-      </c>
-      <c r="C70" t="s">
-        <v>256</v>
-      </c>
-      <c r="D70" t="s">
-        <v>397</v>
       </c>
       <c r="E70">
         <v>8</v>
@@ -4188,33 +4192,33 @@
         <v>18</v>
       </c>
       <c r="G70" t="s">
+        <v>394</v>
+      </c>
+      <c r="H70" t="s">
+        <v>396</v>
+      </c>
+      <c r="I70" t="s">
+        <v>395</v>
+      </c>
+      <c r="J70" t="s">
+        <v>396</v>
+      </c>
+      <c r="K70" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A71" t="s">
         <v>398</v>
       </c>
-      <c r="H70" t="s">
+      <c r="B71" t="s">
+        <v>399</v>
+      </c>
+      <c r="C71" t="s">
+        <v>259</v>
+      </c>
+      <c r="D71" t="s">
         <v>400</v>
-      </c>
-      <c r="I70" t="s">
-        <v>399</v>
-      </c>
-      <c r="J70" t="s">
-        <v>400</v>
-      </c>
-      <c r="K70" t="s">
-        <v>401</v>
-      </c>
-    </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A71" t="s">
-        <v>402</v>
-      </c>
-      <c r="B71" t="s">
-        <v>403</v>
-      </c>
-      <c r="C71" t="s">
-        <v>262</v>
-      </c>
-      <c r="D71" t="s">
-        <v>404</v>
       </c>
       <c r="E71">
         <v>8</v>
@@ -4223,33 +4227,33 @@
         <v>18</v>
       </c>
       <c r="G71" t="s">
+        <v>401</v>
+      </c>
+      <c r="H71" t="s">
+        <v>402</v>
+      </c>
+      <c r="I71" t="s">
+        <v>403</v>
+      </c>
+      <c r="J71" t="s">
+        <v>402</v>
+      </c>
+      <c r="K71" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="72" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A72" t="s">
+        <v>399</v>
+      </c>
+      <c r="B72" t="s">
         <v>405</v>
       </c>
-      <c r="H71" t="s">
+      <c r="C72" t="s">
+        <v>287</v>
+      </c>
+      <c r="D72" t="s">
         <v>406</v>
-      </c>
-      <c r="I71" t="s">
-        <v>407</v>
-      </c>
-      <c r="J71" t="s">
-        <v>406</v>
-      </c>
-      <c r="K71" t="s">
-        <v>408</v>
-      </c>
-    </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A72" t="s">
-        <v>403</v>
-      </c>
-      <c r="B72" t="s">
-        <v>409</v>
-      </c>
-      <c r="C72" t="s">
-        <v>291</v>
-      </c>
-      <c r="D72" t="s">
-        <v>410</v>
       </c>
       <c r="E72">
         <v>9</v>
@@ -4258,33 +4262,33 @@
         <v>24</v>
       </c>
       <c r="G72" t="s">
+        <v>502</v>
+      </c>
+      <c r="H72" t="s">
+        <v>408</v>
+      </c>
+      <c r="I72" t="s">
+        <v>407</v>
+      </c>
+      <c r="J72" t="s">
+        <v>408</v>
+      </c>
+      <c r="K72" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="73" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A73" t="s">
+        <v>405</v>
+      </c>
+      <c r="B73" t="s">
+        <v>410</v>
+      </c>
+      <c r="C73" t="s">
+        <v>292</v>
+      </c>
+      <c r="D73" t="s">
         <v>411</v>
-      </c>
-      <c r="H72" t="s">
-        <v>413</v>
-      </c>
-      <c r="I72" t="s">
-        <v>412</v>
-      </c>
-      <c r="J72" t="s">
-        <v>413</v>
-      </c>
-      <c r="K72" t="s">
-        <v>414</v>
-      </c>
-    </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A73" t="s">
-        <v>409</v>
-      </c>
-      <c r="B73" t="s">
-        <v>415</v>
-      </c>
-      <c r="C73" t="s">
-        <v>296</v>
-      </c>
-      <c r="D73" t="s">
-        <v>416</v>
       </c>
       <c r="E73">
         <v>9</v>
@@ -4293,30 +4297,30 @@
         <v>24</v>
       </c>
       <c r="G73" t="s">
+        <v>412</v>
+      </c>
+      <c r="H73" t="s">
+        <v>413</v>
+      </c>
+      <c r="I73" t="s">
+        <v>414</v>
+      </c>
+      <c r="J73" t="s">
+        <v>413</v>
+      </c>
+      <c r="K73" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="74" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A74" t="s">
+        <v>416</v>
+      </c>
+      <c r="B74" t="s">
+        <v>416</v>
+      </c>
+      <c r="D74" t="s">
         <v>417</v>
-      </c>
-      <c r="H73" t="s">
-        <v>418</v>
-      </c>
-      <c r="I73" t="s">
-        <v>419</v>
-      </c>
-      <c r="J73" t="s">
-        <v>418</v>
-      </c>
-      <c r="K73" t="s">
-        <v>420</v>
-      </c>
-    </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A74" t="s">
-        <v>421</v>
-      </c>
-      <c r="B74" t="s">
-        <v>421</v>
-      </c>
-      <c r="D74" t="s">
-        <v>422</v>
       </c>
       <c r="E74">
         <v>10</v>
@@ -4325,27 +4329,27 @@
         <v>30</v>
       </c>
       <c r="G74" t="s">
-        <v>494</v>
+        <v>488</v>
       </c>
       <c r="H74" t="s">
-        <v>424</v>
+        <v>419</v>
       </c>
       <c r="I74" t="s">
-        <v>423</v>
+        <v>418</v>
       </c>
       <c r="J74" t="s">
-        <v>424</v>
+        <v>419</v>
       </c>
       <c r="K74" t="s">
-        <v>425</v>
-      </c>
-    </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.25">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="75" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
-        <v>426</v>
+        <v>421</v>
       </c>
       <c r="B75" t="s">
-        <v>426</v>
+        <v>421</v>
       </c>
       <c r="E75">
         <v>10</v>
@@ -4354,27 +4358,27 @@
         <v>30</v>
       </c>
       <c r="G75" t="s">
+        <v>422</v>
+      </c>
+      <c r="H75" t="s">
+        <v>424</v>
+      </c>
+      <c r="I75" t="s">
+        <v>423</v>
+      </c>
+      <c r="J75" t="s">
+        <v>424</v>
+      </c>
+      <c r="K75" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="76" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A76" t="s">
+        <v>426</v>
+      </c>
+      <c r="B76" t="s">
         <v>427</v>
-      </c>
-      <c r="H75" t="s">
-        <v>429</v>
-      </c>
-      <c r="I75" t="s">
-        <v>428</v>
-      </c>
-      <c r="J75" t="s">
-        <v>429</v>
-      </c>
-      <c r="K75" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A76" t="s">
-        <v>431</v>
-      </c>
-      <c r="B76" t="s">
-        <v>432</v>
       </c>
       <c r="E76">
         <v>11</v>
@@ -4383,27 +4387,27 @@
         <v>36</v>
       </c>
       <c r="G76" t="s">
-        <v>433</v>
+        <v>428</v>
       </c>
       <c r="H76" t="s">
-        <v>435</v>
+        <v>430</v>
       </c>
       <c r="I76" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
       <c r="J76" t="s">
-        <v>435</v>
+        <v>430</v>
       </c>
       <c r="K76" t="s">
-        <v>436</v>
-      </c>
-    </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.25">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="77" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
-        <v>437</v>
+        <v>432</v>
       </c>
       <c r="B77" t="s">
-        <v>431</v>
+        <v>426</v>
       </c>
       <c r="E77">
         <v>11</v>
@@ -4412,27 +4416,27 @@
         <v>36</v>
       </c>
       <c r="G77" t="s">
-        <v>438</v>
+        <v>433</v>
       </c>
       <c r="H77" t="s">
-        <v>440</v>
+        <v>435</v>
       </c>
       <c r="I77" t="s">
-        <v>439</v>
+        <v>434</v>
       </c>
       <c r="J77" t="s">
-        <v>440</v>
+        <v>435</v>
       </c>
       <c r="K77" t="s">
-        <v>441</v>
-      </c>
-    </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.25">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="78" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
-        <v>442</v>
+        <v>437</v>
       </c>
       <c r="B78" t="s">
-        <v>437</v>
+        <v>432</v>
       </c>
       <c r="E78">
         <v>12</v>
@@ -4441,24 +4445,24 @@
         <v>42</v>
       </c>
       <c r="G78" t="s">
-        <v>443</v>
+        <v>438</v>
       </c>
       <c r="H78" t="s">
-        <v>445</v>
+        <v>440</v>
       </c>
       <c r="I78" t="s">
-        <v>444</v>
+        <v>439</v>
       </c>
       <c r="J78" t="s">
-        <v>445</v>
+        <v>440</v>
       </c>
       <c r="K78" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.25">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="79" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B79" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="E79">
         <v>14</v>
@@ -4467,24 +4471,24 @@
         <v>54</v>
       </c>
       <c r="G79" t="s">
-        <v>447</v>
+        <v>442</v>
       </c>
       <c r="H79" t="s">
-        <v>483</v>
+        <v>478</v>
       </c>
       <c r="I79" t="s">
-        <v>486</v>
+        <v>481</v>
       </c>
       <c r="J79" t="s">
-        <v>483</v>
+        <v>478</v>
       </c>
       <c r="K79" t="s">
-        <v>448</v>
-      </c>
-    </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.25">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="80" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B80" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="E80">
         <v>14</v>
@@ -4493,21 +4497,21 @@
         <v>54</v>
       </c>
       <c r="G80" t="s">
-        <v>449</v>
+        <v>444</v>
       </c>
       <c r="H80" t="s">
-        <v>498</v>
+        <v>492</v>
       </c>
       <c r="I80" t="s">
-        <v>488</v>
+        <v>483</v>
       </c>
       <c r="K80" t="s">
-        <v>450</v>
-      </c>
-    </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.25">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="81" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B81" t="s">
-        <v>442</v>
+        <v>437</v>
       </c>
       <c r="E81">
         <v>14</v>
@@ -4516,21 +4520,21 @@
         <v>54</v>
       </c>
       <c r="G81" t="s">
-        <v>495</v>
+        <v>489</v>
       </c>
       <c r="H81" t="s">
-        <v>497</v>
+        <v>491</v>
       </c>
       <c r="I81" t="s">
-        <v>489</v>
+        <v>484</v>
       </c>
       <c r="K81" t="s">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="82" spans="1:11" x14ac:dyDescent="0.3">
       <c r="D82" t="s">
-        <v>452</v>
+        <v>447</v>
       </c>
       <c r="E82">
         <v>4</v>
@@ -4539,24 +4543,24 @@
         <v>6</v>
       </c>
       <c r="G82" t="s">
-        <v>473</v>
+        <v>468</v>
       </c>
       <c r="H82" t="s">
-        <v>453</v>
+        <v>448</v>
       </c>
       <c r="I82" t="s">
-        <v>479</v>
+        <v>474</v>
       </c>
       <c r="J82" t="s">
-        <v>453</v>
+        <v>448</v>
       </c>
       <c r="K82" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="83" spans="1:11" x14ac:dyDescent="0.3">
       <c r="D83" t="s">
-        <v>454</v>
+        <v>449</v>
       </c>
       <c r="E83">
         <v>7</v>
@@ -4565,21 +4569,21 @@
         <v>15</v>
       </c>
       <c r="G83" t="s">
-        <v>474</v>
+        <v>469</v>
       </c>
       <c r="H83" t="s">
-        <v>455</v>
+        <v>450</v>
       </c>
       <c r="J83" t="s">
-        <v>455</v>
+        <v>450</v>
       </c>
       <c r="K83" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="84" spans="1:11" x14ac:dyDescent="0.3">
       <c r="D84" t="s">
-        <v>456</v>
+        <v>451</v>
       </c>
       <c r="E84">
         <v>8</v>
@@ -4588,24 +4592,24 @@
         <v>18</v>
       </c>
       <c r="G84" t="s">
-        <v>475</v>
+        <v>470</v>
       </c>
       <c r="H84" t="s">
-        <v>457</v>
+        <v>452</v>
       </c>
       <c r="I84" t="s">
-        <v>485</v>
+        <v>480</v>
       </c>
       <c r="J84" t="s">
-        <v>457</v>
+        <v>452</v>
       </c>
       <c r="K84" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.25">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="85" spans="1:11" x14ac:dyDescent="0.3">
       <c r="D85" t="s">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="E85">
         <v>9</v>
@@ -4614,24 +4618,24 @@
         <v>24</v>
       </c>
       <c r="G85" t="s">
-        <v>476</v>
+        <v>471</v>
       </c>
       <c r="H85" t="s">
-        <v>459</v>
+        <v>454</v>
       </c>
       <c r="I85" t="s">
-        <v>480</v>
+        <v>475</v>
       </c>
       <c r="J85" t="s">
-        <v>459</v>
+        <v>454</v>
       </c>
       <c r="K85" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.25">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="86" spans="1:11" x14ac:dyDescent="0.3">
       <c r="D86" t="s">
-        <v>460</v>
+        <v>455</v>
       </c>
       <c r="E86">
         <v>9</v>
@@ -4640,21 +4644,21 @@
         <v>24</v>
       </c>
       <c r="G86" t="s">
-        <v>477</v>
+        <v>472</v>
       </c>
       <c r="H86" t="s">
-        <v>461</v>
+        <v>456</v>
       </c>
       <c r="J86" t="s">
-        <v>461</v>
+        <v>456</v>
       </c>
       <c r="K86" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.25">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="87" spans="1:11" x14ac:dyDescent="0.3">
       <c r="D87" t="s">
-        <v>462</v>
+        <v>457</v>
       </c>
       <c r="E87">
         <v>10</v>
@@ -4663,33 +4667,33 @@
         <v>30</v>
       </c>
       <c r="G87" t="s">
-        <v>478</v>
+        <v>473</v>
       </c>
       <c r="H87" t="s">
-        <v>463</v>
+        <v>458</v>
       </c>
       <c r="I87" t="s">
-        <v>481</v>
+        <v>476</v>
       </c>
       <c r="J87" t="s">
-        <v>463</v>
+        <v>458</v>
       </c>
       <c r="K87" t="s">
-        <v>464</v>
-      </c>
-    </row>
-    <row r="88" spans="1:11" x14ac:dyDescent="0.25">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="88" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="B88" t="s">
-        <v>465</v>
+        <v>460</v>
       </c>
       <c r="C88" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D88" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="E88">
         <v>1</v>
@@ -4698,33 +4702,33 @@
         <v>1</v>
       </c>
       <c r="G88" t="s">
-        <v>471</v>
+        <v>466</v>
       </c>
       <c r="H88" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="I88" t="s">
-        <v>468</v>
+        <v>463</v>
       </c>
       <c r="J88" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="K88" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="89" spans="1:11" x14ac:dyDescent="0.25">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="89" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="B89" t="s">
-        <v>466</v>
+        <v>461</v>
       </c>
       <c r="C89" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D89" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="E89">
         <v>2</v>
@@ -4733,33 +4737,33 @@
         <v>2</v>
       </c>
       <c r="G89" t="s">
-        <v>471</v>
+        <v>466</v>
       </c>
       <c r="H89" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="I89" t="s">
-        <v>469</v>
+        <v>464</v>
       </c>
       <c r="J89" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="K89" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.25">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="90" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="B90" t="s">
-        <v>467</v>
+        <v>462</v>
       </c>
       <c r="C90" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D90" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="E90">
         <v>3</v>
@@ -4768,19 +4772,19 @@
         <v>3</v>
       </c>
       <c r="G90" t="s">
-        <v>471</v>
+        <v>466</v>
       </c>
       <c r="H90" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="I90" t="s">
-        <v>470</v>
+        <v>465</v>
       </c>
       <c r="J90" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="K90" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
     </row>
   </sheetData>

</xml_diff>